<commit_message>
Correct IE tax residence wording
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Savings comparison" sheetId="1" r:id="Re748c0c5ba764d4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rab1a3d405e874236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L - add-on" sheetId="3" r:id="R8c1854d81e4f4553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Savings comparison" sheetId="1" r:id="R77d2b785ccfc4574"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R8e4089c7782843b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P&amp;L - add-on" sheetId="3" r:id="Rebe857aae8844b16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,7 +704,7 @@
         <x:v>Option 3 - Pension reserve</x:v>
       </x:c>
       <x:c r="F4" s="37" t="str">
-        <x:v>Option 4 - IE resident</x:v>
+        <x:v>Option 4 - IE tax residence</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="37.5" customHeight="1">
@@ -724,7 +724,7 @@
         <x:v>Full opt. incl. pension reserve</x:v>
       </x:c>
       <x:c r="F5" s="39" t="str">
-        <x:v>IE resident + director fee</x:v>
+        <x:v>IE tax residence + director fee</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="16.5" customHeight="1">
@@ -2095,7 +2095,7 @@
     </x:row>
     <x:row r="46" ht="30" customHeight="1">
       <x:c r="A46" s="38" t="str">
-        <x:v>Director fee required for IE tax resident company</x:v>
+        <x:v>Director fee required for IE tax residence option</x:v>
       </x:c>
       <x:c r="B46" s="98" t="n">
         <x:v>0</x:v>
@@ -2208,7 +2208,7 @@
     </x:row>
     <x:row r="55" ht="16.5" customHeight="1">
       <x:c r="A55" s="93" t="str">
-        <x:v>Option 4 IE resident / director fee</x:v>
+        <x:v>Option 4 IE tax residence / director fee</x:v>
       </x:c>
       <x:c r="B55" s="100" t="n">
         <x:v>1500</x:v>
@@ -2298,13 +2298,13 @@
     </x:row>
     <x:row r="63" ht="43.5" customHeight="1">
       <x:c r="A63" s="38" t="str">
-        <x:v>Option 4 - IE resident</x:v>
+        <x:v>Option 4 - IE tax residence</x:v>
       </x:c>
       <x:c r="B63" s="86" t="str">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="C63" s="39" t="str">
-        <x:v>Option 2 scope for IE tax resident company plus director fee</x:v>
+        <x:v>Option 2 scope for IE tax residence plus director fee</x:v>
       </x:c>
       <x:c r="D63" s="39" t="str">
         <x:v>Confirm director fee and IE company tax rate</x:v>
@@ -2409,7 +2409,7 @@
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B8">
-      <x:formula1>"Client choice pending,Option 1 - Basic analysis,Option 2 - Full optimisation,Option 3 - Pension reserve,Option 4 - IE resident"</x:formula1>
+      <x:formula1>"Client choice pending,Option 1 - Basic analysis,Option 2 - Full optimisation,Option 3 - Pension reserve,Option 4 - IE tax residence"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B10">
       <x:formula1>"Yes,No"</x:formula1>

</xml_diff>

<commit_message>
Refine savings template assumptions
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="286">
   <si>
     <t>Savings Calculation Template</t>
   </si>
@@ -118,7 +118,7 @@
     <t>Company model</t>
   </si>
   <si>
-    <t>Taxable profit before optimisation</t>
+    <t>Estimated status quo profit</t>
   </si>
   <si>
     <t>Office rent deductible</t>
@@ -145,7 +145,7 @@
     <t>Total additional deductions</t>
   </si>
   <si>
-    <t>Taxable profit after scenario</t>
+    <t>Estimated taxable profit after scenario</t>
   </si>
   <si>
     <t>Corporation tax rate</t>
@@ -160,7 +160,7 @@
     <t>Personal / owner value</t>
   </si>
   <si>
-    <t>Office rent after personal tax</t>
+    <t>Office rent net owner benefit</t>
   </si>
   <si>
     <t>Travel / other costs shifted from personal</t>
@@ -172,7 +172,7 @@
     <t>Pension reserve value</t>
   </si>
   <si>
-    <t>Director fee after personal tax</t>
+    <t>Director fee net owner benefit</t>
   </si>
   <si>
     <t>Outcome</t>
@@ -334,7 +334,7 @@
     <t>Owner marginal personal tax rate</t>
   </si>
   <si>
-    <t>Used for owner-level after-tax value estimates</t>
+    <t>Review-only rate used for net owner benefit estimates; not a client data input</t>
   </si>
   <si>
     <t>Operating model</t>
@@ -343,10 +343,10 @@
     <t>Operating model note</t>
   </si>
   <si>
-    <t>Inputs below feed the comparison tab</t>
-  </si>
-  <si>
-    <t>Use annual amounts</t>
+    <t>Status quo estimated from earnings and spend</t>
+  </si>
+  <si>
+    <t>Future gross-net calculator workflow can use https://www.brutto-netto-rechner.info/gehalt/gehaltsrechner-arbeitgeber.php</t>
   </si>
   <si>
     <t>Annual revenue</t>
@@ -370,7 +370,10 @@
     <t>Set previous accounting fee below to 0 if already embedded and not replaced</t>
   </si>
   <si>
-    <t>Before RB changes</t>
+    <t>Estimated status quo profit (calculated)</t>
+  </si>
+  <si>
+    <t>Calculated from annual revenue minus current operating costs; not a client input</t>
   </si>
   <si>
     <t>Office rent and expense optimisation</t>
@@ -394,10 +397,10 @@
     <t>Used in comparison tab</t>
   </si>
   <si>
-    <t>Personal taxable share of office rent</t>
-  </si>
-  <si>
-    <t>Share assumed taxable to owner</t>
+    <t>Taxable share of company-paid office rent</t>
+  </si>
+  <si>
+    <t>Use 0 if tax-free and 1 if fully taxable to the owner; review case by case</t>
   </si>
   <si>
     <t>Business travel deductible</t>
@@ -463,10 +466,10 @@
     <t>Only included in Option 4</t>
   </si>
   <si>
-    <t>Director personal tax / leakage rate</t>
-  </si>
-  <si>
-    <t>After-tax owner value assumption</t>
+    <t>Estimated tax on director fee</t>
+  </si>
+  <si>
+    <t>Applied to director fee only to estimate after-tax owner benefit; review case by case</t>
   </si>
   <si>
     <t>Current annual accounting, legal, or advisory fee that RB replaces</t>
@@ -953,15 +956,15 @@
     </font>
     <font>
       <sz val="11.0"/>
-      <color rgb="FF0000FF"/>
-      <name val="Roboto"/>
+      <color rgb="FF000000"/>
+      <name val="Carlito"/>
     </font>
     <font>
       <u/>
       <color rgb="FF0000FF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1002,6 +1005,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFB6D7A8"/>
         <bgColor rgb="FFB6D7A8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1202,7 +1211,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="113">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1329,104 +1338,112 @@
     <xf borderId="4" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="8" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="8" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="2" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="3" fillId="9" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="12" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="9" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="12" numFmtId="168" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="8" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="12" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="8" fontId="9" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="6" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="3" fillId="8" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="12" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="1" fillId="8" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="3" fillId="8" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="6" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="9" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="8" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="9" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="9" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="8" fontId="12" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="10" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="6" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="8" fontId="9" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="8" fontId="6" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="14" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="8" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="15" fillId="8" fontId="12" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="15" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="15" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="16" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1459,6 +1476,7 @@
     <xf borderId="1" fillId="0" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -3761,94 +3779,94 @@
       </c>
     </row>
     <row r="5" ht="16.5" customHeight="1">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="52" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="11" t="s">
+      <c r="B5" s="53"/>
+      <c r="C5" s="54" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="54" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="52" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="11" t="s">
+      <c r="B6" s="53"/>
+      <c r="C6" s="54" t="s">
         <v>79</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="54" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="53"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
+      <c r="A7" s="52"/>
+      <c r="B7" s="55"/>
+      <c r="C7" s="54"/>
+      <c r="D7" s="54"/>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="54" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="52" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="53">
+      <c r="B9" s="56">
         <v>1.0</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="54" t="s">
         <v>88</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="54" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="52" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="11" t="s">
+      <c r="B10" s="56"/>
+      <c r="C10" s="54" t="s">
         <v>79</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="54" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="52" t="s">
         <v>92</v>
       </c>
-      <c r="B11" s="53" t="s">
+      <c r="B11" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="54" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="4"/>
-      <c r="B12" s="52"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
+      <c r="A12" s="52"/>
+      <c r="B12" s="57"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="58"/>
     </row>
     <row r="13" ht="16.5" customHeight="1">
       <c r="A13" s="18" t="s">
@@ -3859,66 +3877,66 @@
       <c r="D13" s="20"/>
     </row>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="55" t="s">
+      <c r="A14" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="56" t="s">
+      <c r="B14" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="C14" s="57" t="s">
+      <c r="C14" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="58" t="s">
+      <c r="D14" s="61" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="B15" s="59">
+      <c r="B15" s="62">
         <v>0.3</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="54" t="s">
         <v>99</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="54" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="52" t="s">
         <v>101</v>
       </c>
-      <c r="B16" s="59">
+      <c r="B16" s="62">
         <v>0.125</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="54" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="B17" s="59">
+      <c r="B17" s="62">
         <v>0.42</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="54" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="4"/>
-      <c r="B18" s="60"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
+      <c r="A18" s="52"/>
+      <c r="B18" s="63"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
     </row>
     <row r="19" ht="16.5" customHeight="1">
       <c r="A19" s="18" t="s">
@@ -3929,588 +3947,588 @@
       <c r="D19" s="20"/>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="61" t="s">
+      <c r="A20" s="64" t="s">
         <v>107</v>
       </c>
-      <c r="B20" s="62" t="s">
+      <c r="B20" s="65" t="s">
         <v>108</v>
       </c>
-      <c r="C20" s="63" t="s">
+      <c r="C20" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="64" t="s">
+      <c r="D20" s="66" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="52" t="s">
         <v>110</v>
       </c>
-      <c r="B21" s="65">
+      <c r="B21" s="67">
         <v>180000.0</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="54" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="55" t="s">
+      <c r="A22" s="59" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="66">
+      <c r="B22" s="68">
         <v>60000.0</v>
       </c>
-      <c r="C22" s="57" t="s">
+      <c r="C22" s="60" t="s">
         <v>111</v>
       </c>
-      <c r="D22" s="58" t="s">
+      <c r="D22" s="61" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="52" t="s">
         <v>115</v>
       </c>
-      <c r="B23" s="65" t="s">
+      <c r="B23" s="69" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="C23" s="54" t="s">
         <v>79</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="54" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1">
-      <c r="A24" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="65">
+      <c r="A24" s="52" t="s">
+        <v>117</v>
+      </c>
+      <c r="B24" s="70">
         <f>B21-B22</f>
         <v>120000</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="11" t="s">
-        <v>117</v>
+      <c r="D24" s="54" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="4"/>
-      <c r="B25" s="67"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
+      <c r="A25" s="52"/>
+      <c r="B25" s="71"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
     </row>
     <row r="26" ht="16.5" customHeight="1">
       <c r="A26" s="18" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B26" s="19"/>
       <c r="C26" s="19"/>
       <c r="D26" s="20"/>
     </row>
     <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="61" t="s">
-        <v>119</v>
-      </c>
-      <c r="B27" s="68" t="s">
+      <c r="A27" s="64" t="s">
         <v>120</v>
       </c>
-      <c r="C27" s="63" t="s">
+      <c r="B27" s="72" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="D27" s="64" t="s">
-        <v>121</v>
+      <c r="D27" s="66" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="28" ht="16.5" customHeight="1">
-      <c r="A28" s="55" t="s">
+      <c r="A28" s="59" t="s">
+        <v>123</v>
+      </c>
+      <c r="B28" s="68">
+        <v>0.0</v>
+      </c>
+      <c r="C28" s="60" t="s">
+        <v>111</v>
+      </c>
+      <c r="D28" s="61" t="s">
         <v>122</v>
       </c>
-      <c r="B28" s="66">
-        <v>0.0</v>
-      </c>
-      <c r="C28" s="57" t="s">
-        <v>111</v>
-      </c>
-      <c r="D28" s="58" t="s">
-        <v>121</v>
-      </c>
     </row>
     <row r="29" ht="30.0" customHeight="1">
-      <c r="A29" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="B29" s="69">
+      <c r="A29" s="52" t="s">
+        <v>124</v>
+      </c>
+      <c r="B29" s="71">
         <f>B28</f>
         <v>0</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D29" s="11" t="s">
-        <v>124</v>
+      <c r="D29" s="54" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="30" ht="16.5" customHeight="1">
-      <c r="A30" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B30" s="59">
+      <c r="A30" s="52" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" s="62">
         <v>0.5</v>
       </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="D30" s="11" t="s">
-        <v>126</v>
+      <c r="D30" s="54" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="31" ht="16.5" customHeight="1">
-      <c r="A31" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B31" s="65">
+      <c r="A31" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="B31" s="67">
         <v>0.0</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D31" s="11" t="s">
-        <v>128</v>
+      <c r="D31" s="54" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="32" ht="16.5" customHeight="1">
-      <c r="A32" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="B32" s="65">
+      <c r="A32" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" s="67">
         <v>0.0</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D32" s="11" t="s">
-        <v>130</v>
+      <c r="D32" s="54" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="33" ht="16.5" customHeight="1">
-      <c r="A33" s="4"/>
-      <c r="B33" s="65"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
+      <c r="A33" s="52"/>
+      <c r="B33" s="70"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="54"/>
     </row>
     <row r="34" ht="16.5" customHeight="1">
       <c r="A34" s="18" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B34" s="19"/>
       <c r="C34" s="19"/>
       <c r="D34" s="20"/>
     </row>
     <row r="35" ht="16.5" customHeight="1">
-      <c r="A35" s="55" t="s">
-        <v>132</v>
-      </c>
-      <c r="B35" s="66">
+      <c r="A35" s="59" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" s="68">
         <v>0.0</v>
       </c>
-      <c r="C35" s="57" t="s">
+      <c r="C35" s="60" t="s">
         <v>111</v>
       </c>
-      <c r="D35" s="58" t="s">
-        <v>133</v>
+      <c r="D35" s="61" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="36" ht="16.5" customHeight="1">
-      <c r="A36" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="B36" s="65">
+      <c r="A36" s="52" t="s">
+        <v>135</v>
+      </c>
+      <c r="B36" s="73">
         <v>5.0</v>
       </c>
-      <c r="C36" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="D36" s="11" t="s">
+      <c r="C36" s="54" t="s">
         <v>136</v>
       </c>
+      <c r="D36" s="54" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="37" ht="16.5" customHeight="1">
-      <c r="A37" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B37" s="59">
+      <c r="A37" s="52" t="s">
+        <v>138</v>
+      </c>
+      <c r="B37" s="74">
         <v>0.8</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="D37" s="11" t="s">
-        <v>138</v>
+      <c r="D37" s="54" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1">
-      <c r="A38" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="B38" s="65">
+      <c r="A38" s="52" t="s">
+        <v>140</v>
+      </c>
+      <c r="B38" s="70">
         <f>IF(B36&gt;0,B35/B36,0)</f>
         <v>0</v>
       </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D38" s="11" t="s">
-        <v>140</v>
+      <c r="D38" s="54" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="39" ht="16.5" customHeight="1">
-      <c r="A39" s="4" t="s">
-        <v>141</v>
+      <c r="A39" s="52" t="s">
+        <v>142</v>
       </c>
       <c r="B39" s="70">
         <f>B38*B37</f>
         <v>0</v>
       </c>
-      <c r="C39" s="11" t="s">
+      <c r="C39" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D39" s="11" t="s">
-        <v>124</v>
+      <c r="D39" s="54" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="40" ht="16.5" customHeight="1">
-      <c r="A40" s="71"/>
-      <c r="B40" s="69"/>
-      <c r="C40" s="54"/>
-      <c r="D40" s="54"/>
+      <c r="A40" s="75"/>
+      <c r="B40" s="71"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
     </row>
     <row r="41" ht="16.5" customHeight="1">
       <c r="A41" s="49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B41" s="19"/>
       <c r="C41" s="19"/>
       <c r="D41" s="20"/>
     </row>
     <row r="42" ht="16.5" customHeight="1">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="B42" s="65">
+      <c r="B42" s="67">
         <v>0.0</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D42" s="11" t="s">
-        <v>143</v>
+      <c r="D42" s="54" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="B43" s="65">
+      <c r="B43" s="67">
         <v>0.0</v>
       </c>
-      <c r="C43" s="11" t="s">
+      <c r="C43" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D43" s="11" t="s">
-        <v>144</v>
+      <c r="D43" s="54" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1">
-      <c r="A44" s="71"/>
-      <c r="B44" s="69"/>
-      <c r="C44" s="54"/>
-      <c r="D44" s="54"/>
+      <c r="A44" s="75"/>
+      <c r="B44" s="71"/>
+      <c r="C44" s="58"/>
+      <c r="D44" s="58"/>
     </row>
     <row r="45" ht="16.5" customHeight="1">
       <c r="A45" s="49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B45" s="19"/>
       <c r="C45" s="19"/>
       <c r="D45" s="20"/>
     </row>
     <row r="46" ht="30.0" customHeight="1">
-      <c r="A46" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B46" s="65">
+      <c r="A46" s="52" t="s">
+        <v>147</v>
+      </c>
+      <c r="B46" s="67">
         <v>0.0</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D46" s="11" t="s">
-        <v>147</v>
+      <c r="D46" s="54" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="47" ht="16.5" customHeight="1">
-      <c r="A47" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="B47" s="72">
+      <c r="A47" s="52" t="s">
+        <v>149</v>
+      </c>
+      <c r="B47" s="62">
         <v>0.2</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C47" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="D47" s="11" t="s">
-        <v>149</v>
+      <c r="D47" s="54" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="48" ht="16.5" customHeight="1">
-      <c r="A48" s="73"/>
-      <c r="B48" s="74"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="25"/>
+      <c r="A48" s="76"/>
+      <c r="B48" s="77"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="78"/>
     </row>
     <row r="49" ht="16.5" customHeight="1">
-      <c r="A49" s="75" t="s">
+      <c r="A49" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="B49" s="76">
+      <c r="B49" s="80">
         <v>0.0</v>
       </c>
-      <c r="C49" s="77" t="s">
+      <c r="C49" s="81" t="s">
         <v>111</v>
       </c>
-      <c r="D49" s="78" t="s">
-        <v>150</v>
+      <c r="D49" s="82" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="50" ht="16.5" customHeight="1">
-      <c r="A50" s="79" t="s">
-        <v>151</v>
-      </c>
-      <c r="B50" s="65">
+      <c r="A50" s="83" t="s">
+        <v>152</v>
+      </c>
+      <c r="B50" s="70">
         <v>500.0</v>
       </c>
-      <c r="C50" s="11" t="s">
+      <c r="C50" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D50" s="80" t="s">
-        <v>152</v>
+      <c r="D50" s="84" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="51" ht="16.5" customHeight="1">
-      <c r="A51" s="79" t="s">
-        <v>153</v>
-      </c>
-      <c r="B51" s="65">
+      <c r="A51" s="83" t="s">
+        <v>154</v>
+      </c>
+      <c r="B51" s="70">
         <v>1000.0</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C51" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D51" s="80" t="s">
-        <v>154</v>
+      <c r="D51" s="84" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="52" ht="16.5" customHeight="1">
-      <c r="A52" s="79" t="s">
-        <v>155</v>
-      </c>
-      <c r="B52" s="65">
+      <c r="A52" s="83" t="s">
+        <v>156</v>
+      </c>
+      <c r="B52" s="85">
         <v>3.0</v>
       </c>
-      <c r="C52" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="D52" s="80" t="s">
+      <c r="C52" s="54" t="s">
         <v>157</v>
       </c>
+      <c r="D52" s="84" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="53" ht="16.5" customHeight="1">
-      <c r="A53" s="79" t="s">
-        <v>158</v>
-      </c>
-      <c r="B53" s="65">
+      <c r="A53" s="83" t="s">
+        <v>159</v>
+      </c>
+      <c r="B53" s="70">
         <v>200.0</v>
       </c>
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D53" s="80" t="s">
-        <v>159</v>
+      <c r="D53" s="84" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="54" ht="16.5" customHeight="1">
-      <c r="A54" s="79" t="s">
+      <c r="A54" s="83" t="s">
         <v>28</v>
       </c>
-      <c r="B54" s="65">
+      <c r="B54" s="70">
         <v>200.0</v>
       </c>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D54" s="80" t="s">
-        <v>160</v>
+      <c r="D54" s="84" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="55" ht="16.5" customHeight="1">
-      <c r="A55" s="81" t="s">
+      <c r="A55" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="B55" s="82">
+      <c r="B55" s="87">
         <v>200.0</v>
       </c>
-      <c r="C55" s="83" t="s">
+      <c r="C55" s="88" t="s">
         <v>111</v>
       </c>
-      <c r="D55" s="84" t="s">
-        <v>161</v>
+      <c r="D55" s="89" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="56" ht="16.5" customHeight="1">
-      <c r="A56" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="B56" s="65">
+      <c r="A56" s="52" t="s">
+        <v>163</v>
+      </c>
+      <c r="B56" s="70">
         <v>400.0</v>
       </c>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D56" s="11" t="s">
-        <v>163</v>
+      <c r="D56" s="54" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="57" ht="16.5" customHeight="1">
-      <c r="A57" s="4"/>
-      <c r="B57" s="65"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
+      <c r="A57" s="52"/>
+      <c r="B57" s="70"/>
+      <c r="C57" s="54"/>
+      <c r="D57" s="54"/>
     </row>
     <row r="58" ht="16.5" customHeight="1">
-      <c r="A58" s="55"/>
-      <c r="B58" s="57"/>
-      <c r="C58" s="57"/>
-      <c r="D58" s="58"/>
+      <c r="A58" s="59"/>
+      <c r="B58" s="60"/>
+      <c r="C58" s="60"/>
+      <c r="D58" s="61"/>
     </row>
     <row r="59" ht="43.5" customHeight="1">
       <c r="A59" s="18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B59" s="19"/>
       <c r="C59" s="19"/>
       <c r="D59" s="20"/>
     </row>
     <row r="60" ht="43.5" customHeight="1">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="B60" s="85">
+      <c r="B60" s="52">
         <v>0.0</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="D60" s="5" t="s">
-        <v>165</v>
+      <c r="D60" s="52" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="61" ht="43.5" customHeight="1">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="B61" s="85">
+      <c r="B61" s="52">
         <v>500.0</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C61" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="D61" s="5" t="s">
-        <v>166</v>
+      <c r="D61" s="52" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="62" ht="43.5" customHeight="1">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="B62" s="85" t="s">
-        <v>167</v>
-      </c>
-      <c r="C62" s="5" t="s">
+      <c r="B62" s="52" t="s">
+        <v>168</v>
+      </c>
+      <c r="C62" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="D62" s="5" t="s">
-        <v>168</v>
+      <c r="D62" s="52" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="63" ht="43.5" customHeight="1">
-      <c r="A63" s="4" t="s">
+      <c r="A63" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="B63" s="85" t="s">
-        <v>169</v>
-      </c>
-      <c r="C63" s="5" t="s">
+      <c r="B63" s="52" t="s">
+        <v>170</v>
+      </c>
+      <c r="C63" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="D63" s="5" t="s">
-        <v>170</v>
+      <c r="D63" s="52" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="64" ht="16.5" customHeight="1">
-      <c r="A64" s="4" t="s">
+      <c r="A64" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="B64" s="86" t="s">
-        <v>171</v>
-      </c>
-      <c r="C64" s="11" t="s">
+      <c r="B64" s="55" t="s">
+        <v>172</v>
+      </c>
+      <c r="C64" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="D64" s="11" t="s">
-        <v>172</v>
+      <c r="D64" s="54" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="65" ht="16.5" customHeight="1">
-      <c r="A65" s="71"/>
-      <c r="B65" s="87"/>
-      <c r="C65" s="54"/>
-      <c r="D65" s="54"/>
+      <c r="A65" s="75"/>
+      <c r="B65" s="57"/>
+      <c r="C65" s="58"/>
+      <c r="D65" s="58"/>
     </row>
     <row r="66" ht="16.5" customHeight="1">
-      <c r="A66" s="88"/>
-      <c r="B66" s="89"/>
-      <c r="C66" s="89"/>
-      <c r="D66" s="90"/>
+      <c r="A66" s="90"/>
+      <c r="B66" s="91"/>
+      <c r="C66" s="91"/>
+      <c r="D66" s="92"/>
     </row>
     <row r="67" ht="51.0" customHeight="1">
-      <c r="A67" s="91"/>
-      <c r="B67" s="92"/>
-      <c r="C67" s="93"/>
-      <c r="D67" s="93"/>
+      <c r="A67" s="93"/>
+      <c r="B67" s="94"/>
+      <c r="C67" s="95"/>
+      <c r="D67" s="95"/>
     </row>
     <row r="68" ht="51.0" customHeight="1">
-      <c r="A68" s="91"/>
-      <c r="B68" s="92"/>
-      <c r="C68" s="93"/>
-      <c r="D68" s="93"/>
+      <c r="A68" s="93"/>
+      <c r="B68" s="94"/>
+      <c r="C68" s="95"/>
+      <c r="D68" s="95"/>
     </row>
     <row r="69" ht="51.0" customHeight="1">
-      <c r="A69" s="91"/>
-      <c r="B69" s="92"/>
-      <c r="C69" s="93"/>
-      <c r="D69" s="93"/>
+      <c r="A69" s="93"/>
+      <c r="B69" s="94"/>
+      <c r="C69" s="95"/>
+      <c r="D69" s="95"/>
     </row>
     <row r="70" ht="51.0" customHeight="1">
-      <c r="A70" s="91"/>
-      <c r="B70" s="92"/>
-      <c r="C70" s="93"/>
-      <c r="D70" s="93"/>
+      <c r="A70" s="93"/>
+      <c r="B70" s="94"/>
+      <c r="C70" s="95"/>
+      <c r="D70" s="95"/>
     </row>
     <row r="71" ht="16.5" customHeight="1"/>
     <row r="72" ht="16.5" customHeight="1"/>
@@ -5461,6 +5479,9 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B8">
       <formula1>"Client choice pending,Option 1 - Basic operating entity,Option 2 - Full optimisation,Option 3 - Pension reserve,Option 4 - IE tax residence"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B23">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
   </dataValidations>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -5484,26 +5505,26 @@
   <sheetData>
     <row r="1" ht="16.5" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" ht="31.5" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
-      <c r="A3" s="94" t="s">
-        <v>175</v>
-      </c>
-      <c r="B3" s="95" t="str">
+      <c r="A3" s="96" t="s">
+        <v>176</v>
+      </c>
+      <c r="B3" s="97" t="str">
         <f>Assumptions!$B$8</f>
         <v>Client choice pending</v>
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1">
-      <c r="A4" s="94" t="s">
-        <v>176</v>
+      <c r="A4" s="96" t="s">
+        <v>177</v>
       </c>
       <c r="B4" s="22" t="str">
         <f t="array" ref="B4">IFERROR(INDEX('Savings comparison'!$C$46:$F$46,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0)),"")</f>
@@ -5513,54 +5534,54 @@
     <row r="5" ht="16.5" customHeight="1"/>
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C7" s="13">
         <f t="array" ref="C7:N7">Assumptions!$B$21/12+COLUMN(C6:N6)*0</f>
@@ -5601,56 +5622,56 @@
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="96" t="s">
-        <v>193</v>
-      </c>
-      <c r="B8" s="97" t="s">
+      <c r="A8" s="98" t="s">
         <v>194</v>
       </c>
-      <c r="C8" s="98">
+      <c r="B8" s="99" t="s">
+        <v>195</v>
+      </c>
+      <c r="C8" s="100">
         <f t="array" ref="C8:N8">Assumptions!$B$22/12+COLUMN(C6:N6)*0</f>
         <v>5000</v>
       </c>
-      <c r="D8" s="98">
+      <c r="D8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="E8" s="98">
+      <c r="E8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="F8" s="98">
+      <c r="F8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="G8" s="98">
+      <c r="G8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="H8" s="98">
+      <c r="H8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="I8" s="98">
+      <c r="I8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="J8" s="98">
+      <c r="J8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="K8" s="98">
+      <c r="K8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="L8" s="98">
+      <c r="L8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="M8" s="98">
+      <c r="M8" s="100">
         <v>5000.0</v>
       </c>
-      <c r="N8" s="98">
+      <c r="N8" s="100">
         <v>5000.0</v>
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="B9" s="99" t="s">
         <v>196</v>
+      </c>
+      <c r="B9" s="101" t="s">
+        <v>197</v>
       </c>
       <c r="C9" s="13">
         <f t="array" ref="C9:N9">Assumptions!$B$49/12+COLUMN(C6:N6)*0</f>
@@ -5691,34 +5712,34 @@
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="96" t="s">
-        <v>197</v>
-      </c>
-      <c r="B10" s="97" t="s">
-        <v>175</v>
-      </c>
-      <c r="C10" s="98" t="str">
+      <c r="A10" s="98" t="s">
+        <v>198</v>
+      </c>
+      <c r="B10" s="99" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="100" t="str">
         <f t="array" ref="C10:N10">IFERROR(INDEX('Savings comparison'!$C$23:$F$23,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
         <v/>
       </c>
-      <c r="D10" s="98"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98"/>
-      <c r="G10" s="98"/>
-      <c r="H10" s="98"/>
-      <c r="I10" s="98"/>
-      <c r="J10" s="98"/>
-      <c r="K10" s="98"/>
-      <c r="L10" s="98"/>
-      <c r="M10" s="98"/>
-      <c r="N10" s="98"/>
+      <c r="D10" s="100"/>
+      <c r="E10" s="100"/>
+      <c r="F10" s="100"/>
+      <c r="G10" s="100"/>
+      <c r="H10" s="100"/>
+      <c r="I10" s="100"/>
+      <c r="J10" s="100"/>
+      <c r="K10" s="100"/>
+      <c r="L10" s="100"/>
+      <c r="M10" s="100"/>
+      <c r="N10" s="100"/>
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="B11" s="99" t="s">
-        <v>175</v>
+        <v>199</v>
+      </c>
+      <c r="B11" s="101" t="s">
+        <v>176</v>
       </c>
       <c r="C11" s="13" t="str">
         <f t="array" ref="C11:N11">IFERROR(INDEX('Savings comparison'!$C$24:$F$24,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -5738,10 +5759,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="B12" s="99" t="s">
-        <v>175</v>
+        <v>200</v>
+      </c>
+      <c r="B12" s="101" t="s">
+        <v>176</v>
       </c>
       <c r="C12" s="13" t="str">
         <f t="array" ref="C12:N12">IFERROR(INDEX('Savings comparison'!$C$26:$F$26,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -5763,8 +5784,8 @@
       <c r="A13" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="99" t="s">
-        <v>175</v>
+      <c r="B13" s="101" t="s">
+        <v>176</v>
       </c>
       <c r="C13" s="13" t="str">
         <f t="array" ref="C13:N13">IFERROR(INDEX('Savings comparison'!$C$27:$F$27,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -5784,10 +5805,10 @@
     </row>
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="B14" s="99" t="s">
-        <v>175</v>
+        <v>201</v>
+      </c>
+      <c r="B14" s="101" t="s">
+        <v>176</v>
       </c>
       <c r="C14" s="13" t="str">
         <f t="array" ref="C14:N14">IFERROR(INDEX('Savings comparison'!$C$28:$F$28,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -5807,10 +5828,10 @@
     </row>
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="B15" s="99" t="s">
-        <v>175</v>
+        <v>202</v>
+      </c>
+      <c r="B15" s="101" t="s">
+        <v>176</v>
       </c>
       <c r="C15" s="13" t="str">
         <f t="array" ref="C15:N15">IFERROR(INDEX('Savings comparison'!$C$19:$F$19,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -5829,7 +5850,7 @@
       <c r="N15" s="13"/>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="54"/>
+      <c r="A16" s="102"/>
       <c r="B16" s="17"/>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
@@ -5846,10 +5867,10 @@
     </row>
     <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>202</v>
-      </c>
-      <c r="B17" s="99" t="s">
         <v>203</v>
+      </c>
+      <c r="B17" s="101" t="s">
+        <v>204</v>
       </c>
       <c r="C17" s="13">
         <f t="array" ref="C17">IF(COUNTIF('Savings comparison'!$C$4:$F$4,$B$3)=0,0,C8:N8-C9:N9-C11:N11-C12:N12-C13:N13-C14:N14-C15:N15-C16:N16+C10:N10)</f>
@@ -5868,11 +5889,11 @@
       <c r="N17" s="13"/>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="94" t="s">
-        <v>204</v>
-      </c>
-      <c r="B18" s="100" t="s">
+      <c r="A18" s="96" t="s">
         <v>205</v>
+      </c>
+      <c r="B18" s="103" t="s">
+        <v>206</v>
       </c>
       <c r="C18" s="22">
         <f t="array" ref="C18">IF(COUNTIF('Savings comparison'!$C$4:$F$4,$B$3)=0,0,IF(C17:N17&gt;0,C17:N17*INDEX('Savings comparison'!$C$32:$F$32,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0)),0))</f>
@@ -5891,11 +5912,11 @@
       <c r="N18" s="22"/>
     </row>
     <row r="19" ht="16.5" customHeight="1">
-      <c r="A19" s="94" t="s">
-        <v>206</v>
-      </c>
-      <c r="B19" s="100" t="s">
-        <v>203</v>
+      <c r="A19" s="96" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" s="103" t="s">
+        <v>204</v>
       </c>
       <c r="C19" s="22">
         <f t="array" ref="C19">IF(COUNTIF('Savings comparison'!$C$4:$F$4,$B$3)=0,0,C17:N17-C18:N18)</f>
@@ -5914,8 +5935,8 @@
       <c r="N19" s="22"/>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="95"/>
-      <c r="B20" s="101"/>
+      <c r="A20" s="97"/>
+      <c r="B20" s="104"/>
       <c r="C20" s="22"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
@@ -5930,56 +5951,56 @@
       <c r="N20" s="22"/>
     </row>
     <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="94" t="s">
+      <c r="A21" s="96" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="100" t="s">
-        <v>207</v>
-      </c>
-      <c r="C21" s="101"/>
-      <c r="D21" s="101"/>
-      <c r="E21" s="101"/>
-      <c r="F21" s="101"/>
-      <c r="G21" s="101"/>
-      <c r="H21" s="101"/>
-      <c r="I21" s="101"/>
-      <c r="J21" s="101"/>
-      <c r="K21" s="101"/>
-      <c r="L21" s="101"/>
-      <c r="M21" s="101"/>
-      <c r="N21" s="101"/>
+      <c r="B21" s="103" t="s">
+        <v>208</v>
+      </c>
+      <c r="C21" s="104"/>
+      <c r="D21" s="104"/>
+      <c r="E21" s="104"/>
+      <c r="F21" s="104"/>
+      <c r="G21" s="104"/>
+      <c r="H21" s="104"/>
+      <c r="I21" s="104"/>
+      <c r="J21" s="104"/>
+      <c r="K21" s="104"/>
+      <c r="L21" s="104"/>
+      <c r="M21" s="104"/>
+      <c r="N21" s="104"/>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="95"/>
-      <c r="B22" s="101"/>
-      <c r="C22" s="101"/>
-      <c r="D22" s="101"/>
-      <c r="E22" s="101"/>
-      <c r="F22" s="101"/>
-      <c r="G22" s="101"/>
-      <c r="H22" s="101"/>
-      <c r="I22" s="101"/>
-      <c r="J22" s="101"/>
-      <c r="K22" s="101"/>
-      <c r="L22" s="101"/>
-      <c r="M22" s="101"/>
-      <c r="N22" s="101"/>
+      <c r="A22" s="97"/>
+      <c r="B22" s="104"/>
+      <c r="C22" s="104"/>
+      <c r="D22" s="104"/>
+      <c r="E22" s="104"/>
+      <c r="F22" s="104"/>
+      <c r="G22" s="104"/>
+      <c r="H22" s="104"/>
+      <c r="I22" s="104"/>
+      <c r="J22" s="104"/>
+      <c r="K22" s="104"/>
+      <c r="L22" s="104"/>
+      <c r="M22" s="104"/>
+      <c r="N22" s="104"/>
     </row>
     <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="95"/>
-      <c r="B23" s="101"/>
-      <c r="C23" s="101"/>
-      <c r="D23" s="101"/>
-      <c r="E23" s="101"/>
-      <c r="F23" s="101"/>
-      <c r="G23" s="101"/>
-      <c r="H23" s="101"/>
-      <c r="I23" s="101"/>
-      <c r="J23" s="101"/>
-      <c r="K23" s="101"/>
-      <c r="L23" s="101"/>
-      <c r="M23" s="101"/>
-      <c r="N23" s="101"/>
+      <c r="A23" s="97"/>
+      <c r="B23" s="104"/>
+      <c r="C23" s="104"/>
+      <c r="D23" s="104"/>
+      <c r="E23" s="104"/>
+      <c r="F23" s="104"/>
+      <c r="G23" s="104"/>
+      <c r="H23" s="104"/>
+      <c r="I23" s="104"/>
+      <c r="J23" s="104"/>
+      <c r="K23" s="104"/>
+      <c r="L23" s="104"/>
+      <c r="M23" s="104"/>
+      <c r="N23" s="104"/>
     </row>
     <row r="24" ht="16.5" customHeight="1"/>
     <row r="25" ht="16.5" customHeight="1"/>
@@ -6991,344 +7012,344 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="102" t="s">
-        <v>208</v>
+      <c r="A1" s="105" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="103" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2" s="104">
+      <c r="A2" s="106" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="107">
         <f>'Savings comparison'!C19</f>
         <v>500</v>
       </c>
-      <c r="C2" s="105" t="s">
-        <v>210</v>
-      </c>
-      <c r="D2" s="104">
+      <c r="C2" s="108" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="107">
         <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
         <v>824</v>
       </c>
-      <c r="E2" s="103" t="s">
-        <v>211</v>
-      </c>
-      <c r="F2" s="106">
+      <c r="E2" s="106" t="s">
+        <v>212</v>
+      </c>
+      <c r="F2" s="109">
         <v>46185.0</v>
       </c>
-      <c r="G2" s="107"/>
+      <c r="G2" s="110"/>
     </row>
     <row r="3">
-      <c r="A3" s="103" t="s">
-        <v>212</v>
+      <c r="A3" s="106" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="107"/>
-      <c r="B4" s="107"/>
-      <c r="C4" s="107"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
+      <c r="A4" s="110"/>
+      <c r="B4" s="110"/>
+      <c r="C4" s="110"/>
+      <c r="D4" s="110"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
     </row>
     <row r="5">
-      <c r="A5" s="108" t="s">
-        <v>213</v>
-      </c>
-      <c r="B5" s="108" t="s">
+      <c r="A5" s="111" t="s">
         <v>214</v>
       </c>
-      <c r="C5" s="108" t="s">
+      <c r="B5" s="111" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="108" t="s">
+      <c r="C5" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="E5" s="108" t="s">
+      <c r="D5" s="111" t="s">
         <v>217</v>
       </c>
-      <c r="F5" s="108" t="s">
+      <c r="E5" s="111" t="s">
         <v>218</v>
       </c>
-      <c r="G5" s="108" t="s">
+      <c r="F5" s="111" t="s">
         <v>219</v>
       </c>
+      <c r="G5" s="111" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="103" t="b">
+      <c r="A6" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B6" s="103" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="103" t="s">
+      <c r="B6" s="106" t="s">
         <v>221</v>
       </c>
-      <c r="D6" s="105">
+      <c r="C6" s="106" t="s">
+        <v>222</v>
+      </c>
+      <c r="D6" s="108">
         <v>824.0</v>
       </c>
-      <c r="E6" s="103" t="s">
-        <v>222</v>
-      </c>
-      <c r="F6" s="103" t="s">
+      <c r="E6" s="106" t="s">
         <v>223</v>
       </c>
-      <c r="G6" s="103" t="s">
+      <c r="F6" s="106" t="s">
         <v>224</v>
       </c>
+      <c r="G6" s="106" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="103" t="b">
+      <c r="A7" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B7" s="103" t="s">
-        <v>225</v>
-      </c>
-      <c r="C7" s="103" t="s">
+      <c r="B7" s="106" t="s">
         <v>226</v>
       </c>
-      <c r="D7" s="105">
+      <c r="C7" s="106" t="s">
+        <v>227</v>
+      </c>
+      <c r="D7" s="108">
         <v>2028.0</v>
       </c>
-      <c r="E7" s="103" t="s">
-        <v>227</v>
-      </c>
-      <c r="F7" s="109" t="s">
+      <c r="E7" s="106" t="s">
         <v>228</v>
       </c>
-      <c r="G7" s="103" t="s">
+      <c r="F7" s="112" t="s">
         <v>229</v>
       </c>
+      <c r="G7" s="106" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="103" t="b">
+      <c r="A8" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B8" s="103" t="s">
-        <v>230</v>
-      </c>
-      <c r="C8" s="103" t="s">
+      <c r="B8" s="106" t="s">
         <v>231</v>
       </c>
-      <c r="D8" s="105">
+      <c r="C8" s="106" t="s">
+        <v>232</v>
+      </c>
+      <c r="D8" s="108">
         <v>540.0</v>
       </c>
-      <c r="E8" s="103" t="s">
-        <v>232</v>
-      </c>
-      <c r="F8" s="109" t="s">
+      <c r="E8" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="G8" s="103" t="s">
+      <c r="F8" s="112" t="s">
         <v>234</v>
       </c>
+      <c r="G8" s="106" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="103" t="b">
+      <c r="A9" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B9" s="103" t="s">
-        <v>235</v>
-      </c>
-      <c r="C9" s="103" t="s">
+      <c r="B9" s="106" t="s">
         <v>236</v>
       </c>
-      <c r="D9" s="105">
+      <c r="C9" s="106" t="s">
+        <v>237</v>
+      </c>
+      <c r="D9" s="108">
         <v>1949.0</v>
       </c>
-      <c r="E9" s="103" t="s">
-        <v>237</v>
-      </c>
-      <c r="F9" s="103" t="s">
+      <c r="E9" s="106" t="s">
         <v>238</v>
       </c>
-      <c r="G9" s="103" t="s">
+      <c r="F9" s="106" t="s">
         <v>239</v>
       </c>
+      <c r="G9" s="106" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="103" t="b">
+      <c r="A10" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B10" s="103" t="s">
-        <v>240</v>
-      </c>
-      <c r="C10" s="103" t="s">
+      <c r="B10" s="106" t="s">
         <v>241</v>
       </c>
-      <c r="D10" s="105">
+      <c r="C10" s="106" t="s">
+        <v>242</v>
+      </c>
+      <c r="D10" s="108">
         <v>240.0</v>
       </c>
-      <c r="E10" s="103" t="s">
-        <v>242</v>
-      </c>
-      <c r="F10" s="103" t="s">
+      <c r="E10" s="106" t="s">
         <v>243</v>
       </c>
-      <c r="G10" s="103" t="s">
+      <c r="F10" s="106" t="s">
         <v>244</v>
       </c>
+      <c r="G10" s="106" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="103" t="b">
+      <c r="A11" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B11" s="103" t="s">
-        <v>245</v>
-      </c>
-      <c r="C11" s="103" t="s">
+      <c r="B11" s="106" t="s">
         <v>246</v>
       </c>
-      <c r="D11" s="105">
+      <c r="C11" s="106" t="s">
+        <v>247</v>
+      </c>
+      <c r="D11" s="108">
         <v>400.0</v>
       </c>
-      <c r="E11" s="103" t="s">
+      <c r="E11" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F11" s="106" t="s">
+        <v>249</v>
+      </c>
+      <c r="G11" s="106" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="106" t="b">
+        <v>0</v>
+      </c>
+      <c r="B12" s="106" t="s">
+        <v>251</v>
+      </c>
+      <c r="C12" s="106" t="s">
         <v>247</v>
       </c>
-      <c r="F11" s="103" t="s">
+      <c r="D12" s="108">
+        <v>350.0</v>
+      </c>
+      <c r="E12" s="106" t="s">
         <v>248</v>
       </c>
-      <c r="G11" s="103" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="103" t="b">
+      <c r="F12" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G12" s="106" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B12" s="103" t="s">
-        <v>250</v>
-      </c>
-      <c r="C12" s="103" t="s">
-        <v>246</v>
-      </c>
-      <c r="D12" s="105">
+      <c r="B13" s="106" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" s="106" t="s">
+        <v>247</v>
+      </c>
+      <c r="D13" s="108">
         <v>350.0</v>
       </c>
-      <c r="E12" s="103" t="s">
+      <c r="E13" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F13" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G13" s="106" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="106" t="b">
+        <v>0</v>
+      </c>
+      <c r="B14" s="106" t="s">
+        <v>256</v>
+      </c>
+      <c r="C14" s="106" t="s">
         <v>247</v>
       </c>
-      <c r="F12" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G12" s="103" t="s">
+      <c r="D14" s="108">
+        <v>350.0</v>
+      </c>
+      <c r="E14" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F14" s="106" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="103" t="b">
+      <c r="G14" s="106" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B13" s="103" t="s">
-        <v>253</v>
-      </c>
-      <c r="C13" s="103" t="s">
-        <v>246</v>
-      </c>
-      <c r="D13" s="105">
-        <v>350.0</v>
-      </c>
-      <c r="E13" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F13" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G13" s="103" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="103" t="b">
+      <c r="B15" s="106" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="D15" s="108">
+        <v>500.0</v>
+      </c>
+      <c r="E15" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F15" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G15" s="106" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B14" s="103" t="s">
-        <v>255</v>
-      </c>
-      <c r="C14" s="103" t="s">
-        <v>246</v>
-      </c>
-      <c r="D14" s="105">
-        <v>350.0</v>
-      </c>
-      <c r="E14" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F14" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G14" s="103" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="103" t="b">
+      <c r="B16" s="106" t="s">
+        <v>260</v>
+      </c>
+      <c r="C16" s="106" t="s">
+        <v>261</v>
+      </c>
+      <c r="D16" s="108">
+        <v>1000.0</v>
+      </c>
+      <c r="E16" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F16" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G16" s="106" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B15" s="103" t="s">
-        <v>257</v>
-      </c>
-      <c r="C15" s="103" t="s">
-        <v>258</v>
-      </c>
-      <c r="D15" s="105">
+      <c r="B17" s="106" t="s">
+        <v>263</v>
+      </c>
+      <c r="C17" s="106" t="s">
+        <v>264</v>
+      </c>
+      <c r="D17" s="108">
         <v>500.0</v>
       </c>
-      <c r="E15" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F15" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G15" s="103" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="103" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="103" t="s">
-        <v>259</v>
-      </c>
-      <c r="C16" s="103" t="s">
-        <v>260</v>
-      </c>
-      <c r="D16" s="105">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F16" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G16" s="103" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="103" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="103" t="s">
-        <v>262</v>
-      </c>
-      <c r="C17" s="103" t="s">
-        <v>263</v>
-      </c>
-      <c r="D17" s="105">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F17" s="103" t="s">
-        <v>264</v>
-      </c>
-      <c r="G17" s="103" t="s">
+      <c r="E17" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F17" s="106" t="s">
         <v>265</v>
+      </c>
+      <c r="G17" s="106" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -7360,344 +7381,344 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="102" t="s">
-        <v>266</v>
+      <c r="A1" s="105" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="103" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2" s="104">
+      <c r="A2" s="106" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="107">
         <f>'Savings comparison'!D19</f>
         <v>1000</v>
       </c>
-      <c r="C2" s="105" t="s">
-        <v>210</v>
-      </c>
-      <c r="D2" s="104">
+      <c r="C2" s="108" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="107">
         <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
         <v>7031</v>
       </c>
-      <c r="E2" s="103" t="s">
-        <v>211</v>
-      </c>
-      <c r="F2" s="106">
+      <c r="E2" s="106" t="s">
+        <v>212</v>
+      </c>
+      <c r="F2" s="109">
         <v>46185.0</v>
       </c>
-      <c r="G2" s="107"/>
+      <c r="G2" s="110"/>
     </row>
     <row r="3">
-      <c r="A3" s="103" t="s">
-        <v>212</v>
+      <c r="A3" s="106" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="107"/>
-      <c r="B4" s="107"/>
-      <c r="C4" s="107"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
+      <c r="A4" s="110"/>
+      <c r="B4" s="110"/>
+      <c r="C4" s="110"/>
+      <c r="D4" s="110"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
     </row>
     <row r="5">
-      <c r="A5" s="108" t="s">
-        <v>213</v>
-      </c>
-      <c r="B5" s="108" t="s">
+      <c r="A5" s="111" t="s">
         <v>214</v>
       </c>
-      <c r="C5" s="108" t="s">
+      <c r="B5" s="111" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="108" t="s">
+      <c r="C5" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="E5" s="108" t="s">
+      <c r="D5" s="111" t="s">
         <v>217</v>
       </c>
-      <c r="F5" s="108" t="s">
+      <c r="E5" s="111" t="s">
         <v>218</v>
       </c>
-      <c r="G5" s="108" t="s">
+      <c r="F5" s="111" t="s">
         <v>219</v>
       </c>
+      <c r="G5" s="111" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="103" t="b">
+      <c r="A6" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B6" s="103" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="103" t="s">
-        <v>267</v>
-      </c>
-      <c r="D6" s="105">
+      <c r="B6" s="106" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" s="106" t="s">
+        <v>268</v>
+      </c>
+      <c r="D6" s="108">
         <v>824.0</v>
       </c>
-      <c r="E6" s="103" t="s">
-        <v>222</v>
-      </c>
-      <c r="F6" s="103" t="s">
+      <c r="E6" s="106" t="s">
         <v>223</v>
       </c>
-      <c r="G6" s="103" t="s">
+      <c r="F6" s="106" t="s">
         <v>224</v>
       </c>
+      <c r="G6" s="106" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="103" t="b">
+      <c r="A7" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="103" t="s">
-        <v>225</v>
-      </c>
-      <c r="C7" s="103" t="s">
-        <v>268</v>
-      </c>
-      <c r="D7" s="105">
+      <c r="B7" s="106" t="s">
+        <v>226</v>
+      </c>
+      <c r="C7" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="D7" s="108">
         <v>2028.0</v>
       </c>
-      <c r="E7" s="103" t="s">
-        <v>227</v>
-      </c>
-      <c r="F7" s="109" t="s">
+      <c r="E7" s="106" t="s">
         <v>228</v>
       </c>
-      <c r="G7" s="103" t="s">
+      <c r="F7" s="112" t="s">
         <v>229</v>
       </c>
+      <c r="G7" s="106" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="103" t="b">
+      <c r="A8" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B8" s="103" t="s">
-        <v>230</v>
-      </c>
-      <c r="C8" s="103" t="s">
-        <v>269</v>
-      </c>
-      <c r="D8" s="105">
+      <c r="B8" s="106" t="s">
+        <v>231</v>
+      </c>
+      <c r="C8" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="108">
         <v>540.0</v>
       </c>
-      <c r="E8" s="103" t="s">
-        <v>232</v>
-      </c>
-      <c r="F8" s="109" t="s">
+      <c r="E8" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="G8" s="103" t="s">
+      <c r="F8" s="112" t="s">
         <v>234</v>
       </c>
+      <c r="G8" s="106" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="103" t="b">
+      <c r="A9" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B9" s="103" t="s">
-        <v>235</v>
-      </c>
-      <c r="C9" s="103" t="s">
-        <v>270</v>
-      </c>
-      <c r="D9" s="105">
+      <c r="B9" s="106" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" s="106" t="s">
+        <v>271</v>
+      </c>
+      <c r="D9" s="108">
         <v>1949.0</v>
       </c>
-      <c r="E9" s="103" t="s">
-        <v>237</v>
-      </c>
-      <c r="F9" s="103" t="s">
+      <c r="E9" s="106" t="s">
         <v>238</v>
       </c>
-      <c r="G9" s="103" t="s">
+      <c r="F9" s="106" t="s">
         <v>239</v>
       </c>
+      <c r="G9" s="106" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="103" t="b">
+      <c r="A10" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B10" s="103" t="s">
-        <v>240</v>
-      </c>
-      <c r="C10" s="103" t="s">
-        <v>271</v>
-      </c>
-      <c r="D10" s="105">
+      <c r="B10" s="106" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" s="106" t="s">
+        <v>272</v>
+      </c>
+      <c r="D10" s="108">
         <v>240.0</v>
       </c>
-      <c r="E10" s="103" t="s">
-        <v>242</v>
-      </c>
-      <c r="F10" s="103" t="s">
+      <c r="E10" s="106" t="s">
         <v>243</v>
       </c>
-      <c r="G10" s="103" t="s">
+      <c r="F10" s="106" t="s">
         <v>244</v>
       </c>
+      <c r="G10" s="106" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="103" t="b">
+      <c r="A11" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B11" s="103" t="s">
-        <v>245</v>
-      </c>
-      <c r="C11" s="103" t="s">
-        <v>272</v>
-      </c>
-      <c r="D11" s="105">
+      <c r="B11" s="106" t="s">
+        <v>246</v>
+      </c>
+      <c r="C11" s="106" t="s">
+        <v>273</v>
+      </c>
+      <c r="D11" s="108">
         <v>400.0</v>
       </c>
-      <c r="E11" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F11" s="103" t="s">
+      <c r="E11" s="106" t="s">
         <v>248</v>
       </c>
-      <c r="G11" s="103" t="s">
+      <c r="F11" s="106" t="s">
         <v>249</v>
       </c>
+      <c r="G11" s="106" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="103" t="b">
+      <c r="A12" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B12" s="103" t="s">
-        <v>250</v>
-      </c>
-      <c r="C12" s="103" t="s">
-        <v>273</v>
-      </c>
-      <c r="D12" s="105">
+      <c r="B12" s="106" t="s">
+        <v>251</v>
+      </c>
+      <c r="C12" s="106" t="s">
+        <v>274</v>
+      </c>
+      <c r="D12" s="108">
         <v>350.0</v>
       </c>
-      <c r="E12" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F12" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G12" s="103" t="s">
+      <c r="E12" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F12" s="106" t="s">
         <v>252</v>
       </c>
+      <c r="G12" s="106" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="103" t="b">
+      <c r="A13" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B13" s="103" t="s">
-        <v>253</v>
-      </c>
-      <c r="C13" s="103" t="s">
-        <v>274</v>
-      </c>
-      <c r="D13" s="105">
+      <c r="B13" s="106" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" s="106" t="s">
+        <v>275</v>
+      </c>
+      <c r="D13" s="108">
         <v>350.0</v>
       </c>
-      <c r="E13" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F13" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G13" s="103" t="s">
-        <v>254</v>
+      <c r="E13" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F13" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G13" s="106" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="103" t="b">
+      <c r="A14" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B14" s="103" t="s">
-        <v>255</v>
-      </c>
-      <c r="C14" s="103" t="s">
-        <v>275</v>
-      </c>
-      <c r="D14" s="105">
+      <c r="B14" s="106" t="s">
+        <v>256</v>
+      </c>
+      <c r="C14" s="106" t="s">
+        <v>276</v>
+      </c>
+      <c r="D14" s="108">
         <v>350.0</v>
       </c>
-      <c r="E14" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F14" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G14" s="103" t="s">
-        <v>256</v>
+      <c r="E14" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F14" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G14" s="106" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="103" t="b">
+      <c r="A15" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B15" s="103" t="s">
+      <c r="B15" s="106" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" s="106" t="s">
+        <v>277</v>
+      </c>
+      <c r="D15" s="108">
+        <v>500.0</v>
+      </c>
+      <c r="E15" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F15" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G15" s="106" t="s">
         <v>257</v>
       </c>
-      <c r="C15" s="103" t="s">
-        <v>276</v>
-      </c>
-      <c r="D15" s="105">
+    </row>
+    <row r="16">
+      <c r="A16" s="106" t="b">
+        <v>0</v>
+      </c>
+      <c r="B16" s="106" t="s">
+        <v>260</v>
+      </c>
+      <c r="C16" s="106" t="s">
+        <v>278</v>
+      </c>
+      <c r="D16" s="108">
+        <v>1000.0</v>
+      </c>
+      <c r="E16" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F16" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G16" s="106" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="b">
+        <v>0</v>
+      </c>
+      <c r="B17" s="106" t="s">
+        <v>263</v>
+      </c>
+      <c r="C17" s="106" t="s">
+        <v>279</v>
+      </c>
+      <c r="D17" s="108">
         <v>500.0</v>
       </c>
-      <c r="E15" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F15" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G15" s="103" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="103" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="103" t="s">
-        <v>259</v>
-      </c>
-      <c r="C16" s="103" t="s">
-        <v>277</v>
-      </c>
-      <c r="D16" s="105">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F16" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G16" s="103" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="103" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="103" t="s">
-        <v>262</v>
-      </c>
-      <c r="C17" s="103" t="s">
-        <v>278</v>
-      </c>
-      <c r="D17" s="105">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F17" s="103" t="s">
-        <v>264</v>
-      </c>
-      <c r="G17" s="103" t="s">
+      <c r="E17" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F17" s="106" t="s">
         <v>265</v>
+      </c>
+      <c r="G17" s="106" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -7729,344 +7750,344 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="102" t="s">
-        <v>279</v>
+      <c r="A1" s="105" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="103" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2" s="104">
+      <c r="A2" s="106" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="107">
         <f>'Savings comparison'!E19</f>
         <v>1200</v>
       </c>
-      <c r="C2" s="105" t="s">
-        <v>210</v>
-      </c>
-      <c r="D2" s="104">
+      <c r="C2" s="108" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="107">
         <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
         <v>7531</v>
       </c>
-      <c r="E2" s="103" t="s">
-        <v>211</v>
-      </c>
-      <c r="F2" s="106">
+      <c r="E2" s="106" t="s">
+        <v>212</v>
+      </c>
+      <c r="F2" s="109">
         <v>46185.0</v>
       </c>
-      <c r="G2" s="107"/>
+      <c r="G2" s="110"/>
     </row>
     <row r="3">
-      <c r="A3" s="103" t="s">
-        <v>212</v>
+      <c r="A3" s="106" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="107"/>
-      <c r="B4" s="107"/>
-      <c r="C4" s="107"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
+      <c r="A4" s="110"/>
+      <c r="B4" s="110"/>
+      <c r="C4" s="110"/>
+      <c r="D4" s="110"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
     </row>
     <row r="5">
-      <c r="A5" s="108" t="s">
-        <v>213</v>
-      </c>
-      <c r="B5" s="108" t="s">
+      <c r="A5" s="111" t="s">
         <v>214</v>
       </c>
-      <c r="C5" s="108" t="s">
+      <c r="B5" s="111" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="108" t="s">
+      <c r="C5" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="E5" s="108" t="s">
+      <c r="D5" s="111" t="s">
         <v>217</v>
       </c>
-      <c r="F5" s="108" t="s">
+      <c r="E5" s="111" t="s">
         <v>218</v>
       </c>
-      <c r="G5" s="108" t="s">
+      <c r="F5" s="111" t="s">
         <v>219</v>
       </c>
+      <c r="G5" s="111" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="103" t="b">
+      <c r="A6" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B6" s="103" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="103" t="s">
-        <v>267</v>
-      </c>
-      <c r="D6" s="105">
+      <c r="B6" s="106" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" s="106" t="s">
+        <v>268</v>
+      </c>
+      <c r="D6" s="108">
         <v>824.0</v>
       </c>
-      <c r="E6" s="103" t="s">
-        <v>222</v>
-      </c>
-      <c r="F6" s="103" t="s">
+      <c r="E6" s="106" t="s">
         <v>223</v>
       </c>
-      <c r="G6" s="103" t="s">
+      <c r="F6" s="106" t="s">
         <v>224</v>
       </c>
+      <c r="G6" s="106" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="103" t="b">
+      <c r="A7" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="103" t="s">
-        <v>225</v>
-      </c>
-      <c r="C7" s="103" t="s">
-        <v>268</v>
-      </c>
-      <c r="D7" s="105">
+      <c r="B7" s="106" t="s">
+        <v>226</v>
+      </c>
+      <c r="C7" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="D7" s="108">
         <v>2028.0</v>
       </c>
-      <c r="E7" s="103" t="s">
-        <v>227</v>
-      </c>
-      <c r="F7" s="109" t="s">
+      <c r="E7" s="106" t="s">
         <v>228</v>
       </c>
-      <c r="G7" s="103" t="s">
+      <c r="F7" s="112" t="s">
         <v>229</v>
       </c>
+      <c r="G7" s="106" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="103" t="b">
+      <c r="A8" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B8" s="103" t="s">
-        <v>230</v>
-      </c>
-      <c r="C8" s="103" t="s">
-        <v>269</v>
-      </c>
-      <c r="D8" s="105">
+      <c r="B8" s="106" t="s">
+        <v>231</v>
+      </c>
+      <c r="C8" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="108">
         <v>540.0</v>
       </c>
-      <c r="E8" s="103" t="s">
-        <v>232</v>
-      </c>
-      <c r="F8" s="109" t="s">
+      <c r="E8" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="G8" s="103" t="s">
+      <c r="F8" s="112" t="s">
         <v>234</v>
       </c>
+      <c r="G8" s="106" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="103" t="b">
+      <c r="A9" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B9" s="103" t="s">
-        <v>235</v>
-      </c>
-      <c r="C9" s="103" t="s">
-        <v>270</v>
-      </c>
-      <c r="D9" s="105">
+      <c r="B9" s="106" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" s="106" t="s">
+        <v>271</v>
+      </c>
+      <c r="D9" s="108">
         <v>1949.0</v>
       </c>
-      <c r="E9" s="103" t="s">
-        <v>237</v>
-      </c>
-      <c r="F9" s="103" t="s">
+      <c r="E9" s="106" t="s">
         <v>238</v>
       </c>
-      <c r="G9" s="103" t="s">
+      <c r="F9" s="106" t="s">
         <v>239</v>
       </c>
+      <c r="G9" s="106" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="103" t="b">
+      <c r="A10" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B10" s="103" t="s">
-        <v>240</v>
-      </c>
-      <c r="C10" s="103" t="s">
-        <v>271</v>
-      </c>
-      <c r="D10" s="105">
+      <c r="B10" s="106" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" s="106" t="s">
+        <v>272</v>
+      </c>
+      <c r="D10" s="108">
         <v>240.0</v>
       </c>
-      <c r="E10" s="103" t="s">
-        <v>242</v>
-      </c>
-      <c r="F10" s="103" t="s">
+      <c r="E10" s="106" t="s">
         <v>243</v>
       </c>
-      <c r="G10" s="103" t="s">
+      <c r="F10" s="106" t="s">
         <v>244</v>
       </c>
+      <c r="G10" s="106" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="103" t="b">
+      <c r="A11" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B11" s="103" t="s">
-        <v>245</v>
-      </c>
-      <c r="C11" s="103" t="s">
-        <v>272</v>
-      </c>
-      <c r="D11" s="105">
+      <c r="B11" s="106" t="s">
+        <v>246</v>
+      </c>
+      <c r="C11" s="106" t="s">
+        <v>273</v>
+      </c>
+      <c r="D11" s="108">
         <v>400.0</v>
       </c>
-      <c r="E11" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F11" s="103" t="s">
+      <c r="E11" s="106" t="s">
         <v>248</v>
       </c>
-      <c r="G11" s="103" t="s">
+      <c r="F11" s="106" t="s">
         <v>249</v>
       </c>
+      <c r="G11" s="106" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="103" t="b">
+      <c r="A12" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B12" s="103" t="s">
-        <v>250</v>
-      </c>
-      <c r="C12" s="103" t="s">
-        <v>273</v>
-      </c>
-      <c r="D12" s="105">
+      <c r="B12" s="106" t="s">
+        <v>251</v>
+      </c>
+      <c r="C12" s="106" t="s">
+        <v>274</v>
+      </c>
+      <c r="D12" s="108">
         <v>350.0</v>
       </c>
-      <c r="E12" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F12" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G12" s="103" t="s">
+      <c r="E12" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F12" s="106" t="s">
         <v>252</v>
       </c>
+      <c r="G12" s="106" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="103" t="b">
+      <c r="A13" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B13" s="103" t="s">
-        <v>253</v>
-      </c>
-      <c r="C13" s="103" t="s">
-        <v>274</v>
-      </c>
-      <c r="D13" s="105">
+      <c r="B13" s="106" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" s="106" t="s">
+        <v>275</v>
+      </c>
+      <c r="D13" s="108">
         <v>350.0</v>
       </c>
-      <c r="E13" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F13" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G13" s="103" t="s">
-        <v>254</v>
+      <c r="E13" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F13" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G13" s="106" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="103" t="b">
+      <c r="A14" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B14" s="103" t="s">
-        <v>255</v>
-      </c>
-      <c r="C14" s="103" t="s">
-        <v>275</v>
-      </c>
-      <c r="D14" s="105">
+      <c r="B14" s="106" t="s">
+        <v>256</v>
+      </c>
+      <c r="C14" s="106" t="s">
+        <v>276</v>
+      </c>
+      <c r="D14" s="108">
         <v>350.0</v>
       </c>
-      <c r="E14" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F14" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G14" s="103" t="s">
-        <v>256</v>
+      <c r="E14" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F14" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G14" s="106" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="103" t="b">
+      <c r="A15" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B15" s="103" t="s">
+      <c r="B15" s="106" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" s="106" t="s">
+        <v>281</v>
+      </c>
+      <c r="D15" s="108">
+        <v>500.0</v>
+      </c>
+      <c r="E15" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F15" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G15" s="106" t="s">
         <v>257</v>
       </c>
-      <c r="C15" s="103" t="s">
-        <v>280</v>
-      </c>
-      <c r="D15" s="105">
+    </row>
+    <row r="16">
+      <c r="A16" s="106" t="b">
+        <v>0</v>
+      </c>
+      <c r="B16" s="106" t="s">
+        <v>260</v>
+      </c>
+      <c r="C16" s="106" t="s">
+        <v>278</v>
+      </c>
+      <c r="D16" s="108">
+        <v>1000.0</v>
+      </c>
+      <c r="E16" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F16" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G16" s="106" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="b">
+        <v>0</v>
+      </c>
+      <c r="B17" s="106" t="s">
+        <v>263</v>
+      </c>
+      <c r="C17" s="106" t="s">
+        <v>279</v>
+      </c>
+      <c r="D17" s="108">
         <v>500.0</v>
       </c>
-      <c r="E15" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F15" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G15" s="103" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="103" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="103" t="s">
-        <v>259</v>
-      </c>
-      <c r="C16" s="103" t="s">
-        <v>277</v>
-      </c>
-      <c r="D16" s="105">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F16" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G16" s="103" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="103" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="103" t="s">
-        <v>262</v>
-      </c>
-      <c r="C17" s="103" t="s">
-        <v>278</v>
-      </c>
-      <c r="D17" s="105">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F17" s="103" t="s">
-        <v>264</v>
-      </c>
-      <c r="G17" s="103" t="s">
+      <c r="E17" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F17" s="106" t="s">
         <v>265</v>
+      </c>
+      <c r="G17" s="106" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -8098,344 +8119,344 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="102" t="s">
-        <v>281</v>
+      <c r="A1" s="105" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="103" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2" s="104">
+      <c r="A2" s="106" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="107">
         <f>'Savings comparison'!F19</f>
         <v>1600</v>
       </c>
-      <c r="C2" s="105" t="s">
-        <v>210</v>
-      </c>
-      <c r="D2" s="104">
+      <c r="C2" s="108" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="107">
         <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
         <v>8531</v>
       </c>
-      <c r="E2" s="103" t="s">
-        <v>211</v>
-      </c>
-      <c r="F2" s="106">
+      <c r="E2" s="106" t="s">
+        <v>212</v>
+      </c>
+      <c r="F2" s="109">
         <v>46185.0</v>
       </c>
-      <c r="G2" s="107"/>
+      <c r="G2" s="110"/>
     </row>
     <row r="3">
-      <c r="A3" s="103" t="s">
-        <v>212</v>
+      <c r="A3" s="106" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="107"/>
-      <c r="B4" s="107"/>
-      <c r="C4" s="107"/>
-      <c r="D4" s="107"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
+      <c r="A4" s="110"/>
+      <c r="B4" s="110"/>
+      <c r="C4" s="110"/>
+      <c r="D4" s="110"/>
+      <c r="E4" s="110"/>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
     </row>
     <row r="5">
-      <c r="A5" s="108" t="s">
-        <v>213</v>
-      </c>
-      <c r="B5" s="108" t="s">
+      <c r="A5" s="111" t="s">
         <v>214</v>
       </c>
-      <c r="C5" s="108" t="s">
+      <c r="B5" s="111" t="s">
         <v>215</v>
       </c>
-      <c r="D5" s="108" t="s">
+      <c r="C5" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="E5" s="108" t="s">
+      <c r="D5" s="111" t="s">
         <v>217</v>
       </c>
-      <c r="F5" s="108" t="s">
+      <c r="E5" s="111" t="s">
         <v>218</v>
       </c>
-      <c r="G5" s="108" t="s">
+      <c r="F5" s="111" t="s">
         <v>219</v>
       </c>
+      <c r="G5" s="111" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="103" t="b">
+      <c r="A6" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B6" s="103" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" s="103" t="s">
-        <v>267</v>
-      </c>
-      <c r="D6" s="105">
+      <c r="B6" s="106" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" s="106" t="s">
+        <v>268</v>
+      </c>
+      <c r="D6" s="108">
         <v>824.0</v>
       </c>
-      <c r="E6" s="103" t="s">
-        <v>222</v>
-      </c>
-      <c r="F6" s="103" t="s">
+      <c r="E6" s="106" t="s">
         <v>223</v>
       </c>
-      <c r="G6" s="103" t="s">
+      <c r="F6" s="106" t="s">
         <v>224</v>
       </c>
+      <c r="G6" s="106" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="103" t="b">
+      <c r="A7" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="103" t="s">
-        <v>225</v>
-      </c>
-      <c r="C7" s="103" t="s">
-        <v>268</v>
-      </c>
-      <c r="D7" s="105">
+      <c r="B7" s="106" t="s">
+        <v>226</v>
+      </c>
+      <c r="C7" s="106" t="s">
+        <v>269</v>
+      </c>
+      <c r="D7" s="108">
         <v>2028.0</v>
       </c>
-      <c r="E7" s="103" t="s">
-        <v>227</v>
-      </c>
-      <c r="F7" s="109" t="s">
+      <c r="E7" s="106" t="s">
         <v>228</v>
       </c>
-      <c r="G7" s="103" t="s">
+      <c r="F7" s="112" t="s">
         <v>229</v>
       </c>
+      <c r="G7" s="106" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="103" t="b">
+      <c r="A8" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B8" s="103" t="s">
-        <v>230</v>
-      </c>
-      <c r="C8" s="103" t="s">
-        <v>269</v>
-      </c>
-      <c r="D8" s="105">
+      <c r="B8" s="106" t="s">
+        <v>231</v>
+      </c>
+      <c r="C8" s="106" t="s">
+        <v>270</v>
+      </c>
+      <c r="D8" s="108">
         <v>540.0</v>
       </c>
-      <c r="E8" s="103" t="s">
-        <v>232</v>
-      </c>
-      <c r="F8" s="109" t="s">
+      <c r="E8" s="106" t="s">
         <v>233</v>
       </c>
-      <c r="G8" s="103" t="s">
+      <c r="F8" s="112" t="s">
         <v>234</v>
       </c>
+      <c r="G8" s="106" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="103" t="b">
+      <c r="A9" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B9" s="103" t="s">
-        <v>235</v>
-      </c>
-      <c r="C9" s="103" t="s">
-        <v>270</v>
-      </c>
-      <c r="D9" s="105">
+      <c r="B9" s="106" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" s="106" t="s">
+        <v>271</v>
+      </c>
+      <c r="D9" s="108">
         <v>1949.0</v>
       </c>
-      <c r="E9" s="103" t="s">
-        <v>237</v>
-      </c>
-      <c r="F9" s="103" t="s">
+      <c r="E9" s="106" t="s">
         <v>238</v>
       </c>
-      <c r="G9" s="103" t="s">
+      <c r="F9" s="106" t="s">
         <v>239</v>
       </c>
+      <c r="G9" s="106" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="103" t="b">
+      <c r="A10" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B10" s="103" t="s">
-        <v>240</v>
-      </c>
-      <c r="C10" s="103" t="s">
-        <v>271</v>
-      </c>
-      <c r="D10" s="105">
+      <c r="B10" s="106" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" s="106" t="s">
+        <v>272</v>
+      </c>
+      <c r="D10" s="108">
         <v>240.0</v>
       </c>
-      <c r="E10" s="103" t="s">
-        <v>242</v>
-      </c>
-      <c r="F10" s="103" t="s">
+      <c r="E10" s="106" t="s">
         <v>243</v>
       </c>
-      <c r="G10" s="103" t="s">
+      <c r="F10" s="106" t="s">
         <v>244</v>
       </c>
+      <c r="G10" s="106" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="103" t="b">
+      <c r="A11" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B11" s="103" t="s">
-        <v>245</v>
-      </c>
-      <c r="C11" s="103" t="s">
-        <v>272</v>
-      </c>
-      <c r="D11" s="105">
+      <c r="B11" s="106" t="s">
+        <v>246</v>
+      </c>
+      <c r="C11" s="106" t="s">
+        <v>273</v>
+      </c>
+      <c r="D11" s="108">
         <v>400.0</v>
       </c>
-      <c r="E11" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F11" s="103" t="s">
+      <c r="E11" s="106" t="s">
         <v>248</v>
       </c>
-      <c r="G11" s="103" t="s">
+      <c r="F11" s="106" t="s">
         <v>249</v>
       </c>
+      <c r="G11" s="106" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="103" t="b">
+      <c r="A12" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B12" s="103" t="s">
-        <v>250</v>
-      </c>
-      <c r="C12" s="103" t="s">
-        <v>273</v>
-      </c>
-      <c r="D12" s="105">
+      <c r="B12" s="106" t="s">
+        <v>251</v>
+      </c>
+      <c r="C12" s="106" t="s">
+        <v>274</v>
+      </c>
+      <c r="D12" s="108">
         <v>350.0</v>
       </c>
-      <c r="E12" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F12" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G12" s="103" t="s">
+      <c r="E12" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F12" s="106" t="s">
         <v>252</v>
       </c>
+      <c r="G12" s="106" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="103" t="b">
+      <c r="A13" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B13" s="103" t="s">
-        <v>253</v>
-      </c>
-      <c r="C13" s="103" t="s">
-        <v>274</v>
-      </c>
-      <c r="D13" s="105">
+      <c r="B13" s="106" t="s">
+        <v>254</v>
+      </c>
+      <c r="C13" s="106" t="s">
+        <v>275</v>
+      </c>
+      <c r="D13" s="108">
         <v>350.0</v>
       </c>
-      <c r="E13" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F13" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G13" s="103" t="s">
-        <v>254</v>
+      <c r="E13" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F13" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G13" s="106" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="103" t="b">
+      <c r="A14" s="106" t="b">
         <v>1</v>
       </c>
-      <c r="B14" s="103" t="s">
-        <v>255</v>
-      </c>
-      <c r="C14" s="103" t="s">
-        <v>275</v>
-      </c>
-      <c r="D14" s="105">
+      <c r="B14" s="106" t="s">
+        <v>256</v>
+      </c>
+      <c r="C14" s="106" t="s">
+        <v>276</v>
+      </c>
+      <c r="D14" s="108">
         <v>350.0</v>
       </c>
-      <c r="E14" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F14" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G14" s="103" t="s">
-        <v>256</v>
+      <c r="E14" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F14" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G14" s="106" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="103" t="b">
+      <c r="A15" s="106" t="b">
         <v>0</v>
       </c>
-      <c r="B15" s="103" t="s">
+      <c r="B15" s="106" t="s">
+        <v>258</v>
+      </c>
+      <c r="C15" s="106" t="s">
+        <v>283</v>
+      </c>
+      <c r="D15" s="108">
+        <v>500.0</v>
+      </c>
+      <c r="E15" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F15" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G15" s="106" t="s">
         <v>257</v>
       </c>
-      <c r="C15" s="103" t="s">
-        <v>282</v>
-      </c>
-      <c r="D15" s="105">
+    </row>
+    <row r="16">
+      <c r="A16" s="106" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" s="106" t="s">
+        <v>260</v>
+      </c>
+      <c r="C16" s="106" t="s">
+        <v>284</v>
+      </c>
+      <c r="D16" s="108">
+        <v>1000.0</v>
+      </c>
+      <c r="E16" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F16" s="106" t="s">
+        <v>252</v>
+      </c>
+      <c r="G16" s="106" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" s="106" t="s">
+        <v>263</v>
+      </c>
+      <c r="C17" s="106" t="s">
+        <v>285</v>
+      </c>
+      <c r="D17" s="108">
         <v>500.0</v>
       </c>
-      <c r="E15" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F15" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G15" s="103" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="103" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" s="103" t="s">
-        <v>259</v>
-      </c>
-      <c r="C16" s="103" t="s">
-        <v>283</v>
-      </c>
-      <c r="D16" s="105">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F16" s="103" t="s">
-        <v>251</v>
-      </c>
-      <c r="G16" s="103" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="103" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" s="103" t="s">
-        <v>262</v>
-      </c>
-      <c r="C17" s="103" t="s">
-        <v>284</v>
-      </c>
-      <c r="D17" s="105">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="103" t="s">
-        <v>247</v>
-      </c>
-      <c r="F17" s="103" t="s">
-        <v>264</v>
-      </c>
-      <c r="G17" s="103" t="s">
+      <c r="E17" s="106" t="s">
+        <v>248</v>
+      </c>
+      <c r="F17" s="106" t="s">
         <v>265</v>
+      </c>
+      <c r="G17" s="106" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consolidate savings service checklist
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -6,18 +6,17 @@
     <sheet state="visible" name="Savings comparison" sheetId="1" r:id="rId5"/>
     <sheet state="visible" name="Assumptions" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="P&amp;L - add-on" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Option 1 services" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Option 2 services" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="Option 3 services" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="Option 4 services" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="Services checklist" sheetId="4" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Services checklist'!$A$6:$J$18</definedName>
+  </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="268">
   <si>
     <t>Savings Calculation Template</t>
   </si>
@@ -646,7 +645,7 @@
     <t>Keep this add-on hidden from the client conversation until an option has been selected.</t>
   </si>
   <si>
-    <t>Option 1 services</t>
+    <t>Services checklist</t>
   </si>
   <si>
     <t>RB option fee</t>
@@ -655,39 +654,30 @@
     <t>Standalone DE market value checked</t>
   </si>
   <si>
-    <t>Reference date</t>
-  </si>
-  <si>
     <t>Status: provisional. Source: RB service list plus public DE pricing references. Review market prices before client reliance.</t>
   </si>
   <si>
-    <t>Included</t>
-  </si>
-  <si>
     <t>Service</t>
   </si>
   <si>
+    <t>Standalone DE market estimate</t>
+  </si>
+  <si>
+    <t>Basis</t>
+  </si>
+  <si>
+    <t>Reference URL</t>
+  </si>
+  <si>
+    <t>Reference note</t>
+  </si>
+  <si>
     <t>RB / client discussion point</t>
   </si>
   <si>
-    <t>Standalone DE market estimate</t>
-  </si>
-  <si>
-    <t>Basis</t>
-  </si>
-  <si>
-    <t>Reference URL</t>
-  </si>
-  <si>
-    <t>Reference note</t>
-  </si>
-  <si>
     <t>Basic operating entity review</t>
   </si>
   <si>
-    <t>Accounting, legal and structuring intake; no optimisation work</t>
-  </si>
-  <si>
     <t>One-off</t>
   </si>
   <si>
@@ -697,12 +687,12 @@
     <t>firma.de tax consultation 89, legal consultation 135, Startup Satzung 599</t>
   </si>
   <si>
+    <t>Accounting, legal and structuring intake</t>
+  </si>
+  <si>
     <t>Monthly bookkeeping/accounting package</t>
   </si>
   <si>
-    <t>Market benchmark if client buys bookkeeping separately</t>
-  </si>
-  <si>
     <t>Annual, 169 per month</t>
   </si>
   <si>
@@ -712,12 +702,12 @@
     <t>firma.de Basis bookkeeping package 169 per month</t>
   </si>
   <si>
+    <t>Accounting support benchmark in DE</t>
+  </si>
+  <si>
     <t>VAT compliance / VAT filings</t>
   </si>
   <si>
-    <t>Market benchmark for periodic VAT support</t>
-  </si>
-  <si>
     <t>Annual planning estimate</t>
   </si>
   <si>
@@ -727,12 +717,12 @@
     <t>StBVV section 24 sets VAT filing fee ranges; use as review benchmark</t>
   </si>
   <si>
+    <t>VAT support benchmark</t>
+  </si>
+  <si>
     <t>Annual accounts and corporate tax filings</t>
   </si>
   <si>
-    <t>Market benchmark for annual accounts and corporate filings</t>
-  </si>
-  <si>
     <t>Annual</t>
   </si>
   <si>
@@ -742,12 +732,12 @@
     <t>firma.de Basis annual accounts 1949; StBVV sections 24 and 35 support statutory fee basis</t>
   </si>
   <si>
+    <t>Annual accounts and corporate filings benchmark</t>
+  </si>
+  <si>
     <t>Payroll for one employee</t>
   </si>
   <si>
-    <t>Market benchmark for one employee payroll</t>
-  </si>
-  <si>
     <t>Annual, 19.99 per month rounded</t>
   </si>
   <si>
@@ -757,12 +747,12 @@
     <t>firma.de Starter payroll 19.99 per month; StBVV section 34 payroll range 6-30 per employee per period</t>
   </si>
   <si>
+    <t>One employee payroll benchmark</t>
+  </si>
+  <si>
     <t>Office rent / company-address optimisation</t>
   </si>
   <si>
-    <t>Not included in basic operating entity option</t>
-  </si>
-  <si>
     <t>One-off planning estimate</t>
   </si>
   <si>
@@ -772,6 +762,9 @@
     <t>Benchmark uses tax and legal consultation plus address-market reference</t>
   </si>
   <si>
+    <t>Optimise office rent or company-rented workspace arrangement</t>
+  </si>
+  <si>
     <t>Business travel and expense policy optimisation</t>
   </si>
   <si>
@@ -781,97 +774,49 @@
     <t>StBVV section 18 gives travel-cost framework; consultation benchmark anchors pricing</t>
   </si>
   <si>
+    <t>Optimise business travel and other eligible expenses</t>
+  </si>
+  <si>
     <t>Car purchase / depreciation planning</t>
   </si>
   <si>
     <t>StBVV sections 24 and 35 plus tax consultation benchmark</t>
   </si>
   <si>
+    <t>Optimise company car purchase and depreciation planning</t>
+  </si>
+  <si>
     <t>Investment / retained-profit planning</t>
   </si>
   <si>
     <t>StBVV section 22 written-opinion basis plus tax consultation benchmark</t>
   </si>
   <si>
+    <t>Help with investment and retained-profit planning</t>
+  </si>
+  <si>
     <t>Pension reserve planning</t>
   </si>
   <si>
-    <t>Excluded; add Option 3 if needed</t>
+    <t>Tax-efficient pension / pension reserve planning</t>
   </si>
   <si>
     <t>Dual tax jurisdiction / IE-DE tax residence review</t>
   </si>
   <si>
-    <t>Excluded; add Option 4 if company is IE tax resident</t>
-  </si>
-  <si>
     <t>Complex cross-border written-opinion benchmark under StBVV section 22</t>
   </si>
   <si>
+    <t>IE tax residence, not IE-resident person</t>
+  </si>
+  <si>
     <t>Director fee planning / director-service structuring</t>
   </si>
   <si>
-    <t>Excluded; add Option 4 if director fee is required</t>
-  </si>
-  <si>
     <t>https://www.firma.de/beratung-anwalt/ | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/satzung/</t>
   </si>
   <si>
     <t>Legal plus tax consultation and company-constitution pricing benchmark</t>
-  </si>
-  <si>
-    <t>Option 2 services</t>
-  </si>
-  <si>
-    <t>Accounting, legal and structuring intake</t>
-  </si>
-  <si>
-    <t>Accounting support benchmark in DE</t>
-  </si>
-  <si>
-    <t>VAT support benchmark</t>
-  </si>
-  <si>
-    <t>Annual accounts and corporate filings benchmark</t>
-  </si>
-  <si>
-    <t>One employee payroll benchmark</t>
-  </si>
-  <si>
-    <t>Optimise office rent or company-rented workspace arrangement</t>
-  </si>
-  <si>
-    <t>Optimise business travel and other eligible expenses</t>
-  </si>
-  <si>
-    <t>Optimise company car purchase and depreciation planning</t>
-  </si>
-  <si>
-    <t>Help with investment and retained-profit planning</t>
-  </si>
-  <si>
-    <t>Excluded from Option 2; add Option 3 if needed</t>
-  </si>
-  <si>
-    <t>Excluded unless company is IE tax resident</t>
-  </si>
-  <si>
-    <t>Excluded unless director fee is required</t>
-  </si>
-  <si>
-    <t>Option 3 services</t>
-  </si>
-  <si>
-    <t>Tax-efficient pension / pension reserve planning</t>
-  </si>
-  <si>
-    <t>Option 4 services</t>
-  </si>
-  <si>
-    <t>Excluded unless added separately</t>
-  </si>
-  <si>
-    <t>IE tax residence, not IE-resident person</t>
   </si>
   <si>
     <t>Discounted director-support line in RB option</t>
@@ -887,9 +832,9 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="0.0%;[Red](0.0%);-"/>
-    <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="169" formatCode="€#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -960,11 +905,24 @@
       <name val="Carlito"/>
     </font>
     <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Carlito"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.0"/>
+      <color rgb="FF4A4A4A"/>
+      <name val="Carlito"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <color rgb="FF0000FF"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1019,8 +977,26 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF15312C"/>
+        <bgColor rgb="FF15312C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6EEE7"/>
+        <bgColor rgb="FFE6EEE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F1F1"/>
+        <bgColor rgb="FFF1F1F1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="17">
+  <borders count="26">
     <border/>
     <border>
       <left style="thin">
@@ -1207,11 +1183,137 @@
         <color rgb="FF21352E"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDBDBDB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDBDBDB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDBDBDB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDBDBDB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDBDBDB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDBDBDB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDBDBDB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDBDBDB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDBDBDB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDBDBDB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDBDBDB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDBDBDB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDBDBDB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDBDBDB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDBDBDB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDBDBDB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDBDBDB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDBDBDB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDBDBDB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDBDBDB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDBDBDB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDBDBDB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDBDBDB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDBDBDB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="124">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1481,28 +1583,61 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="165" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="17" fillId="10" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="18" fillId="10" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="19" fillId="10" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="20" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="21" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="21" fillId="0" fontId="11" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="21" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="22" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="21" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="23" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="24" fillId="0" fontId="11" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1526,18 +1661,6 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -7003,15 +7126,15 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="84.25"/>
-    <col customWidth="1" min="2" max="2" width="13.13"/>
-    <col customWidth="1" min="3" max="3" width="13.0"/>
-    <col customWidth="1" min="4" max="4" width="13.13"/>
-    <col customWidth="1" min="5" max="5" width="12.13"/>
-    <col customWidth="1" min="6" max="7" width="12.75"/>
+    <col customWidth="1" min="1" max="1" width="31.38"/>
+    <col customWidth="1" min="2" max="5" width="15.13"/>
+    <col customWidth="1" min="6" max="6" width="17.0"/>
+    <col customWidth="1" min="7" max="7" width="18.88"/>
+    <col customWidth="1" min="8" max="8" width="37.63"/>
+    <col customWidth="1" min="9" max="10" width="35.13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="27.0" customHeight="1">
       <c r="A1" s="105" t="s">
         <v>209</v>
       </c>
@@ -7024,1449 +7147,492 @@
         <f>'Savings comparison'!C19</f>
         <v>500</v>
       </c>
-      <c r="C2" s="108" t="s">
-        <v>211</v>
+      <c r="C2" s="107">
+        <f>'Savings comparison'!D19</f>
+        <v>1000</v>
       </c>
       <c r="D2" s="107">
-        <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
-        <v>824</v>
-      </c>
-      <c r="E2" s="106" t="s">
-        <v>212</v>
-      </c>
-      <c r="F2" s="109">
-        <v>46185.0</v>
-      </c>
-      <c r="G2" s="110"/>
+        <f>'Savings comparison'!E19</f>
+        <v>1200</v>
+      </c>
+      <c r="E2" s="107">
+        <f>'Savings comparison'!F19</f>
+        <v>1600</v>
+      </c>
+      <c r="F2" s="108"/>
+      <c r="G2" s="108"/>
+      <c r="H2" s="108"/>
+      <c r="I2" s="108"/>
+      <c r="J2" s="108"/>
     </row>
     <row r="3">
       <c r="A3" s="106" t="s">
+        <v>211</v>
+      </c>
+      <c r="B3" s="107">
+        <f t="shared" ref="B3:E3" si="1">SUMIF(B7:B18,TRUE,$F$7:$F$18)</f>
+        <v>824</v>
+      </c>
+      <c r="C3" s="107">
+        <f t="shared" si="1"/>
+        <v>7031</v>
+      </c>
+      <c r="D3" s="107">
+        <f t="shared" si="1"/>
+        <v>7531</v>
+      </c>
+      <c r="E3" s="107">
+        <f t="shared" si="1"/>
+        <v>8531</v>
+      </c>
+      <c r="F3" s="108"/>
+      <c r="G3" s="108"/>
+      <c r="H3" s="108"/>
+      <c r="I3" s="108"/>
+      <c r="J3" s="108"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="109" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="108"/>
+      <c r="B5" s="108"/>
+      <c r="C5" s="108"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="108"/>
+      <c r="F5" s="108"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="108"/>
+      <c r="I5" s="108"/>
+      <c r="J5" s="108"/>
+    </row>
+    <row r="6" ht="39.0" customHeight="1">
+      <c r="A6" s="110" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="110"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="111" t="s">
+      <c r="B6" s="111" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="111" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="111" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="111" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="111" t="s">
         <v>214</v>
       </c>
-      <c r="B5" s="111" t="s">
+      <c r="G6" s="111" t="s">
         <v>215</v>
       </c>
-      <c r="C5" s="111" t="s">
+      <c r="H6" s="111" t="s">
         <v>216</v>
       </c>
-      <c r="D5" s="111" t="s">
+      <c r="I6" s="111" t="s">
         <v>217</v>
       </c>
-      <c r="E5" s="111" t="s">
+      <c r="J6" s="112" t="s">
         <v>218</v>
       </c>
-      <c r="F5" s="111" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" s="113" t="s">
         <v>219</v>
       </c>
-      <c r="G5" s="111" t="s">
+      <c r="B7" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="115">
+        <v>824.0</v>
+      </c>
+      <c r="G7" s="116" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="106" t="b">
+      <c r="H7" s="116" t="s">
+        <v>221</v>
+      </c>
+      <c r="I7" s="116" t="s">
+        <v>222</v>
+      </c>
+      <c r="J7" s="117" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="113" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C8" s="114" t="b">
         <v>1</v>
       </c>
-      <c r="B6" s="106" t="s">
-        <v>221</v>
-      </c>
-      <c r="C6" s="106" t="s">
-        <v>222</v>
-      </c>
-      <c r="D6" s="108">
-        <v>824.0</v>
-      </c>
-      <c r="E6" s="106" t="s">
-        <v>223</v>
-      </c>
-      <c r="F6" s="106" t="s">
-        <v>224</v>
-      </c>
-      <c r="G6" s="106" t="s">
+      <c r="D8" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="115">
+        <v>2028.0</v>
+      </c>
+      <c r="G8" s="116" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="106" t="b">
+      <c r="H8" s="118" t="s">
+        <v>226</v>
+      </c>
+      <c r="I8" s="116" t="s">
+        <v>227</v>
+      </c>
+      <c r="J8" s="117" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="113" t="s">
+        <v>229</v>
+      </c>
+      <c r="B9" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B7" s="106" t="s">
-        <v>226</v>
-      </c>
-      <c r="C7" s="106" t="s">
-        <v>227</v>
-      </c>
-      <c r="D7" s="108">
-        <v>2028.0</v>
-      </c>
-      <c r="E7" s="106" t="s">
-        <v>228</v>
-      </c>
-      <c r="F7" s="112" t="s">
-        <v>229</v>
-      </c>
-      <c r="G7" s="106" t="s">
+      <c r="C9" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="115">
+        <v>540.0</v>
+      </c>
+      <c r="G9" s="116" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="106" t="b">
+      <c r="H9" s="118" t="s">
+        <v>231</v>
+      </c>
+      <c r="I9" s="116" t="s">
+        <v>232</v>
+      </c>
+      <c r="J9" s="117" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="113" t="s">
+        <v>234</v>
+      </c>
+      <c r="B10" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B8" s="106" t="s">
-        <v>231</v>
-      </c>
-      <c r="C8" s="106" t="s">
-        <v>232</v>
-      </c>
-      <c r="D8" s="108">
-        <v>540.0</v>
-      </c>
-      <c r="E8" s="106" t="s">
-        <v>233</v>
-      </c>
-      <c r="F8" s="112" t="s">
-        <v>234</v>
-      </c>
-      <c r="G8" s="106" t="s">
+      <c r="C10" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="115">
+        <v>1949.0</v>
+      </c>
+      <c r="G10" s="116" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="106" t="b">
+      <c r="H10" s="116" t="s">
+        <v>236</v>
+      </c>
+      <c r="I10" s="116" t="s">
+        <v>237</v>
+      </c>
+      <c r="J10" s="117" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="113" t="s">
+        <v>239</v>
+      </c>
+      <c r="B11" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B9" s="106" t="s">
-        <v>236</v>
-      </c>
-      <c r="C9" s="106" t="s">
-        <v>237</v>
-      </c>
-      <c r="D9" s="108">
-        <v>1949.0</v>
-      </c>
-      <c r="E9" s="106" t="s">
-        <v>238</v>
-      </c>
-      <c r="F9" s="106" t="s">
-        <v>239</v>
-      </c>
-      <c r="G9" s="106" t="s">
+      <c r="C11" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="115">
+        <v>240.0</v>
+      </c>
+      <c r="G11" s="116" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="106" t="b">
+      <c r="H11" s="116" t="s">
+        <v>241</v>
+      </c>
+      <c r="I11" s="116" t="s">
+        <v>242</v>
+      </c>
+      <c r="J11" s="117" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="113" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B10" s="106" t="s">
-        <v>241</v>
-      </c>
-      <c r="C10" s="106" t="s">
-        <v>242</v>
-      </c>
-      <c r="D10" s="108">
-        <v>240.0</v>
-      </c>
-      <c r="E10" s="106" t="s">
-        <v>243</v>
-      </c>
-      <c r="F10" s="106" t="s">
-        <v>244</v>
-      </c>
-      <c r="G10" s="106" t="s">
+      <c r="C12" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="115">
+        <v>400.0</v>
+      </c>
+      <c r="G12" s="116" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="106" t="b">
+      <c r="H12" s="116" t="s">
+        <v>246</v>
+      </c>
+      <c r="I12" s="116" t="s">
+        <v>247</v>
+      </c>
+      <c r="J12" s="117" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="113" t="s">
+        <v>249</v>
+      </c>
+      <c r="B13" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B11" s="106" t="s">
-        <v>246</v>
-      </c>
-      <c r="C11" s="106" t="s">
-        <v>247</v>
-      </c>
-      <c r="D11" s="108">
-        <v>400.0</v>
-      </c>
-      <c r="E11" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F11" s="106" t="s">
-        <v>249</v>
-      </c>
-      <c r="G11" s="106" t="s">
+      <c r="C13" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="115">
+        <v>350.0</v>
+      </c>
+      <c r="G13" s="116" t="s">
+        <v>245</v>
+      </c>
+      <c r="H13" s="116" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="106" t="b">
+      <c r="I13" s="116" t="s">
+        <v>251</v>
+      </c>
+      <c r="J13" s="117" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="113" t="s">
+        <v>253</v>
+      </c>
+      <c r="B14" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B12" s="106" t="s">
-        <v>251</v>
-      </c>
-      <c r="C12" s="106" t="s">
-        <v>247</v>
-      </c>
-      <c r="D12" s="108">
+      <c r="C14" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="115">
         <v>350.0</v>
       </c>
-      <c r="E12" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F12" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G12" s="106" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="106" t="b">
+      <c r="G14" s="116" t="s">
+        <v>245</v>
+      </c>
+      <c r="H14" s="116" t="s">
+        <v>250</v>
+      </c>
+      <c r="I14" s="116" t="s">
+        <v>254</v>
+      </c>
+      <c r="J14" s="117" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="113" t="s">
+        <v>256</v>
+      </c>
+      <c r="B15" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B13" s="106" t="s">
-        <v>254</v>
-      </c>
-      <c r="C13" s="106" t="s">
-        <v>247</v>
-      </c>
-      <c r="D13" s="108">
+      <c r="C15" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="115">
         <v>350.0</v>
       </c>
-      <c r="E13" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F13" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G13" s="106" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="106" t="b">
+      <c r="G15" s="116" t="s">
+        <v>245</v>
+      </c>
+      <c r="H15" s="116" t="s">
+        <v>250</v>
+      </c>
+      <c r="I15" s="116" t="s">
+        <v>257</v>
+      </c>
+      <c r="J15" s="117" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="113" t="s">
+        <v>259</v>
+      </c>
+      <c r="B16" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B14" s="106" t="s">
-        <v>256</v>
-      </c>
-      <c r="C14" s="106" t="s">
-        <v>247</v>
-      </c>
-      <c r="D14" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E14" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F14" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G14" s="106" t="s">
+      <c r="C16" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="115">
+        <v>500.0</v>
+      </c>
+      <c r="G16" s="116" t="s">
+        <v>245</v>
+      </c>
+      <c r="H16" s="116" t="s">
+        <v>250</v>
+      </c>
+      <c r="I16" s="116" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="106" t="b">
+      <c r="J16" s="117" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="113" t="s">
+        <v>261</v>
+      </c>
+      <c r="B17" s="114" t="b">
         <v>0</v>
       </c>
-      <c r="B15" s="106" t="s">
-        <v>258</v>
-      </c>
-      <c r="C15" s="106" t="s">
-        <v>259</v>
-      </c>
-      <c r="D15" s="108">
+      <c r="C17" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="115">
+        <v>1000.0</v>
+      </c>
+      <c r="G17" s="116" t="s">
+        <v>245</v>
+      </c>
+      <c r="H17" s="116" t="s">
+        <v>250</v>
+      </c>
+      <c r="I17" s="116" t="s">
+        <v>262</v>
+      </c>
+      <c r="J17" s="117" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="119" t="s">
+        <v>264</v>
+      </c>
+      <c r="B18" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C18" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" s="121">
         <v>500.0</v>
       </c>
-      <c r="E15" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F15" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G15" s="106" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="106" t="s">
-        <v>260</v>
-      </c>
-      <c r="C16" s="106" t="s">
-        <v>261</v>
-      </c>
-      <c r="D16" s="108">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F16" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G16" s="106" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="106" t="s">
-        <v>263</v>
-      </c>
-      <c r="C17" s="106" t="s">
-        <v>264</v>
-      </c>
-      <c r="D17" s="108">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F17" s="106" t="s">
+      <c r="G18" s="122" t="s">
+        <v>245</v>
+      </c>
+      <c r="H18" s="122" t="s">
         <v>265</v>
       </c>
-      <c r="G17" s="106" t="s">
+      <c r="I18" s="122" t="s">
         <v>266</v>
       </c>
+      <c r="J18" s="123" t="s">
+        <v>267</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="$A$6:$J$18"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A4:J4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="F7"/>
-    <hyperlink r:id="rId2" ref="F8"/>
-  </hyperlinks>
-  <drawing r:id="rId3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="84.25"/>
-    <col customWidth="1" min="2" max="2" width="13.13"/>
-    <col customWidth="1" min="3" max="3" width="13.0"/>
-    <col customWidth="1" min="4" max="4" width="13.13"/>
-    <col customWidth="1" min="5" max="5" width="12.13"/>
-    <col customWidth="1" min="6" max="7" width="12.75"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="105" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="106" t="s">
-        <v>210</v>
-      </c>
-      <c r="B2" s="107">
-        <f>'Savings comparison'!D19</f>
-        <v>1000</v>
-      </c>
-      <c r="C2" s="108" t="s">
-        <v>211</v>
-      </c>
-      <c r="D2" s="107">
-        <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
-        <v>7031</v>
-      </c>
-      <c r="E2" s="106" t="s">
-        <v>212</v>
-      </c>
-      <c r="F2" s="109">
-        <v>46185.0</v>
-      </c>
-      <c r="G2" s="110"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="106" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="110"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="111" t="s">
-        <v>214</v>
-      </c>
-      <c r="B5" s="111" t="s">
-        <v>215</v>
-      </c>
-      <c r="C5" s="111" t="s">
-        <v>216</v>
-      </c>
-      <c r="D5" s="111" t="s">
-        <v>217</v>
-      </c>
-      <c r="E5" s="111" t="s">
-        <v>218</v>
-      </c>
-      <c r="F5" s="111" t="s">
-        <v>219</v>
-      </c>
-      <c r="G5" s="111" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B6" s="106" t="s">
-        <v>221</v>
-      </c>
-      <c r="C6" s="106" t="s">
-        <v>268</v>
-      </c>
-      <c r="D6" s="108">
-        <v>824.0</v>
-      </c>
-      <c r="E6" s="106" t="s">
-        <v>223</v>
-      </c>
-      <c r="F6" s="106" t="s">
-        <v>224</v>
-      </c>
-      <c r="G6" s="106" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" s="106" t="s">
-        <v>226</v>
-      </c>
-      <c r="C7" s="106" t="s">
-        <v>269</v>
-      </c>
-      <c r="D7" s="108">
-        <v>2028.0</v>
-      </c>
-      <c r="E7" s="106" t="s">
-        <v>228</v>
-      </c>
-      <c r="F7" s="112" t="s">
-        <v>229</v>
-      </c>
-      <c r="G7" s="106" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B8" s="106" t="s">
-        <v>231</v>
-      </c>
-      <c r="C8" s="106" t="s">
-        <v>270</v>
-      </c>
-      <c r="D8" s="108">
-        <v>540.0</v>
-      </c>
-      <c r="E8" s="106" t="s">
-        <v>233</v>
-      </c>
-      <c r="F8" s="112" t="s">
-        <v>234</v>
-      </c>
-      <c r="G8" s="106" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" s="106" t="s">
-        <v>236</v>
-      </c>
-      <c r="C9" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="D9" s="108">
-        <v>1949.0</v>
-      </c>
-      <c r="E9" s="106" t="s">
-        <v>238</v>
-      </c>
-      <c r="F9" s="106" t="s">
-        <v>239</v>
-      </c>
-      <c r="G9" s="106" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" s="106" t="s">
-        <v>241</v>
-      </c>
-      <c r="C10" s="106" t="s">
-        <v>272</v>
-      </c>
-      <c r="D10" s="108">
-        <v>240.0</v>
-      </c>
-      <c r="E10" s="106" t="s">
-        <v>243</v>
-      </c>
-      <c r="F10" s="106" t="s">
-        <v>244</v>
-      </c>
-      <c r="G10" s="106" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" s="106" t="s">
-        <v>246</v>
-      </c>
-      <c r="C11" s="106" t="s">
-        <v>273</v>
-      </c>
-      <c r="D11" s="108">
-        <v>400.0</v>
-      </c>
-      <c r="E11" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F11" s="106" t="s">
-        <v>249</v>
-      </c>
-      <c r="G11" s="106" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" s="106" t="s">
-        <v>251</v>
-      </c>
-      <c r="C12" s="106" t="s">
-        <v>274</v>
-      </c>
-      <c r="D12" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E12" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F12" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G12" s="106" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B13" s="106" t="s">
-        <v>254</v>
-      </c>
-      <c r="C13" s="106" t="s">
-        <v>275</v>
-      </c>
-      <c r="D13" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E13" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F13" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G13" s="106" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" s="106" t="s">
-        <v>256</v>
-      </c>
-      <c r="C14" s="106" t="s">
-        <v>276</v>
-      </c>
-      <c r="D14" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E14" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F14" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G14" s="106" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B15" s="106" t="s">
-        <v>258</v>
-      </c>
-      <c r="C15" s="106" t="s">
-        <v>277</v>
-      </c>
-      <c r="D15" s="108">
-        <v>500.0</v>
-      </c>
-      <c r="E15" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F15" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G15" s="106" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="106" t="s">
-        <v>260</v>
-      </c>
-      <c r="C16" s="106" t="s">
-        <v>278</v>
-      </c>
-      <c r="D16" s="108">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F16" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G16" s="106" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="106" t="s">
-        <v>263</v>
-      </c>
-      <c r="C17" s="106" t="s">
-        <v>279</v>
-      </c>
-      <c r="D17" s="108">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F17" s="106" t="s">
-        <v>265</v>
-      </c>
-      <c r="G17" s="106" t="s">
-        <v>266</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="F7"/>
-    <hyperlink r:id="rId2" ref="F8"/>
-  </hyperlinks>
-  <drawing r:id="rId3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="84.25"/>
-    <col customWidth="1" min="2" max="2" width="13.13"/>
-    <col customWidth="1" min="3" max="3" width="13.0"/>
-    <col customWidth="1" min="4" max="4" width="13.13"/>
-    <col customWidth="1" min="5" max="5" width="12.13"/>
-    <col customWidth="1" min="6" max="7" width="12.75"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="105" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="106" t="s">
-        <v>210</v>
-      </c>
-      <c r="B2" s="107">
-        <f>'Savings comparison'!E19</f>
-        <v>1200</v>
-      </c>
-      <c r="C2" s="108" t="s">
-        <v>211</v>
-      </c>
-      <c r="D2" s="107">
-        <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
-        <v>7531</v>
-      </c>
-      <c r="E2" s="106" t="s">
-        <v>212</v>
-      </c>
-      <c r="F2" s="109">
-        <v>46185.0</v>
-      </c>
-      <c r="G2" s="110"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="106" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="110"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="111" t="s">
-        <v>214</v>
-      </c>
-      <c r="B5" s="111" t="s">
-        <v>215</v>
-      </c>
-      <c r="C5" s="111" t="s">
-        <v>216</v>
-      </c>
-      <c r="D5" s="111" t="s">
-        <v>217</v>
-      </c>
-      <c r="E5" s="111" t="s">
-        <v>218</v>
-      </c>
-      <c r="F5" s="111" t="s">
-        <v>219</v>
-      </c>
-      <c r="G5" s="111" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B6" s="106" t="s">
-        <v>221</v>
-      </c>
-      <c r="C6" s="106" t="s">
-        <v>268</v>
-      </c>
-      <c r="D6" s="108">
-        <v>824.0</v>
-      </c>
-      <c r="E6" s="106" t="s">
-        <v>223</v>
-      </c>
-      <c r="F6" s="106" t="s">
-        <v>224</v>
-      </c>
-      <c r="G6" s="106" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" s="106" t="s">
-        <v>226</v>
-      </c>
-      <c r="C7" s="106" t="s">
-        <v>269</v>
-      </c>
-      <c r="D7" s="108">
-        <v>2028.0</v>
-      </c>
-      <c r="E7" s="106" t="s">
-        <v>228</v>
-      </c>
-      <c r="F7" s="112" t="s">
-        <v>229</v>
-      </c>
-      <c r="G7" s="106" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B8" s="106" t="s">
-        <v>231</v>
-      </c>
-      <c r="C8" s="106" t="s">
-        <v>270</v>
-      </c>
-      <c r="D8" s="108">
-        <v>540.0</v>
-      </c>
-      <c r="E8" s="106" t="s">
-        <v>233</v>
-      </c>
-      <c r="F8" s="112" t="s">
-        <v>234</v>
-      </c>
-      <c r="G8" s="106" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" s="106" t="s">
-        <v>236</v>
-      </c>
-      <c r="C9" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="D9" s="108">
-        <v>1949.0</v>
-      </c>
-      <c r="E9" s="106" t="s">
-        <v>238</v>
-      </c>
-      <c r="F9" s="106" t="s">
-        <v>239</v>
-      </c>
-      <c r="G9" s="106" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" s="106" t="s">
-        <v>241</v>
-      </c>
-      <c r="C10" s="106" t="s">
-        <v>272</v>
-      </c>
-      <c r="D10" s="108">
-        <v>240.0</v>
-      </c>
-      <c r="E10" s="106" t="s">
-        <v>243</v>
-      </c>
-      <c r="F10" s="106" t="s">
-        <v>244</v>
-      </c>
-      <c r="G10" s="106" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" s="106" t="s">
-        <v>246</v>
-      </c>
-      <c r="C11" s="106" t="s">
-        <v>273</v>
-      </c>
-      <c r="D11" s="108">
-        <v>400.0</v>
-      </c>
-      <c r="E11" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F11" s="106" t="s">
-        <v>249</v>
-      </c>
-      <c r="G11" s="106" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" s="106" t="s">
-        <v>251</v>
-      </c>
-      <c r="C12" s="106" t="s">
-        <v>274</v>
-      </c>
-      <c r="D12" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E12" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F12" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G12" s="106" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B13" s="106" t="s">
-        <v>254</v>
-      </c>
-      <c r="C13" s="106" t="s">
-        <v>275</v>
-      </c>
-      <c r="D13" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E13" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F13" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G13" s="106" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" s="106" t="s">
-        <v>256</v>
-      </c>
-      <c r="C14" s="106" t="s">
-        <v>276</v>
-      </c>
-      <c r="D14" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E14" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F14" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G14" s="106" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" s="106" t="s">
-        <v>258</v>
-      </c>
-      <c r="C15" s="106" t="s">
-        <v>281</v>
-      </c>
-      <c r="D15" s="108">
-        <v>500.0</v>
-      </c>
-      <c r="E15" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F15" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G15" s="106" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="106" t="s">
-        <v>260</v>
-      </c>
-      <c r="C16" s="106" t="s">
-        <v>278</v>
-      </c>
-      <c r="D16" s="108">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F16" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G16" s="106" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="106" t="s">
-        <v>263</v>
-      </c>
-      <c r="C17" s="106" t="s">
-        <v>279</v>
-      </c>
-      <c r="D17" s="108">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F17" s="106" t="s">
-        <v>265</v>
-      </c>
-      <c r="G17" s="106" t="s">
-        <v>266</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="F7"/>
-    <hyperlink r:id="rId2" ref="F8"/>
-  </hyperlinks>
-  <drawing r:id="rId3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="84.25"/>
-    <col customWidth="1" min="2" max="2" width="13.13"/>
-    <col customWidth="1" min="3" max="3" width="13.0"/>
-    <col customWidth="1" min="4" max="4" width="13.13"/>
-    <col customWidth="1" min="5" max="5" width="12.13"/>
-    <col customWidth="1" min="6" max="7" width="12.75"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="105" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="106" t="s">
-        <v>210</v>
-      </c>
-      <c r="B2" s="107">
-        <f>'Savings comparison'!F19</f>
-        <v>1600</v>
-      </c>
-      <c r="C2" s="108" t="s">
-        <v>211</v>
-      </c>
-      <c r="D2" s="107">
-        <f>SUMIF(A6:A17,TRUE,D6:D17)</f>
-        <v>8531</v>
-      </c>
-      <c r="E2" s="106" t="s">
-        <v>212</v>
-      </c>
-      <c r="F2" s="109">
-        <v>46185.0</v>
-      </c>
-      <c r="G2" s="110"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="106" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="110"/>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="111" t="s">
-        <v>214</v>
-      </c>
-      <c r="B5" s="111" t="s">
-        <v>215</v>
-      </c>
-      <c r="C5" s="111" t="s">
-        <v>216</v>
-      </c>
-      <c r="D5" s="111" t="s">
-        <v>217</v>
-      </c>
-      <c r="E5" s="111" t="s">
-        <v>218</v>
-      </c>
-      <c r="F5" s="111" t="s">
-        <v>219</v>
-      </c>
-      <c r="G5" s="111" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B6" s="106" t="s">
-        <v>221</v>
-      </c>
-      <c r="C6" s="106" t="s">
-        <v>268</v>
-      </c>
-      <c r="D6" s="108">
-        <v>824.0</v>
-      </c>
-      <c r="E6" s="106" t="s">
-        <v>223</v>
-      </c>
-      <c r="F6" s="106" t="s">
-        <v>224</v>
-      </c>
-      <c r="G6" s="106" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" s="106" t="s">
-        <v>226</v>
-      </c>
-      <c r="C7" s="106" t="s">
-        <v>269</v>
-      </c>
-      <c r="D7" s="108">
-        <v>2028.0</v>
-      </c>
-      <c r="E7" s="106" t="s">
-        <v>228</v>
-      </c>
-      <c r="F7" s="112" t="s">
-        <v>229</v>
-      </c>
-      <c r="G7" s="106" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B8" s="106" t="s">
-        <v>231</v>
-      </c>
-      <c r="C8" s="106" t="s">
-        <v>270</v>
-      </c>
-      <c r="D8" s="108">
-        <v>540.0</v>
-      </c>
-      <c r="E8" s="106" t="s">
-        <v>233</v>
-      </c>
-      <c r="F8" s="112" t="s">
-        <v>234</v>
-      </c>
-      <c r="G8" s="106" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" s="106" t="s">
-        <v>236</v>
-      </c>
-      <c r="C9" s="106" t="s">
-        <v>271</v>
-      </c>
-      <c r="D9" s="108">
-        <v>1949.0</v>
-      </c>
-      <c r="E9" s="106" t="s">
-        <v>238</v>
-      </c>
-      <c r="F9" s="106" t="s">
-        <v>239</v>
-      </c>
-      <c r="G9" s="106" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" s="106" t="s">
-        <v>241</v>
-      </c>
-      <c r="C10" s="106" t="s">
-        <v>272</v>
-      </c>
-      <c r="D10" s="108">
-        <v>240.0</v>
-      </c>
-      <c r="E10" s="106" t="s">
-        <v>243</v>
-      </c>
-      <c r="F10" s="106" t="s">
-        <v>244</v>
-      </c>
-      <c r="G10" s="106" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" s="106" t="s">
-        <v>246</v>
-      </c>
-      <c r="C11" s="106" t="s">
-        <v>273</v>
-      </c>
-      <c r="D11" s="108">
-        <v>400.0</v>
-      </c>
-      <c r="E11" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F11" s="106" t="s">
-        <v>249</v>
-      </c>
-      <c r="G11" s="106" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" s="106" t="s">
-        <v>251</v>
-      </c>
-      <c r="C12" s="106" t="s">
-        <v>274</v>
-      </c>
-      <c r="D12" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E12" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F12" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G12" s="106" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B13" s="106" t="s">
-        <v>254</v>
-      </c>
-      <c r="C13" s="106" t="s">
-        <v>275</v>
-      </c>
-      <c r="D13" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E13" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F13" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G13" s="106" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" s="106" t="s">
-        <v>256</v>
-      </c>
-      <c r="C14" s="106" t="s">
-        <v>276</v>
-      </c>
-      <c r="D14" s="108">
-        <v>350.0</v>
-      </c>
-      <c r="E14" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F14" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G14" s="106" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="106" t="b">
-        <v>0</v>
-      </c>
-      <c r="B15" s="106" t="s">
-        <v>258</v>
-      </c>
-      <c r="C15" s="106" t="s">
-        <v>283</v>
-      </c>
-      <c r="D15" s="108">
-        <v>500.0</v>
-      </c>
-      <c r="E15" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F15" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G15" s="106" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" s="106" t="s">
-        <v>260</v>
-      </c>
-      <c r="C16" s="106" t="s">
-        <v>284</v>
-      </c>
-      <c r="D16" s="108">
-        <v>1000.0</v>
-      </c>
-      <c r="E16" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F16" s="106" t="s">
-        <v>252</v>
-      </c>
-      <c r="G16" s="106" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="106" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" s="106" t="s">
-        <v>263</v>
-      </c>
-      <c r="C17" s="106" t="s">
-        <v>285</v>
-      </c>
-      <c r="D17" s="108">
-        <v>500.0</v>
-      </c>
-      <c r="E17" s="106" t="s">
-        <v>248</v>
-      </c>
-      <c r="F17" s="106" t="s">
-        <v>265</v>
-      </c>
-      <c r="G17" s="106" t="s">
-        <v>266</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="F7"/>
-    <hyperlink r:id="rId2" ref="F8"/>
+    <hyperlink r:id="rId1" ref="H8"/>
+    <hyperlink r:id="rId2" ref="H9"/>
   </hyperlinks>
   <drawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand savings service checklist
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -9,14 +9,14 @@
     <sheet state="visible" name="Services checklist" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Services checklist'!$A$6:$J$18</definedName>
+    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Services checklist'!$A$6:$J$38</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="347">
   <si>
     <t>Savings Calculation Template</t>
   </si>
@@ -654,7 +654,7 @@
     <t>Standalone DE market value checked</t>
   </si>
   <si>
-    <t>Status: provisional. Source: RB service list plus public DE pricing references. Review market prices before client reliance.</t>
+    <t>Status: provisional. Source: RB Client Process Database search, user corrections, and public pricing references. Review market prices before client reliance.</t>
   </si>
   <si>
     <t>Service</t>
@@ -690,31 +690,64 @@
     <t>Accounting, legal and structuring intake</t>
   </si>
   <si>
+    <t>Company incorporation and compliance approval</t>
+  </si>
+  <si>
+    <t>One-off setup estimate</t>
+  </si>
+  <si>
+    <t>https://www.firma.de/satzung/ | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/</t>
+  </si>
+  <si>
+    <t>Benchmark combines company document, legal and tax setup support</t>
+  </si>
+  <si>
+    <t>Set up the operating entity and compliance basis before optimisation work</t>
+  </si>
+  <si>
+    <t>Client records, document intake and onboarding handover</t>
+  </si>
+  <si>
+    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
+  </si>
+  <si>
+    <t>StBVV time-fee basis for setup and administrative handover</t>
+  </si>
+  <si>
+    <t>Collect client data, documents and handover information into the operating workflow</t>
+  </si>
+  <si>
     <t>Monthly bookkeeping/accounting package</t>
   </si>
   <si>
     <t>Annual, 169 per month</t>
   </si>
   <si>
-    <t>https://www.firma.de/buchhaltung/</t>
-  </si>
-  <si>
-    <t>firma.de Basis bookkeeping package 169 per month</t>
+    <t>https://www.firma.de/buchhaltung/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
+  </si>
+  <si>
+    <t>firma.de Basis bookkeeping package 169 per month; StBVV section 33 supports bookkeeping fee basis</t>
   </si>
   <si>
     <t>Accounting support benchmark in DE</t>
   </si>
   <si>
+    <t>Bookkeeping software setup and filing calendar setup</t>
+  </si>
+  <si>
+    <t>StBVV section 32 supports bookkeeping setup time-fee basis</t>
+  </si>
+  <si>
+    <t>Set up bookkeeping tooling and filing dates so recurring work runs correctly</t>
+  </si>
+  <si>
     <t>VAT compliance / VAT filings</t>
   </si>
   <si>
     <t>Annual planning estimate</t>
   </si>
   <si>
-    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>StBVV section 24 sets VAT filing fee ranges; use as review benchmark</t>
+    <t>StBVV section 24 sets VAT filing fee ranges; includes VIES/RTD-style filings where applicable</t>
   </si>
   <si>
     <t>VAT support benchmark</t>
@@ -747,39 +780,105 @@
     <t>firma.de Starter payroll 19.99 per month; StBVV section 34 payroll range 6-30 per employee per period</t>
   </si>
   <si>
-    <t>One employee payroll benchmark</t>
+    <t>One employee recurring payroll benchmark</t>
+  </si>
+  <si>
+    <t>Payroll setup, retroactive payslips and filings</t>
+  </si>
+  <si>
+    <t>One-off or incident estimate</t>
+  </si>
+  <si>
+    <t>StBVV section 34 covers payroll setup and related payroll support</t>
+  </si>
+  <si>
+    <t>Set up payroll, repair missing periods, generate payslips and handle filings</t>
   </si>
   <si>
     <t>Office rent / company-address optimisation</t>
   </si>
   <si>
+    <t>Advisory setup + recurring monthly administration</t>
+  </si>
+  <si>
+    <t>https://www.firma.de/geschaeftsadresse/ | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/</t>
+  </si>
+  <si>
+    <t>Benchmark combines tax/legal advice, address-market reference and recurring administration; actual rent excluded</t>
+  </si>
+  <si>
+    <t>Advise on structure, analyse rent benchmarks, prepare the contract and administer monthly company rent payments under the contract</t>
+  </si>
+  <si>
+    <t>Business travel and expense policy optimisation</t>
+  </si>
+  <si>
+    <t>Policy setup + recurring per diem/reimbursement administration</t>
+  </si>
+  <si>
+    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/buchhaltung/</t>
+  </si>
+  <si>
+    <t>StBVV section 18 travel-cost framework plus bookkeeping/admin benchmark</t>
+  </si>
+  <si>
+    <t>Advise on correct organisation, track trips and per diems, calculate reimbursement amounts and pay back correctly from the company</t>
+  </si>
+  <si>
+    <t>AP/AR (invoice generation, expense payment, chasing, logging)</t>
+  </si>
+  <si>
+    <t>Annual, 100 per month planning estimate</t>
+  </si>
+  <si>
+    <t>Monthly bookkeeping/admin benchmark for invoice and payment operations</t>
+  </si>
+  <si>
+    <t>Generate invoices, log expenses, pay expenses, chase receivables and keep records current</t>
+  </si>
+  <si>
+    <t>Tax prepayments and tax payments tracking</t>
+  </si>
+  <si>
+    <t>StBVV tax-admin and payment-support benchmark</t>
+  </si>
+  <si>
+    <t>Track prepayments, tax payments and due dates so cash and filings stay aligned</t>
+  </si>
+  <si>
+    <t>Tax registration and Finanzamt correspondence</t>
+  </si>
+  <si>
+    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html | https://www.firma.de/beratung-steuerberater/</t>
+  </si>
+  <si>
+    <t>Tax registration and authority correspondence benchmarked against StBVV time/advisory fees</t>
+  </si>
+  <si>
+    <t>Handle tax registration and routine Finanzamt correspondence for the client</t>
+  </si>
+  <si>
+    <t>Authority, health insurer and penalty/fine resolution</t>
+  </si>
+  <si>
+    <t>Per-incident planning estimate</t>
+  </si>
+  <si>
+    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/</t>
+  </si>
+  <si>
+    <t>StBVV sections for authority discussions/appeals plus legal/tax consultation anchors</t>
+  </si>
+  <si>
+    <t>Call Finanzamt, health insurers and other authorities; investigate penalties and fight fines where supportable</t>
+  </si>
+  <si>
+    <t>Car purchase / depreciation planning</t>
+  </si>
+  <si>
     <t>One-off planning estimate</t>
   </si>
   <si>
-    <t>https://www.firma.de/geschaeftsadresse/ | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/</t>
-  </si>
-  <si>
-    <t>Benchmark uses tax and legal consultation plus address-market reference</t>
-  </si>
-  <si>
-    <t>Optimise office rent or company-rented workspace arrangement</t>
-  </si>
-  <si>
-    <t>Business travel and expense policy optimisation</t>
-  </si>
-  <si>
-    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html | https://www.firma.de/beratung-steuerberater/</t>
-  </si>
-  <si>
-    <t>StBVV section 18 gives travel-cost framework; consultation benchmark anchors pricing</t>
-  </si>
-  <si>
-    <t>Optimise business travel and other eligible expenses</t>
-  </si>
-  <si>
-    <t>Car purchase / depreciation planning</t>
-  </si>
-  <si>
     <t>StBVV sections 24 and 35 plus tax consultation benchmark</t>
   </si>
   <si>
@@ -795,6 +894,15 @@
     <t>Help with investment and retained-profit planning</t>
   </si>
   <si>
+    <t>Investment account setup</t>
+  </si>
+  <si>
+    <t>Planning estimate for administrative setup and records</t>
+  </si>
+  <si>
+    <t>Support setup of an investment account and align documentation with accounting treatment</t>
+  </si>
+  <si>
     <t>Pension reserve planning</t>
   </si>
   <si>
@@ -820,6 +928,135 @@
   </si>
   <si>
     <t>Discounted director-support line in RB option</t>
+  </si>
+  <si>
+    <t>Employer number, accident insurance and VBG registrations</t>
+  </si>
+  <si>
+    <t>https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service | https://www.dguv.de/de/versicherung/mitgliedschaft/index.jsp | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
+  </si>
+  <si>
+    <t>Public registration routes plus StBVV time-fee support benchmark</t>
+  </si>
+  <si>
+    <t>Apply for employer number, accident insurance number and VBG-style registration where required</t>
+  </si>
+  <si>
+    <t>Local business registration (Gewerbeanmeldung)</t>
+  </si>
+  <si>
+    <t>https://service.berlin.de/dienstleistung/121921/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
+  </si>
+  <si>
+    <t>Public filing route plus advisor support benchmark; government fees excluded</t>
+  </si>
+  <si>
+    <t>Handle local business registration where required</t>
+  </si>
+  <si>
+    <t>Bank account setup</t>
+  </si>
+  <si>
+    <t>Planning estimate for administrative setup and evidence handling</t>
+  </si>
+  <si>
+    <t>Support bank-account setup and capture records for accounting</t>
+  </si>
+  <si>
+    <t>Service agreement contracts with client customers</t>
+  </si>
+  <si>
+    <t>Per-contract planning estimate</t>
+  </si>
+  <si>
+    <t>https://www.firma.de/beratung-anwalt/ | https://www.firma.de/satzung/</t>
+  </si>
+  <si>
+    <t>Legal consultation and company-document benchmark</t>
+  </si>
+  <si>
+    <t>Prepare or review service agreement contracts between the company and its customers</t>
+  </si>
+  <si>
+    <t>Employment contract changes</t>
+  </si>
+  <si>
+    <t>Per-change planning estimate</t>
+  </si>
+  <si>
+    <t>https://www.firma.de/beratung-anwalt/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
+  </si>
+  <si>
+    <t>Legal consultation plus payroll/tax support benchmark</t>
+  </si>
+  <si>
+    <t>Change employment/director contracts and align payroll/accounting treatment</t>
+  </si>
+  <si>
+    <t>Share subscription agreements</t>
+  </si>
+  <si>
+    <t>Per-document planning estimate</t>
+  </si>
+  <si>
+    <t>Prepare share subscription agreements where the structure needs them</t>
+  </si>
+  <si>
+    <t>RBO / beneficial-owner filing where applicable</t>
+  </si>
+  <si>
+    <t>One-off or annual planning estimate</t>
+  </si>
+  <si>
+    <t>https://rbo.gov.ie/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
+  </si>
+  <si>
+    <t>Official RBO filing route plus administrative support benchmark</t>
+  </si>
+  <si>
+    <t>Handle beneficial-owner filing where an IE structure requires it</t>
+  </si>
+  <si>
+    <t>Personal tax bookkeeping and filing add-on</t>
+  </si>
+  <si>
+    <t>Annual add-on estimate</t>
+  </si>
+  <si>
+    <t>StBVV personal tax filing and income calculation basis</t>
+  </si>
+  <si>
+    <t>Optional personal tax bookkeeping and personal filing support outside the core option fee</t>
+  </si>
+  <si>
+    <t>Parental leave planning</t>
+  </si>
+  <si>
+    <t>One-off add-on estimate</t>
+  </si>
+  <si>
+    <t>Planning estimate for advisory and calculation support</t>
+  </si>
+  <si>
+    <t>Optional planning for parental leave and owner salary timing</t>
+  </si>
+  <si>
+    <t>Client forecast and life-change planning</t>
+  </si>
+  <si>
+    <t>Tax/advisory benchmark for annual planning and life-change scenarios</t>
+  </si>
+  <si>
+    <t>Refresh client forecast for the new year and after material life/business changes</t>
+  </si>
+  <si>
+    <t>Client calls, inbounds and periodic updates</t>
+  </si>
+  <si>
+    <t>StBVV time-fee benchmark for ongoing client support</t>
+  </si>
+  <si>
+    <t>Handle client calls, inbound messages, meeting notes and monthly/quarterly updates</t>
   </si>
 </sst>
 </file>
@@ -834,7 +1071,7 @@
     <numFmt numFmtId="168" formatCode="0.0%;[Red](0.0%);-"/>
     <numFmt numFmtId="169" formatCode="€#,##0"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -916,6 +1153,10 @@
       <color rgb="FF4A4A4A"/>
       <name val="Carlito"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -1313,7 +1554,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="125">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1635,6 +1876,9 @@
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="24" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="25" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -7138,6 +7382,15 @@
       <c r="A1" s="105" t="s">
         <v>209</v>
       </c>
+      <c r="B1" s="105"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="105"/>
+      <c r="G1" s="105"/>
+      <c r="H1" s="105"/>
+      <c r="I1" s="105"/>
+      <c r="J1" s="105"/>
     </row>
     <row r="2">
       <c r="A2" s="106" t="s">
@@ -7170,20 +7423,20 @@
         <v>211</v>
       </c>
       <c r="B3" s="107">
-        <f t="shared" ref="B3:E3" si="1">SUMIF(B7:B18,TRUE,$F$7:$F$18)</f>
-        <v>824</v>
+        <f t="shared" ref="B3:E3" si="1">SUMIF(B7:B38,TRUE,$F$7:$F$38)</f>
+        <v>1724</v>
       </c>
       <c r="C3" s="107">
         <f t="shared" si="1"/>
-        <v>7031</v>
+        <v>16881</v>
       </c>
       <c r="D3" s="107">
         <f t="shared" si="1"/>
-        <v>7531</v>
+        <v>17381</v>
       </c>
       <c r="E3" s="107">
         <f t="shared" si="1"/>
-        <v>8531</v>
+        <v>18131</v>
       </c>
       <c r="F3" s="108"/>
       <c r="G3" s="108"/>
@@ -7195,6 +7448,15 @@
       <c r="A4" s="109" t="s">
         <v>212</v>
       </c>
+      <c r="B4" s="109"/>
+      <c r="C4" s="109"/>
+      <c r="D4" s="109"/>
+      <c r="E4" s="109"/>
+      <c r="F4" s="109"/>
+      <c r="G4" s="109"/>
+      <c r="H4" s="109"/>
+      <c r="I4" s="109"/>
+      <c r="J4" s="109"/>
     </row>
     <row r="5">
       <c r="A5" s="108"/>
@@ -7208,7 +7470,7 @@
       <c r="I5" s="108"/>
       <c r="J5" s="108"/>
     </row>
-    <row r="6" ht="39.0" customHeight="1">
+    <row r="6" ht="42.0" customHeight="1">
       <c r="A6" s="110" t="s">
         <v>213</v>
       </c>
@@ -7240,7 +7502,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="52.5" customHeight="1">
       <c r="A7" s="113" t="s">
         <v>219</v>
       </c>
@@ -7272,12 +7534,12 @@
         <v>223</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="52.5" customHeight="1">
       <c r="A8" s="113" t="s">
         <v>224</v>
       </c>
       <c r="B8" s="114" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="114" t="b">
         <v>1</v>
@@ -7289,12 +7551,12 @@
         <v>1</v>
       </c>
       <c r="F8" s="115">
-        <v>2028.0</v>
+        <v>900.0</v>
       </c>
       <c r="G8" s="116" t="s">
         <v>225</v>
       </c>
-      <c r="H8" s="118" t="s">
+      <c r="H8" s="116" t="s">
         <v>226</v>
       </c>
       <c r="I8" s="116" t="s">
@@ -7304,7 +7566,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="52.5" customHeight="1">
       <c r="A9" s="113" t="s">
         <v>229</v>
       </c>
@@ -7321,205 +7583,205 @@
         <v>1</v>
       </c>
       <c r="F9" s="115">
+        <v>300.0</v>
+      </c>
+      <c r="G9" s="116" t="s">
+        <v>225</v>
+      </c>
+      <c r="H9" s="118" t="s">
+        <v>230</v>
+      </c>
+      <c r="I9" s="116" t="s">
+        <v>231</v>
+      </c>
+      <c r="J9" s="117" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" ht="52.5" customHeight="1">
+      <c r="A10" s="113" t="s">
+        <v>233</v>
+      </c>
+      <c r="B10" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C10" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="115">
+        <v>2028.0</v>
+      </c>
+      <c r="G10" s="116" t="s">
+        <v>234</v>
+      </c>
+      <c r="H10" s="116" t="s">
+        <v>235</v>
+      </c>
+      <c r="I10" s="116" t="s">
+        <v>236</v>
+      </c>
+      <c r="J10" s="117" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="11" ht="52.5" customHeight="1">
+      <c r="A11" s="113" t="s">
+        <v>238</v>
+      </c>
+      <c r="B11" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="115">
+        <v>300.0</v>
+      </c>
+      <c r="G11" s="116" t="s">
+        <v>225</v>
+      </c>
+      <c r="H11" s="116" t="s">
+        <v>235</v>
+      </c>
+      <c r="I11" s="116" t="s">
+        <v>239</v>
+      </c>
+      <c r="J11" s="117" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="12" ht="52.5" customHeight="1">
+      <c r="A12" s="113" t="s">
+        <v>241</v>
+      </c>
+      <c r="B12" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C12" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="115">
         <v>540.0</v>
       </c>
-      <c r="G9" s="116" t="s">
+      <c r="G12" s="116" t="s">
+        <v>242</v>
+      </c>
+      <c r="H12" s="118" t="s">
         <v>230</v>
       </c>
-      <c r="H9" s="118" t="s">
-        <v>231</v>
-      </c>
-      <c r="I9" s="116" t="s">
-        <v>232</v>
-      </c>
-      <c r="J9" s="117" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="113" t="s">
-        <v>234</v>
-      </c>
-      <c r="B10" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C10" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" s="115">
+      <c r="I12" s="116" t="s">
+        <v>243</v>
+      </c>
+      <c r="J12" s="117" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="13" ht="52.5" customHeight="1">
+      <c r="A13" s="113" t="s">
+        <v>245</v>
+      </c>
+      <c r="B13" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C13" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="115">
         <v>1949.0</v>
       </c>
-      <c r="G10" s="116" t="s">
-        <v>235</v>
-      </c>
-      <c r="H10" s="116" t="s">
-        <v>236</v>
-      </c>
-      <c r="I10" s="116" t="s">
-        <v>237</v>
-      </c>
-      <c r="J10" s="117" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="113" t="s">
-        <v>239</v>
-      </c>
-      <c r="B11" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C11" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E11" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" s="115">
+      <c r="G13" s="116" t="s">
+        <v>246</v>
+      </c>
+      <c r="H13" s="116" t="s">
+        <v>247</v>
+      </c>
+      <c r="I13" s="116" t="s">
+        <v>248</v>
+      </c>
+      <c r="J13" s="117" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" ht="52.5" customHeight="1">
+      <c r="A14" s="113" t="s">
+        <v>250</v>
+      </c>
+      <c r="B14" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C14" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="115">
         <v>240.0</v>
       </c>
-      <c r="G11" s="116" t="s">
-        <v>240</v>
-      </c>
-      <c r="H11" s="116" t="s">
-        <v>241</v>
-      </c>
-      <c r="I11" s="116" t="s">
-        <v>242</v>
-      </c>
-      <c r="J11" s="117" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="113" t="s">
-        <v>244</v>
-      </c>
-      <c r="B12" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C12" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E12" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" s="115">
-        <v>400.0</v>
-      </c>
-      <c r="G12" s="116" t="s">
-        <v>245</v>
-      </c>
-      <c r="H12" s="116" t="s">
-        <v>246</v>
-      </c>
-      <c r="I12" s="116" t="s">
-        <v>247</v>
-      </c>
-      <c r="J12" s="117" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="113" t="s">
-        <v>249</v>
-      </c>
-      <c r="B13" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C13" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E13" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" s="115">
-        <v>350.0</v>
-      </c>
-      <c r="G13" s="116" t="s">
-        <v>245</v>
-      </c>
-      <c r="H13" s="116" t="s">
-        <v>250</v>
-      </c>
-      <c r="I13" s="116" t="s">
+      <c r="G14" s="116" t="s">
         <v>251</v>
       </c>
-      <c r="J13" s="117" t="s">
+      <c r="H14" s="116" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="113" t="s">
+      <c r="I14" s="116" t="s">
         <v>253</v>
       </c>
-      <c r="B14" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C14" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E14" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" s="115">
-        <v>350.0</v>
-      </c>
-      <c r="G14" s="116" t="s">
-        <v>245</v>
-      </c>
-      <c r="H14" s="116" t="s">
-        <v>250</v>
-      </c>
-      <c r="I14" s="116" t="s">
+      <c r="J14" s="117" t="s">
         <v>254</v>
       </c>
-      <c r="J14" s="117" t="s">
+    </row>
+    <row r="15" ht="52.5" customHeight="1">
+      <c r="A15" s="113" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="113" t="s">
+      <c r="B15" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C15" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="115">
+        <v>500.0</v>
+      </c>
+      <c r="G15" s="116" t="s">
         <v>256</v>
       </c>
-      <c r="B15" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C15" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="115">
-        <v>350.0</v>
-      </c>
-      <c r="G15" s="116" t="s">
-        <v>245</v>
-      </c>
       <c r="H15" s="116" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="I15" s="116" t="s">
         <v>257</v>
@@ -7528,7 +7790,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="52.5" customHeight="1">
       <c r="A16" s="113" t="s">
         <v>259</v>
       </c>
@@ -7536,104 +7798,746 @@
         <v>0</v>
       </c>
       <c r="C16" s="114" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="114" t="b">
         <v>1</v>
       </c>
       <c r="E16" s="114" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="115">
+        <v>1200.0</v>
+      </c>
+      <c r="G16" s="116" t="s">
+        <v>260</v>
+      </c>
+      <c r="H16" s="116" t="s">
+        <v>261</v>
+      </c>
+      <c r="I16" s="116" t="s">
+        <v>262</v>
+      </c>
+      <c r="J16" s="117" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="17" ht="52.5" customHeight="1">
+      <c r="A17" s="113" t="s">
+        <v>264</v>
+      </c>
+      <c r="B17" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D17" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="115">
+        <v>900.0</v>
+      </c>
+      <c r="G17" s="116" t="s">
+        <v>265</v>
+      </c>
+      <c r="H17" s="116" t="s">
+        <v>266</v>
+      </c>
+      <c r="I17" s="116" t="s">
+        <v>267</v>
+      </c>
+      <c r="J17" s="117" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="18" ht="52.5" customHeight="1">
+      <c r="A18" s="113" t="s">
+        <v>269</v>
+      </c>
+      <c r="B18" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C18" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D18" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" s="115">
+        <v>1200.0</v>
+      </c>
+      <c r="G18" s="116" t="s">
+        <v>270</v>
+      </c>
+      <c r="H18" s="116" t="s">
+        <v>235</v>
+      </c>
+      <c r="I18" s="116" t="s">
+        <v>271</v>
+      </c>
+      <c r="J18" s="117" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="19" ht="52.5" customHeight="1">
+      <c r="A19" s="113" t="s">
+        <v>273</v>
+      </c>
+      <c r="B19" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D19" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="115">
+        <v>300.0</v>
+      </c>
+      <c r="G19" s="116" t="s">
+        <v>242</v>
+      </c>
+      <c r="H19" s="118" t="s">
+        <v>230</v>
+      </c>
+      <c r="I19" s="116" t="s">
+        <v>274</v>
+      </c>
+      <c r="J19" s="117" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="20" ht="52.5" customHeight="1">
+      <c r="A20" s="113" t="s">
+        <v>276</v>
+      </c>
+      <c r="B20" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C20" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D20" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" s="115">
+        <v>350.0</v>
+      </c>
+      <c r="G20" s="116" t="s">
+        <v>256</v>
+      </c>
+      <c r="H20" s="116" t="s">
+        <v>277</v>
+      </c>
+      <c r="I20" s="116" t="s">
+        <v>278</v>
+      </c>
+      <c r="J20" s="117" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="21" ht="52.5" customHeight="1">
+      <c r="A21" s="113" t="s">
+        <v>280</v>
+      </c>
+      <c r="B21" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C21" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D21" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" s="115">
+        <v>750.0</v>
+      </c>
+      <c r="G21" s="116" t="s">
+        <v>281</v>
+      </c>
+      <c r="H21" s="116" t="s">
+        <v>282</v>
+      </c>
+      <c r="I21" s="116" t="s">
+        <v>283</v>
+      </c>
+      <c r="J21" s="117" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="22" ht="52.5" customHeight="1">
+      <c r="A22" s="113" t="s">
+        <v>285</v>
+      </c>
+      <c r="B22" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C22" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" s="115">
+        <v>350.0</v>
+      </c>
+      <c r="G22" s="116" t="s">
+        <v>286</v>
+      </c>
+      <c r="H22" s="116" t="s">
+        <v>277</v>
+      </c>
+      <c r="I22" s="116" t="s">
+        <v>287</v>
+      </c>
+      <c r="J22" s="117" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="23" ht="52.5" customHeight="1">
+      <c r="A23" s="113" t="s">
+        <v>289</v>
+      </c>
+      <c r="B23" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C23" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" s="115">
+        <v>350.0</v>
+      </c>
+      <c r="G23" s="116" t="s">
+        <v>286</v>
+      </c>
+      <c r="H23" s="116" t="s">
+        <v>277</v>
+      </c>
+      <c r="I23" s="116" t="s">
+        <v>290</v>
+      </c>
+      <c r="J23" s="117" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="24" ht="52.5" customHeight="1">
+      <c r="A24" s="113" t="s">
+        <v>292</v>
+      </c>
+      <c r="B24" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" s="115">
+        <v>250.0</v>
+      </c>
+      <c r="G24" s="116" t="s">
+        <v>225</v>
+      </c>
+      <c r="H24" s="118" t="s">
+        <v>230</v>
+      </c>
+      <c r="I24" s="116" t="s">
+        <v>293</v>
+      </c>
+      <c r="J24" s="117" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="25" ht="52.5" customHeight="1">
+      <c r="A25" s="113" t="s">
+        <v>295</v>
+      </c>
+      <c r="B25" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C25" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D25" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" s="115">
         <v>500.0</v>
       </c>
-      <c r="G16" s="116" t="s">
-        <v>245</v>
-      </c>
-      <c r="H16" s="116" t="s">
-        <v>250</v>
-      </c>
-      <c r="I16" s="116" t="s">
-        <v>257</v>
-      </c>
-      <c r="J16" s="117" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="113" t="s">
-        <v>261</v>
-      </c>
-      <c r="B17" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="D17" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="E17" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="115">
+      <c r="G25" s="116" t="s">
+        <v>286</v>
+      </c>
+      <c r="H25" s="116" t="s">
+        <v>277</v>
+      </c>
+      <c r="I25" s="116" t="s">
+        <v>290</v>
+      </c>
+      <c r="J25" s="117" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="26" ht="52.5" customHeight="1">
+      <c r="A26" s="113" t="s">
+        <v>297</v>
+      </c>
+      <c r="B26" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C26" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E26" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" s="115">
         <v>1000.0</v>
       </c>
-      <c r="G17" s="116" t="s">
-        <v>245</v>
-      </c>
-      <c r="H17" s="116" t="s">
-        <v>250</v>
-      </c>
-      <c r="I17" s="116" t="s">
-        <v>262</v>
-      </c>
-      <c r="J17" s="117" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="119" t="s">
-        <v>264</v>
-      </c>
-      <c r="B18" s="120" t="b">
-        <v>0</v>
-      </c>
-      <c r="C18" s="120" t="b">
-        <v>0</v>
-      </c>
-      <c r="D18" s="120" t="b">
-        <v>0</v>
-      </c>
-      <c r="E18" s="120" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" s="121">
+      <c r="G26" s="116" t="s">
+        <v>286</v>
+      </c>
+      <c r="H26" s="116" t="s">
+        <v>277</v>
+      </c>
+      <c r="I26" s="116" t="s">
+        <v>298</v>
+      </c>
+      <c r="J26" s="117" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="27" ht="52.5" customHeight="1">
+      <c r="A27" s="113" t="s">
+        <v>300</v>
+      </c>
+      <c r="B27" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C27" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D27" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F27" s="115">
         <v>500.0</v>
       </c>
-      <c r="G18" s="122" t="s">
-        <v>245</v>
-      </c>
-      <c r="H18" s="122" t="s">
-        <v>265</v>
-      </c>
-      <c r="I18" s="122" t="s">
-        <v>266</v>
-      </c>
-      <c r="J18" s="123" t="s">
-        <v>267</v>
+      <c r="G27" s="116" t="s">
+        <v>286</v>
+      </c>
+      <c r="H27" s="116" t="s">
+        <v>301</v>
+      </c>
+      <c r="I27" s="116" t="s">
+        <v>302</v>
+      </c>
+      <c r="J27" s="117" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="28" ht="52.5" customHeight="1">
+      <c r="A28" s="113" t="s">
+        <v>304</v>
+      </c>
+      <c r="B28" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C28" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D28" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E28" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="F28" s="115">
+        <v>300.0</v>
+      </c>
+      <c r="G28" s="116" t="s">
+        <v>225</v>
+      </c>
+      <c r="H28" s="116" t="s">
+        <v>305</v>
+      </c>
+      <c r="I28" s="116" t="s">
+        <v>306</v>
+      </c>
+      <c r="J28" s="117" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="29" ht="52.5" customHeight="1">
+      <c r="A29" s="113" t="s">
+        <v>308</v>
+      </c>
+      <c r="B29" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C29" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E29" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="F29" s="115">
+        <v>250.0</v>
+      </c>
+      <c r="G29" s="116" t="s">
+        <v>225</v>
+      </c>
+      <c r="H29" s="116" t="s">
+        <v>309</v>
+      </c>
+      <c r="I29" s="116" t="s">
+        <v>310</v>
+      </c>
+      <c r="J29" s="117" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="30" ht="52.5" customHeight="1">
+      <c r="A30" s="113" t="s">
+        <v>312</v>
+      </c>
+      <c r="B30" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C30" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D30" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E30" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F30" s="115">
+        <v>250.0</v>
+      </c>
+      <c r="G30" s="116" t="s">
+        <v>225</v>
+      </c>
+      <c r="H30" s="118" t="s">
+        <v>230</v>
+      </c>
+      <c r="I30" s="116" t="s">
+        <v>313</v>
+      </c>
+      <c r="J30" s="117" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="31" ht="52.5" customHeight="1">
+      <c r="A31" s="113" t="s">
+        <v>315</v>
+      </c>
+      <c r="B31" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C31" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D31" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E31" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F31" s="115">
+        <v>600.0</v>
+      </c>
+      <c r="G31" s="116" t="s">
+        <v>316</v>
+      </c>
+      <c r="H31" s="116" t="s">
+        <v>317</v>
+      </c>
+      <c r="I31" s="116" t="s">
+        <v>318</v>
+      </c>
+      <c r="J31" s="117" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="32" ht="52.5" customHeight="1">
+      <c r="A32" s="113" t="s">
+        <v>320</v>
+      </c>
+      <c r="B32" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C32" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D32" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E32" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" s="115">
+        <v>500.0</v>
+      </c>
+      <c r="G32" s="116" t="s">
+        <v>321</v>
+      </c>
+      <c r="H32" s="116" t="s">
+        <v>322</v>
+      </c>
+      <c r="I32" s="116" t="s">
+        <v>323</v>
+      </c>
+      <c r="J32" s="117" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="33" ht="52.5" customHeight="1">
+      <c r="A33" s="113" t="s">
+        <v>325</v>
+      </c>
+      <c r="B33" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C33" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E33" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F33" s="115">
+        <v>650.0</v>
+      </c>
+      <c r="G33" s="116" t="s">
+        <v>326</v>
+      </c>
+      <c r="H33" s="116" t="s">
+        <v>317</v>
+      </c>
+      <c r="I33" s="116" t="s">
+        <v>318</v>
+      </c>
+      <c r="J33" s="117" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="34" ht="52.5" customHeight="1">
+      <c r="A34" s="113" t="s">
+        <v>328</v>
+      </c>
+      <c r="B34" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C34" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D34" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F34" s="115">
+        <v>300.0</v>
+      </c>
+      <c r="G34" s="116" t="s">
+        <v>329</v>
+      </c>
+      <c r="H34" s="116" t="s">
+        <v>330</v>
+      </c>
+      <c r="I34" s="116" t="s">
+        <v>331</v>
+      </c>
+      <c r="J34" s="117" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="35" ht="52.5" customHeight="1">
+      <c r="A35" s="113" t="s">
+        <v>333</v>
+      </c>
+      <c r="B35" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C35" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E35" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="F35" s="115">
+        <v>750.0</v>
+      </c>
+      <c r="G35" s="116" t="s">
+        <v>334</v>
+      </c>
+      <c r="H35" s="118" t="s">
+        <v>230</v>
+      </c>
+      <c r="I35" s="116" t="s">
+        <v>335</v>
+      </c>
+      <c r="J35" s="117" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="36" ht="52.5" customHeight="1">
+      <c r="A36" s="113" t="s">
+        <v>337</v>
+      </c>
+      <c r="B36" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C36" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="D36" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36" s="115">
+        <v>450.0</v>
+      </c>
+      <c r="G36" s="116" t="s">
+        <v>338</v>
+      </c>
+      <c r="H36" s="118" t="s">
+        <v>230</v>
+      </c>
+      <c r="I36" s="116" t="s">
+        <v>339</v>
+      </c>
+      <c r="J36" s="117" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="37" ht="52.5" customHeight="1">
+      <c r="A37" s="113" t="s">
+        <v>341</v>
+      </c>
+      <c r="B37" s="114" t="b">
+        <v>0</v>
+      </c>
+      <c r="C37" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="D37" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="E37" s="114" t="b">
+        <v>1</v>
+      </c>
+      <c r="F37" s="115">
+        <v>500.0</v>
+      </c>
+      <c r="G37" s="116" t="s">
+        <v>242</v>
+      </c>
+      <c r="H37" s="116" t="s">
+        <v>277</v>
+      </c>
+      <c r="I37" s="116" t="s">
+        <v>342</v>
+      </c>
+      <c r="J37" s="117" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="38" ht="52.5" customHeight="1">
+      <c r="A38" s="119" t="s">
+        <v>344</v>
+      </c>
+      <c r="B38" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C38" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E38" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F38" s="121">
+        <v>600.0</v>
+      </c>
+      <c r="G38" s="122" t="s">
+        <v>242</v>
+      </c>
+      <c r="H38" s="123" t="s">
+        <v>230</v>
+      </c>
+      <c r="I38" s="122" t="s">
+        <v>345</v>
+      </c>
+      <c r="J38" s="124" t="s">
+        <v>346</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$6:$J$18"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A4:J4"/>
-  </mergeCells>
+  <autoFilter ref="$A$6:$J$38"/>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="H8"/>
-    <hyperlink r:id="rId2" ref="H9"/>
+    <hyperlink r:id="rId1" ref="H9"/>
+    <hyperlink r:id="rId2" ref="H12"/>
+    <hyperlink r:id="rId3" ref="H19"/>
+    <hyperlink r:id="rId4" ref="H24"/>
+    <hyperlink r:id="rId5" ref="H30"/>
+    <hyperlink r:id="rId6" ref="H35"/>
+    <hyperlink r:id="rId7" ref="H36"/>
+    <hyperlink r:id="rId8" ref="H38"/>
   </hyperlinks>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refine savings checklist estimates
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -9,14 +9,14 @@
     <sheet state="visible" name="Services checklist" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Services checklist'!$A$6:$J$38</definedName>
+    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Services checklist'!$A$7:$J$39</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="316">
   <si>
     <t>Savings Calculation Template</t>
   </si>
@@ -651,25 +651,28 @@
     <t>RB option fee</t>
   </si>
   <si>
-    <t>Standalone DE market value checked</t>
-  </si>
-  <si>
-    <t>Status: provisional. Source: RB Client Process Database search, user corrections, and public pricing references. Review market prices before client reliance.</t>
+    <t>Standalone DE market value checked - low</t>
+  </si>
+  <si>
+    <t>Standalone DE market value checked - mid</t>
+  </si>
+  <si>
+    <t>Status: provisional. Source: RB service-list work, user corrections, and public pricing/statutory references checked 2026-06-15. Low/mid estimates include advisory support plus third-party software, filing, and public-authority costs where relevant; review before client reliance.</t>
   </si>
   <si>
     <t>Service</t>
   </si>
   <si>
-    <t>Standalone DE market estimate</t>
-  </si>
-  <si>
-    <t>Basis</t>
-  </si>
-  <si>
-    <t>Reference URL</t>
-  </si>
-  <si>
-    <t>Reference note</t>
+    <t>Low-end DE estimate</t>
+  </si>
+  <si>
+    <t>Mid-end DE estimate</t>
+  </si>
+  <si>
+    <t>Basis / cost components</t>
+  </si>
+  <si>
+    <t>Linked explanation</t>
   </si>
   <si>
     <t>RB / client discussion point</t>
@@ -678,325 +681,241 @@
     <t>Basic operating entity review</t>
   </si>
   <si>
-    <t>One-off</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/ | https://www.firma.de/satzung/</t>
-  </si>
-  <si>
-    <t>firma.de tax consultation 89, legal consultation 135, Startup Satzung 599</t>
-  </si>
-  <si>
-    <t>Accounting, legal and structuring intake</t>
+    <t>Initial entity and accounting review; low uses public tax-advice plus basic support, mid includes deeper bookkeeping/accounting scoping</t>
+  </si>
+  <si>
+    <t>Confirm entity status quo, previous accounting fee, current accountant, and whether the entity is already operational</t>
   </si>
   <si>
     <t>Company incorporation and compliance approval</t>
   </si>
   <si>
-    <t>One-off setup estimate</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/satzung/ | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/</t>
-  </si>
-  <si>
-    <t>Benchmark combines company document, legal and tax setup support</t>
-  </si>
-  <si>
-    <t>Set up the operating entity and compliance basis before optimisation work</t>
+    <t>One-off incorporation/compliance support estimate; public documents/legal review plus accounting setup oversight</t>
+  </si>
+  <si>
+    <t>Review whether a new company or operating entity approval is needed before using the template</t>
   </si>
   <si>
     <t>Client records, document intake and onboarding handover</t>
   </si>
   <si>
-    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>StBVV time-fee basis for setup and administrative handover</t>
-  </si>
-  <si>
-    <t>Collect client data, documents and handover information into the operating workflow</t>
+    <t>One-off intake estimate for source documents, records, opening balances, access, and handover into recurring operations</t>
+  </si>
+  <si>
+    <t>Collect contracts, prior filings, bank records, payroll records, authority letters, and current fee data</t>
   </si>
   <si>
     <t>Monthly bookkeeping/accounting package</t>
   </si>
   <si>
-    <t>Annual, 169 per month</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/buchhaltung/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>firma.de Basis bookkeeping package 169 per month; StBVV section 33 supports bookkeeping fee basis</t>
-  </si>
-  <si>
-    <t>Accounting support benchmark in DE</t>
+    <t>Recurring accounting package; low uses 99/month plus DATEV 15/month, mid uses 169/month plus DATEV 15/month</t>
+  </si>
+  <si>
+    <t>Bookkeeping is a recurring operating service, not a one-off advisory line</t>
   </si>
   <si>
     <t>Bookkeeping software setup and filing calendar setup</t>
   </si>
   <si>
-    <t>StBVV section 32 supports bookkeeping setup time-fee basis</t>
-  </si>
-  <si>
-    <t>Set up bookkeeping tooling and filing dates so recurring work runs correctly</t>
+    <t>Software setup, chart of accounts, filing calendar, access permissions, and recurring tool configuration; excludes monthly bookkeeping above</t>
+  </si>
+  <si>
+    <t>Make the operating calendar and software stack explicit before the client chooses the option</t>
   </si>
   <si>
     <t>VAT compliance / VAT filings</t>
   </si>
   <si>
-    <t>Annual planning estimate</t>
-  </si>
-  <si>
-    <t>StBVV section 24 sets VAT filing fee ranges; includes VIES/RTD-style filings where applicable</t>
-  </si>
-  <si>
-    <t>VAT support benchmark</t>
+    <t>Recurring VAT filing support plus filing-software/transmission setup where needed; low assumes lighter filing volume, mid assumes monthly complexity</t>
+  </si>
+  <si>
+    <t>Track VAT deadlines, prepare filings, submit returns, and retain filing/payment evidence</t>
   </si>
   <si>
     <t>Annual accounts and corporate tax filings</t>
   </si>
   <si>
-    <t>Annual</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/jahresabschluss-kapitalgesellschaft/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>firma.de Basis annual accounts 1949; StBVV sections 24 and 35 support statutory fee basis</t>
-  </si>
-  <si>
-    <t>Annual accounts and corporate filings benchmark</t>
+    <t>Annual accounts plus disclosure/filing; low uses 1249 plus 99 disclosure, mid uses 1949 plus 99 disclosure</t>
+  </si>
+  <si>
+    <t>Annual compliance is separate from monthly bookkeeping and should stay visible in the service comparison</t>
   </si>
   <si>
     <t>Payroll for one employee</t>
   </si>
   <si>
-    <t>Annual, 19.99 per month rounded</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/lohnabrechnung/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>firma.de Starter payroll 19.99 per month; StBVV section 34 payroll range 6-30 per employee per period</t>
-  </si>
-  <si>
-    <t>One employee recurring payroll benchmark</t>
+    <t>Recurring payroll plus payroll-software/filing component; low uses payroll service benchmark, mid adds Lexware payroll add-on at 12.90/month</t>
+  </si>
+  <si>
+    <t>Run payroll, social-insurance and wage-tax filings, payments, and evidence capture for the employee</t>
   </si>
   <si>
     <t>Payroll setup, retroactive payslips and filings</t>
   </si>
   <si>
-    <t>One-off or incident estimate</t>
-  </si>
-  <si>
-    <t>StBVV section 34 covers payroll setup and related payroll support</t>
-  </si>
-  <si>
-    <t>Set up payroll, repair missing periods, generate payslips and handle filings</t>
+    <t>Setup or correction project for payroll history, retroactive payslips, registrations, filings and payment reconciliation</t>
+  </si>
+  <si>
+    <t>Use when payroll history or late setup needs correction before monthly operation is clean</t>
   </si>
   <si>
     <t>Office rent / company-address optimisation</t>
   </si>
   <si>
-    <t>Advisory setup + recurring monthly administration</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/geschaeftsadresse/ | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/</t>
-  </si>
-  <si>
-    <t>Benchmark combines tax/legal advice, address-market reference and recurring administration; actual rent excluded</t>
-  </si>
-  <si>
-    <t>Advise on structure, analyse rent benchmarks, prepare the contract and administer monthly company rent payments under the contract</t>
+    <t>Advisory plus benchmark analysis, company/person rent contract, and recurring monthly rent payment administration</t>
+  </si>
+  <si>
+    <t>Advise, benchmark the office rent, prepare the contract, and pay the rent every month as agreed</t>
   </si>
   <si>
     <t>Business travel and expense policy optimisation</t>
   </si>
   <si>
-    <t>Policy setup + recurring per diem/reimbursement administration</t>
-  </si>
-  <si>
-    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/buchhaltung/</t>
-  </si>
-  <si>
-    <t>StBVV section 18 travel-cost framework plus bookkeeping/admin benchmark</t>
-  </si>
-  <si>
-    <t>Advise on correct organisation, track trips and per diems, calculate reimbursement amounts and pay back correctly from the company</t>
+    <t>Recurring travel policy, per diem calculation, receipt review, reimbursement calculation, company payment, and evidence tracking</t>
+  </si>
+  <si>
+    <t>Help the client organise correctly, calculate per diem amounts, track expenses, and reimburse from the company</t>
   </si>
   <si>
     <t>AP/AR (invoice generation, expense payment, chasing, logging)</t>
   </si>
   <si>
-    <t>Annual, 100 per month planning estimate</t>
-  </si>
-  <si>
-    <t>Monthly bookkeeping/admin benchmark for invoice and payment operations</t>
-  </si>
-  <si>
-    <t>Generate invoices, log expenses, pay expenses, chase receivables and keep records current</t>
+    <t>Recurring invoice generation, expense payment, chasing, logging and evidence matching; includes bookkeeping/payment software component</t>
+  </si>
+  <si>
+    <t>Operate invoices, supplier payments, client chasing and evidence logs instead of only advising once</t>
   </si>
   <si>
     <t>Tax prepayments and tax payments tracking</t>
   </si>
   <si>
-    <t>StBVV tax-admin and payment-support benchmark</t>
-  </si>
-  <si>
-    <t>Track prepayments, tax payments and due dates so cash and filings stay aligned</t>
-  </si>
-  <si>
-    <t>Tax registration and Finanzamt correspondence</t>
-  </si>
-  <si>
-    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html | https://www.firma.de/beratung-steuerberater/</t>
-  </si>
-  <si>
-    <t>Tax registration and authority correspondence benchmarked against StBVV time/advisory fees</t>
-  </si>
-  <si>
-    <t>Handle tax registration and routine Finanzamt correspondence for the client</t>
+    <t>Recurring tracking of tax prepayment notices, payment due dates, cash planning, executing payments, and storing payment evidence</t>
+  </si>
+  <si>
+    <t>Actively track and pay tax prepayments; this is ongoing company-order work, not a one-off log</t>
+  </si>
+  <si>
+    <t>Tax registration, letters and Finanzamt correspondence</t>
+  </si>
+  <si>
+    <t>Recurring registration management plus active reading, classification and actioning of tax letters, deadlines, objections and notices</t>
+  </si>
+  <si>
+    <t>Read tax letters, respond where needed, and keep the company in order before penalties arise</t>
   </si>
   <si>
     <t>Authority, health insurer and penalty/fine resolution</t>
   </si>
   <si>
-    <t>Per-incident planning estimate</t>
-  </si>
-  <si>
-    <t>https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/beratung-anwalt/</t>
-  </si>
-  <si>
-    <t>StBVV sections for authority discussions/appeals plus legal/tax consultation anchors</t>
-  </si>
-  <si>
-    <t>Call Finanzamt, health insurers and other authorities; investigate penalties and fight fines where supportable</t>
+    <t>Active case management: calls, letters, objections, escalation and chasing with Finanzamt, health insurers, payroll/social bodies and fine issuers</t>
+  </si>
+  <si>
+    <t>Call Finanzamt and health insurers, fight fines, and keep issue ownership until resolved</t>
   </si>
   <si>
     <t>Car purchase / depreciation planning</t>
   </si>
   <si>
-    <t>One-off planning estimate</t>
-  </si>
-  <si>
-    <t>StBVV sections 24 and 35 plus tax consultation benchmark</t>
-  </si>
-  <si>
-    <t>Optimise company car purchase and depreciation planning</t>
+    <t>Vehicle purchase, depreciation, benefit-in-kind and accounting treatment analysis; support estimate only, no vehicle cost included</t>
+  </si>
+  <si>
+    <t>Analyse car purchase and depreciation treatment before committing to the company purchase</t>
   </si>
   <si>
     <t>Investment / retained-profit planning</t>
   </si>
   <si>
-    <t>StBVV section 22 written-opinion basis plus tax consultation benchmark</t>
-  </si>
-  <si>
-    <t>Help with investment and retained-profit planning</t>
+    <t>Retained-profit investment planning and accounting/tax treatment review; advisory support estimate, not investment-management fees</t>
+  </si>
+  <si>
+    <t>Help decide whether retained profits should be invested or held for taxes, salary and reserve planning</t>
   </si>
   <si>
     <t>Investment account setup</t>
   </si>
   <si>
-    <t>Planning estimate for administrative setup and records</t>
-  </si>
-  <si>
-    <t>Support setup of an investment account and align documentation with accounting treatment</t>
+    <t>Administrative setup estimate for investment account documents, evidence, accounting treatment and source-record workflow</t>
+  </si>
+  <si>
+    <t>Set up the investment-account records correctly if the client decides to invest retained profits</t>
   </si>
   <si>
     <t>Pension reserve planning</t>
   </si>
   <si>
-    <t>Tax-efficient pension / pension reserve planning</t>
+    <t>Additional pension reserve analysis and documentation; reflected as the separate RB pension surcharge line in option 3</t>
+  </si>
+  <si>
+    <t>Only included when the client chooses the pension reserve add-on</t>
   </si>
   <si>
     <t>Dual tax jurisdiction / IE-DE tax residence review</t>
   </si>
   <si>
-    <t>Complex cross-border written-opinion benchmark under StBVV section 22</t>
-  </si>
-  <si>
-    <t>IE tax residence, not IE-resident person</t>
-  </si>
-  <si>
-    <t>Director fee planning / director-service structuring</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/beratung-anwalt/ | https://www.firma.de/beratung-steuerberater/ | https://www.firma.de/satzung/</t>
-  </si>
-  <si>
-    <t>Legal plus tax consultation and company-constitution pricing benchmark</t>
-  </si>
-  <si>
-    <t>Discounted director-support line in RB option</t>
+    <t>Cross-border tax-residence review and dual-jurisdiction coordination estimate; excludes actual director service below</t>
+  </si>
+  <si>
+    <t>Use for IE tax residence structures, not because a person is IE resident</t>
+  </si>
+  <si>
+    <t>Director fee planning / director-service structuring and board governance</t>
+  </si>
+  <si>
+    <t>Recurring actual director service plus board governance, board meetings, minutes, statutory decisions and keeping the company in order</t>
+  </si>
+  <si>
+    <t>This is an actual director required to operate governance and board meetings, not just fee advice</t>
   </si>
   <si>
     <t>Employer number, accident insurance and VBG registrations</t>
   </si>
   <si>
-    <t>https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service | https://www.dguv.de/de/versicherung/mitgliedschaft/index.jsp | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>Public registration routes plus StBVV time-fee support benchmark</t>
-  </si>
-  <si>
-    <t>Apply for employer number, accident insurance number and VBG-style registration where required</t>
+    <t>Employer-number and statutory employer registration support, accident-insurance/VBG routing, and recurring records handover into payroll</t>
+  </si>
+  <si>
+    <t>Handle employer registrations and keep the payroll compliance file current</t>
   </si>
   <si>
     <t>Local business registration (Gewerbeanmeldung)</t>
   </si>
   <si>
-    <t>https://service.berlin.de/dienstleistung/121921/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>Public filing route plus advisor support benchmark; government fees excluded</t>
-  </si>
-  <si>
-    <t>Handle local business registration where required</t>
+    <t>Public fee plus support estimate; Berlin reference shows 31 legal-person filing fee, added to 250/500 support estimate</t>
+  </si>
+  <si>
+    <t>Handle local business registration where required and keep registration evidence in the file</t>
   </si>
   <si>
     <t>Bank account setup</t>
   </si>
   <si>
-    <t>Planning estimate for administrative setup and evidence handling</t>
-  </si>
-  <si>
-    <t>Support bank-account setup and capture records for accounting</t>
+    <t>Administrative setup estimate for bank account opening, access, evidence, mandate and accounting workflow; bank fees not included</t>
+  </si>
+  <si>
+    <t>Support bank-account setup and capture records for accounting and payments</t>
   </si>
   <si>
     <t>Service agreement contracts with client customers</t>
   </si>
   <si>
-    <t>Per-contract planning estimate</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/beratung-anwalt/ | https://www.firma.de/satzung/</t>
-  </si>
-  <si>
-    <t>Legal consultation and company-document benchmark</t>
-  </si>
-  <si>
-    <t>Prepare or review service agreement contracts between the company and its customers</t>
+    <t>Contract preparation/review support estimate for customer service agreements and accounting/legal alignment</t>
+  </si>
+  <si>
+    <t>Prepare or review service agreements between the company and its customers</t>
   </si>
   <si>
     <t>Employment contract changes</t>
   </si>
   <si>
-    <t>Per-change planning estimate</t>
-  </si>
-  <si>
-    <t>https://www.firma.de/beratung-anwalt/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>Legal consultation plus payroll/tax support benchmark</t>
-  </si>
-  <si>
-    <t>Change employment/director contracts and align payroll/accounting treatment</t>
+    <t>Employment/director contract change support plus payroll/accounting alignment and recurring payroll handover</t>
+  </si>
+  <si>
+    <t>Change employment or director contracts and align payroll/accounting treatment</t>
   </si>
   <si>
     <t>Share subscription agreements</t>
   </si>
   <si>
-    <t>Per-document planning estimate</t>
+    <t>Share subscription agreement support estimate, including legal document review and company-record alignment</t>
   </si>
   <si>
     <t>Prepare share subscription agreements where the structure needs them</t>
@@ -1005,37 +924,25 @@
     <t>RBO / beneficial-owner filing where applicable</t>
   </si>
   <si>
-    <t>One-off or annual planning estimate</t>
-  </si>
-  <si>
-    <t>https://rbo.gov.ie/ | https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html</t>
-  </si>
-  <si>
-    <t>Official RBO filing route plus administrative support benchmark</t>
-  </si>
-  <si>
-    <t>Handle beneficial-owner filing where an IE structure requires it</t>
+    <t>Beneficial-owner filing and annual/trigger-event monitoring support; checked in all options for IE company structures</t>
+  </si>
+  <si>
+    <t>All IE company structures need beneficial-owner filing work, so this is included across plans</t>
   </si>
   <si>
     <t>Personal tax bookkeeping and filing add-on</t>
   </si>
   <si>
-    <t>Annual add-on estimate</t>
-  </si>
-  <si>
-    <t>StBVV personal tax filing and income calculation basis</t>
-  </si>
-  <si>
-    <t>Optional personal tax bookkeeping and personal filing support outside the core option fee</t>
+    <t>Optional annual personal tax bookkeeping and filing estimate; separate from company operating entity services</t>
+  </si>
+  <si>
+    <t>Optional personal tax support outside the core company option fee</t>
   </si>
   <si>
     <t>Parental leave planning</t>
   </si>
   <si>
-    <t>One-off add-on estimate</t>
-  </si>
-  <si>
-    <t>Planning estimate for advisory and calculation support</t>
+    <t>Optional planning estimate for parental leave, owner salary timing, payroll impact and benefit timing</t>
   </si>
   <si>
     <t>Optional planning for parental leave and owner salary timing</t>
@@ -1044,19 +951,19 @@
     <t>Client forecast and life-change planning</t>
   </si>
   <si>
-    <t>Tax/advisory benchmark for annual planning and life-change scenarios</t>
-  </si>
-  <si>
-    <t>Refresh client forecast for the new year and after material life/business changes</t>
+    <t>Recurring annual or event-driven forecast updates after life/business changes; support estimate based on tax/accounting advisory time</t>
+  </si>
+  <si>
+    <t>Refresh the client forecast for the new year and after material life or business changes</t>
   </si>
   <si>
     <t>Client calls, inbounds and periodic updates</t>
   </si>
   <si>
-    <t>StBVV time-fee benchmark for ongoing client support</t>
-  </si>
-  <si>
-    <t>Handle client calls, inbound messages, meeting notes and monthly/quarterly updates</t>
+    <t>Recurring client calls, inbound messages, meeting notes, monthly or quarterly updates, and task ownership</t>
+  </si>
+  <si>
+    <t>Handle client calls, inbound messages, meeting notes and periodic updates</t>
   </si>
 </sst>
 </file>
@@ -1071,7 +978,7 @@
     <numFmt numFmtId="168" formatCode="0.0%;[Red](0.0%);-"/>
     <numFmt numFmtId="169" formatCode="€#,##0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="21">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -1143,27 +1050,53 @@
     </font>
     <font>
       <b/>
+      <sz val="14.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
       <color theme="1"/>
-      <name val="Carlito"/>
-      <scheme val="minor"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF1E1E1E"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <i/>
       <sz val="9.0"/>
-      <color rgb="FF4A4A4A"/>
-      <name val="Carlito"/>
-      <scheme val="minor"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <u/>
-      <color rgb="FF0000FF"/>
+      <sz val="10.0"/>
+      <color rgb="FF1E1E1E"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <u/>
-      <color rgb="FF0000FF"/>
+      <sz val="10.0"/>
+      <color rgb="FF1E1E1E"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10.0"/>
+      <color rgb="FF1E1E1E"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1216,24 +1149,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF15312C"/>
-        <bgColor rgb="FF15312C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6EEE7"/>
-        <bgColor rgb="FFE6EEE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1F1F1"/>
-        <bgColor rgb="FFF1F1F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -1554,7 +1469,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="136">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1824,65 +1739,98 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="4" numFmtId="165" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="14" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="14" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="17" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="18" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="19" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="20" fillId="4" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="21" fillId="4" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="21" fillId="4" fontId="17" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="22" fillId="4" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="20" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="12" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="21" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="21" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="21" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="21" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="21" fillId="8" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="22" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="23" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="17" fillId="10" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="18" fillId="10" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="19" fillId="10" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="20" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="24" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="24" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="24" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="24" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="24" fillId="8" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="25" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="21" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="21" fillId="0" fontId="11" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="21" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="22" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="21" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="23" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="24" fillId="0" fontId="11" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="24" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="25" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="0" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2113,7 +2061,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="90.0"/>
+    <col customWidth="1" min="1" max="1" width="52.63"/>
     <col customWidth="1" min="2" max="2" width="13.63"/>
     <col customWidth="1" min="3" max="3" width="30.75"/>
     <col customWidth="1" min="4" max="4" width="38.38"/>
@@ -7370,27 +7318,18 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="31.38"/>
+    <col customWidth="1" min="1" max="1" width="33.88"/>
     <col customWidth="1" min="2" max="5" width="15.13"/>
-    <col customWidth="1" min="6" max="6" width="17.0"/>
-    <col customWidth="1" min="7" max="7" width="18.88"/>
-    <col customWidth="1" min="8" max="8" width="37.63"/>
-    <col customWidth="1" min="9" max="10" width="35.13"/>
+    <col customWidth="1" min="6" max="7" width="15.75"/>
+    <col customWidth="1" min="8" max="8" width="30.75"/>
+    <col customWidth="1" min="9" max="9" width="45.13"/>
+    <col customWidth="1" min="10" max="10" width="57.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.0" customHeight="1">
       <c r="A1" s="105" t="s">
         <v>209</v>
       </c>
-      <c r="B1" s="105"/>
-      <c r="C1" s="105"/>
-      <c r="D1" s="105"/>
-      <c r="E1" s="105"/>
-      <c r="F1" s="105"/>
-      <c r="G1" s="105"/>
-      <c r="H1" s="105"/>
-      <c r="I1" s="105"/>
-      <c r="J1" s="105"/>
     </row>
     <row r="2">
       <c r="A2" s="106" t="s">
@@ -7423,20 +7362,20 @@
         <v>211</v>
       </c>
       <c r="B3" s="107">
-        <f t="shared" ref="B3:E3" si="1">SUMIF(B7:B38,TRUE,$F$7:$F$38)</f>
-        <v>1724</v>
+        <f t="shared" ref="B3:E3" si="1">SUMIF(B8:B39,TRUE,$F$8:$F$39)</f>
+        <v>9511</v>
       </c>
       <c r="C3" s="107">
         <f t="shared" si="1"/>
-        <v>16881</v>
+        <v>17016</v>
       </c>
       <c r="D3" s="107">
         <f t="shared" si="1"/>
-        <v>17381</v>
+        <v>17516</v>
       </c>
       <c r="E3" s="107">
         <f t="shared" si="1"/>
-        <v>18131</v>
+        <v>21016</v>
       </c>
       <c r="F3" s="108"/>
       <c r="G3" s="108"/>
@@ -7445,1099 +7384,1142 @@
       <c r="J3" s="108"/>
     </row>
     <row r="4">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="106" t="s">
         <v>212</v>
       </c>
-      <c r="B4" s="109"/>
-      <c r="C4" s="109"/>
-      <c r="D4" s="109"/>
-      <c r="E4" s="109"/>
-      <c r="F4" s="109"/>
-      <c r="G4" s="109"/>
-      <c r="H4" s="109"/>
-      <c r="I4" s="109"/>
-      <c r="J4" s="109"/>
+      <c r="B4" s="109">
+        <f t="shared" ref="B4:E4" si="2">SUMIF(B8:B39,TRUE,$G$8:$G$39)</f>
+        <v>17005</v>
+      </c>
+      <c r="C4" s="109">
+        <f t="shared" si="2"/>
+        <v>31968</v>
+      </c>
+      <c r="D4" s="109">
+        <f t="shared" si="2"/>
+        <v>32968</v>
+      </c>
+      <c r="E4" s="109">
+        <f t="shared" si="2"/>
+        <v>39968</v>
+      </c>
+      <c r="F4" s="110"/>
+      <c r="G4" s="110"/>
+      <c r="H4" s="110"/>
+      <c r="I4" s="110"/>
+      <c r="J4" s="110"/>
     </row>
     <row r="5">
-      <c r="A5" s="108"/>
-      <c r="B5" s="108"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108"/>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108"/>
-      <c r="I5" s="108"/>
-      <c r="J5" s="108"/>
+      <c r="A5" s="111" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="6" ht="42.0" customHeight="1">
-      <c r="A6" s="110" t="s">
-        <v>213</v>
-      </c>
-      <c r="B6" s="111" t="s">
+      <c r="A6" s="112"/>
+      <c r="B6" s="113"/>
+      <c r="C6" s="113"/>
+      <c r="D6" s="113"/>
+      <c r="E6" s="113"/>
+      <c r="F6" s="113"/>
+      <c r="G6" s="113"/>
+      <c r="H6" s="113"/>
+      <c r="I6" s="113"/>
+      <c r="J6" s="114"/>
+    </row>
+    <row r="7" ht="37.5" customHeight="1">
+      <c r="A7" s="115" t="s">
+        <v>214</v>
+      </c>
+      <c r="B7" s="116" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="111" t="s">
+      <c r="C7" s="116" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="111" t="s">
+      <c r="D7" s="116" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="111" t="s">
+      <c r="E7" s="116" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="111" t="s">
-        <v>214</v>
-      </c>
-      <c r="G6" s="111" t="s">
+      <c r="F7" s="117" t="s">
         <v>215</v>
       </c>
-      <c r="H6" s="111" t="s">
+      <c r="G7" s="116" t="s">
         <v>216</v>
       </c>
-      <c r="I6" s="111" t="s">
+      <c r="H7" s="116" t="s">
         <v>217</v>
       </c>
-      <c r="J6" s="112" t="s">
+      <c r="I7" s="116" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="7" ht="52.5" customHeight="1">
-      <c r="A7" s="113" t="s">
+      <c r="J7" s="118" t="s">
         <v>219</v>
       </c>
-      <c r="B7" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E7" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F7" s="115">
+    </row>
+    <row r="8" ht="31.5" customHeight="1">
+      <c r="A8" s="119" t="s">
+        <v>220</v>
+      </c>
+      <c r="B8" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="121">
         <v>824.0</v>
       </c>
-      <c r="G7" s="116" t="s">
-        <v>220</v>
-      </c>
-      <c r="H7" s="116" t="s">
+      <c r="G8" s="122">
+        <v>1223.0</v>
+      </c>
+      <c r="H8" s="123" t="s">
         <v>221</v>
       </c>
-      <c r="I7" s="116" t="s">
+      <c r="I8" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","firma.de tax-advice benchmark plus professional-support estimate")</f>
+        <v>firma.de tax-advice benchmark plus professional-support estimate</v>
+      </c>
+      <c r="J8" s="125" t="s">
         <v>222</v>
       </c>
-      <c r="J7" s="117" t="s">
+    </row>
+    <row r="9" ht="31.5" customHeight="1">
+      <c r="A9" s="119" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="8" ht="52.5" customHeight="1">
-      <c r="A8" s="113" t="s">
+      <c r="B9" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="121">
+        <v>900.0</v>
+      </c>
+      <c r="G9" s="122">
+        <v>1500.0</v>
+      </c>
+      <c r="H9" s="123" t="s">
         <v>224</v>
       </c>
-      <c r="B8" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E8" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" s="115">
+      <c r="I9" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/satzung/","firma.de company-document benchmark plus incorporation support estimate")</f>
+        <v>firma.de company-document benchmark plus incorporation support estimate</v>
+      </c>
+      <c r="J9" s="125" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="10" ht="31.5" customHeight="1">
+      <c r="A10" s="119" t="s">
+        <v>226</v>
+      </c>
+      <c r="B10" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="121">
+        <v>300.0</v>
+      </c>
+      <c r="G10" s="122">
+        <v>600.0</v>
+      </c>
+      <c r="H10" s="123" t="s">
+        <v>227</v>
+      </c>
+      <c r="I10" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for document intake and admin support")</f>
+        <v>StBVV-style time-fee benchmark for document intake and admin support</v>
+      </c>
+      <c r="J10" s="125" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="11" ht="31.5" customHeight="1">
+      <c r="A11" s="119" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="121">
+        <v>1368.0</v>
+      </c>
+      <c r="G11" s="122">
+        <v>2208.0</v>
+      </c>
+      <c r="H11" s="123" t="s">
+        <v>230</v>
+      </c>
+      <c r="I11" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/buchhaltung/","firma.de bookkeeping package prices including DATEV software add-on")</f>
+        <v>firma.de bookkeeping package prices including DATEV software add-on</v>
+      </c>
+      <c r="J11" s="125" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="12" ht="31.5" customHeight="1">
+      <c r="A12" s="119" t="s">
+        <v>232</v>
+      </c>
+      <c r="B12" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="121">
+        <v>300.0</v>
+      </c>
+      <c r="G12" s="122">
+        <v>600.0</v>
+      </c>
+      <c r="H12" s="123" t="s">
+        <v>233</v>
+      </c>
+      <c r="I12" s="124" t="str">
+        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware Office software prices used where a tool cost is needed")</f>
+        <v>Lexware Office software prices used where a tool cost is needed</v>
+      </c>
+      <c r="J12" s="125" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="13" ht="31.5" customHeight="1">
+      <c r="A13" s="119" t="s">
+        <v>235</v>
+      </c>
+      <c r="B13" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="121">
+        <v>600.0</v>
+      </c>
+      <c r="G13" s="122">
+        <v>1200.0</v>
+      </c>
+      <c r="H13" s="123" t="s">
+        <v>236</v>
+      </c>
+      <c r="I13" s="124" t="str">
+        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware VAT filing and software-pricing reference for tool costs")</f>
+        <v>Lexware VAT filing and software-pricing reference for tool costs</v>
+      </c>
+      <c r="J13" s="125" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="14" ht="31.5" customHeight="1">
+      <c r="A14" s="119" t="s">
+        <v>238</v>
+      </c>
+      <c r="B14" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E14" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="121">
+        <v>1348.0</v>
+      </c>
+      <c r="G14" s="122">
+        <v>2048.0</v>
+      </c>
+      <c r="H14" s="123" t="s">
+        <v>239</v>
+      </c>
+      <c r="I14" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/jahresabschluss-kapitalgesellschaft/","firma.de annual accounts prices plus disclosure filing add-on")</f>
+        <v>firma.de annual accounts prices plus disclosure filing add-on</v>
+      </c>
+      <c r="J14" s="125" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" ht="31.5" customHeight="1">
+      <c r="A15" s="119" t="s">
+        <v>241</v>
+      </c>
+      <c r="B15" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="121">
+        <v>240.0</v>
+      </c>
+      <c r="G15" s="122">
+        <v>395.0</v>
+      </c>
+      <c r="H15" s="123" t="s">
+        <v>242</v>
+      </c>
+      <c r="I15" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/lohnabrechnung/","firma.de payroll benchmark; mid estimate also includes payroll tool cost")</f>
+        <v>firma.de payroll benchmark; mid estimate also includes payroll tool cost</v>
+      </c>
+      <c r="J15" s="125" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="16" ht="31.5" customHeight="1">
+      <c r="A16" s="119" t="s">
+        <v>244</v>
+      </c>
+      <c r="B16" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" s="121">
+        <v>500.0</v>
+      </c>
+      <c r="G16" s="122">
+        <v>1000.0</v>
+      </c>
+      <c r="H16" s="123" t="s">
+        <v>245</v>
+      </c>
+      <c r="I16" s="124" t="str">
+        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware payroll filing/tool reference plus setup-support estimate")</f>
+        <v>Lexware payroll filing/tool reference plus setup-support estimate</v>
+      </c>
+      <c r="J16" s="125" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="17" ht="31.5" customHeight="1">
+      <c r="A17" s="119" t="s">
+        <v>247</v>
+      </c>
+      <c r="B17" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D17" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="121">
+        <v>1200.0</v>
+      </c>
+      <c r="G17" s="122">
+        <v>2400.0</v>
+      </c>
+      <c r="H17" s="123" t="s">
+        <v>248</v>
+      </c>
+      <c r="I17" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for rent analysis, contract and recurring payment work")</f>
+        <v>Professional time-fee benchmark for rent analysis, contract and recurring payment work</v>
+      </c>
+      <c r="J17" s="125" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" ht="31.5" customHeight="1">
+      <c r="A18" s="119" t="s">
+        <v>250</v>
+      </c>
+      <c r="B18" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C18" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D18" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" s="121">
         <v>900.0</v>
       </c>
-      <c r="G8" s="116" t="s">
-        <v>225</v>
-      </c>
-      <c r="H8" s="116" t="s">
-        <v>226</v>
-      </c>
-      <c r="I8" s="116" t="s">
-        <v>227</v>
-      </c>
-      <c r="J8" s="117" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="9" ht="52.5" customHeight="1">
-      <c r="A9" s="113" t="s">
-        <v>229</v>
-      </c>
-      <c r="B9" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C9" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" s="115">
+      <c r="G18" s="122">
+        <v>1800.0</v>
+      </c>
+      <c r="H18" s="123" t="s">
+        <v>251</v>
+      </c>
+      <c r="I18" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for recurring expense and travel-support work")</f>
+        <v>Professional time-fee benchmark for recurring expense and travel-support work</v>
+      </c>
+      <c r="J18" s="125" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="19" ht="31.5" customHeight="1">
+      <c r="A19" s="119" t="s">
+        <v>253</v>
+      </c>
+      <c r="B19" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D19" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="121">
+        <v>1355.0</v>
+      </c>
+      <c r="G19" s="122">
+        <v>2663.0</v>
+      </c>
+      <c r="H19" s="123" t="s">
+        <v>254</v>
+      </c>
+      <c r="I19" s="124" t="str">
+        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware invoicing, banking, payment and bookkeeping tool-cost reference")</f>
+        <v>Lexware invoicing, banking, payment and bookkeeping tool-cost reference</v>
+      </c>
+      <c r="J19" s="125" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="20" ht="31.5" customHeight="1">
+      <c r="A20" s="119" t="s">
+        <v>256</v>
+      </c>
+      <c r="B20" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C20" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D20" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" s="121">
+        <v>600.0</v>
+      </c>
+      <c r="G20" s="122">
+        <v>1200.0</v>
+      </c>
+      <c r="H20" s="123" t="s">
+        <v>257</v>
+      </c>
+      <c r="I20" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style recurring support benchmark for tax-payment tracking")</f>
+        <v>StBVV-style recurring support benchmark for tax-payment tracking</v>
+      </c>
+      <c r="J20" s="125" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="21" ht="31.5" customHeight="1">
+      <c r="A21" s="119" t="s">
+        <v>259</v>
+      </c>
+      <c r="B21" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C21" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D21" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" s="121">
+        <v>900.0</v>
+      </c>
+      <c r="G21" s="122">
+        <v>1800.0</v>
+      </c>
+      <c r="H21" s="123" t="s">
+        <v>260</v>
+      </c>
+      <c r="I21" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for correspondence support and authority letters")</f>
+        <v>Tax-advice benchmark for correspondence support and authority letters</v>
+      </c>
+      <c r="J21" s="125" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="22" ht="31.5" customHeight="1">
+      <c r="A22" s="119" t="s">
+        <v>262</v>
+      </c>
+      <c r="B22" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C22" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" s="121">
+        <v>750.0</v>
+      </c>
+      <c r="G22" s="122">
+        <v>1500.0</v>
+      </c>
+      <c r="H22" s="123" t="s">
+        <v>263</v>
+      </c>
+      <c r="I22" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for authority correspondence and case work")</f>
+        <v>Professional time-fee benchmark for authority correspondence and case work</v>
+      </c>
+      <c r="J22" s="125" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="23" ht="31.5" customHeight="1">
+      <c r="A23" s="119" t="s">
+        <v>265</v>
+      </c>
+      <c r="B23" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C23" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" s="121">
+        <v>350.0</v>
+      </c>
+      <c r="G23" s="122">
+        <v>700.0</v>
+      </c>
+      <c r="H23" s="123" t="s">
+        <v>266</v>
+      </c>
+      <c r="I23" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for depreciation and tax-planning analysis")</f>
+        <v>Professional benchmark for depreciation and tax-planning analysis</v>
+      </c>
+      <c r="J23" s="125" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="24" ht="31.5" customHeight="1">
+      <c r="A24" s="119" t="s">
+        <v>268</v>
+      </c>
+      <c r="B24" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" s="121">
+        <v>350.0</v>
+      </c>
+      <c r="G24" s="122">
+        <v>700.0</v>
+      </c>
+      <c r="H24" s="123" t="s">
+        <v>269</v>
+      </c>
+      <c r="I24" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for retained-profit and investment planning")</f>
+        <v>Tax-advice benchmark for retained-profit and investment planning</v>
+      </c>
+      <c r="J24" s="125" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="25" ht="31.5" customHeight="1">
+      <c r="A25" s="119" t="s">
+        <v>271</v>
+      </c>
+      <c r="B25" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C25" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D25" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" s="121">
+        <v>250.0</v>
+      </c>
+      <c r="G25" s="122">
+        <v>500.0</v>
+      </c>
+      <c r="H25" s="123" t="s">
+        <v>272</v>
+      </c>
+      <c r="I25" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for setup and evidence handling")</f>
+        <v>Professional support benchmark for setup and evidence handling</v>
+      </c>
+      <c r="J25" s="125" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="26" ht="31.5" customHeight="1">
+      <c r="A26" s="119" t="s">
+        <v>274</v>
+      </c>
+      <c r="B26" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C26" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" s="121">
+        <v>500.0</v>
+      </c>
+      <c r="G26" s="122">
+        <v>1000.0</v>
+      </c>
+      <c r="H26" s="123" t="s">
+        <v>275</v>
+      </c>
+      <c r="I26" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for pension reserve planning support")</f>
+        <v>Tax-advice benchmark for pension reserve planning support</v>
+      </c>
+      <c r="J26" s="125" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="27" ht="31.5" customHeight="1">
+      <c r="A27" s="119" t="s">
+        <v>277</v>
+      </c>
+      <c r="B27" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C27" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="D27" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F27" s="121">
+        <v>1000.0</v>
+      </c>
+      <c r="G27" s="122">
+        <v>2000.0</v>
+      </c>
+      <c r="H27" s="123" t="s">
+        <v>278</v>
+      </c>
+      <c r="I27" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for complex cross-border tax and accounting work")</f>
+        <v>Professional benchmark for complex cross-border tax and accounting work</v>
+      </c>
+      <c r="J27" s="125" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="28" ht="31.5" customHeight="1">
+      <c r="A28" s="119" t="s">
+        <v>280</v>
+      </c>
+      <c r="B28" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C28" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E28" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" s="121">
+        <v>3000.0</v>
+      </c>
+      <c r="G28" s="122">
+        <v>6000.0</v>
+      </c>
+      <c r="H28" s="123" t="s">
+        <v>281</v>
+      </c>
+      <c r="I28" s="124" t="str">
+        <f>HYPERLINK("https://www.irishstatutebook.ie/eli/2014/act/38/section/137/enacted/en/html","Irish Companies Act director-residence reference plus annual director-service estimate")</f>
+        <v>Irish Companies Act director-residence reference plus annual director-service estimate</v>
+      </c>
+      <c r="J28" s="125" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="29" ht="31.5" customHeight="1">
+      <c r="A29" s="119" t="s">
+        <v>283</v>
+      </c>
+      <c r="B29" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C29" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E29" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F29" s="121">
         <v>300.0</v>
       </c>
-      <c r="G9" s="116" t="s">
-        <v>225</v>
-      </c>
-      <c r="H9" s="118" t="s">
-        <v>230</v>
-      </c>
-      <c r="I9" s="116" t="s">
-        <v>231</v>
-      </c>
-      <c r="J9" s="117" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="10" ht="52.5" customHeight="1">
-      <c r="A10" s="113" t="s">
-        <v>233</v>
-      </c>
-      <c r="B10" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C10" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" s="115">
-        <v>2028.0</v>
-      </c>
-      <c r="G10" s="116" t="s">
-        <v>234</v>
-      </c>
-      <c r="H10" s="116" t="s">
-        <v>235</v>
-      </c>
-      <c r="I10" s="116" t="s">
-        <v>236</v>
-      </c>
-      <c r="J10" s="117" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="11" ht="52.5" customHeight="1">
-      <c r="A11" s="113" t="s">
-        <v>238</v>
-      </c>
-      <c r="B11" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C11" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E11" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" s="115">
+      <c r="G29" s="122">
+        <v>600.0</v>
+      </c>
+      <c r="H29" s="123" t="s">
+        <v>284</v>
+      </c>
+      <c r="I29" s="124" t="str">
+        <f>HYPERLINK("https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service","Bundesagentur employer-number service plus employer registration support estimate")</f>
+        <v>Bundesagentur employer-number service plus employer registration support estimate</v>
+      </c>
+      <c r="J29" s="125" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="30" ht="31.5" customHeight="1">
+      <c r="A30" s="119" t="s">
+        <v>286</v>
+      </c>
+      <c r="B30" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C30" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D30" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E30" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F30" s="121">
+        <v>281.0</v>
+      </c>
+      <c r="G30" s="122">
+        <v>531.0</v>
+      </c>
+      <c r="H30" s="123" t="s">
+        <v>287</v>
+      </c>
+      <c r="I30" s="124" t="str">
+        <f>HYPERLINK("https://service.berlin.de/dienstleistung/121921/","Berlin Gewerbeanmeldung fee reference plus registration support estimate")</f>
+        <v>Berlin Gewerbeanmeldung fee reference plus registration support estimate</v>
+      </c>
+      <c r="J30" s="125" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="31" ht="31.5" customHeight="1">
+      <c r="A31" s="119" t="s">
+        <v>289</v>
+      </c>
+      <c r="B31" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C31" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D31" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E31" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F31" s="121">
+        <v>250.0</v>
+      </c>
+      <c r="G31" s="122">
+        <v>500.0</v>
+      </c>
+      <c r="H31" s="123" t="s">
+        <v>290</v>
+      </c>
+      <c r="I31" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for bank-account setup and records")</f>
+        <v>Professional support benchmark for bank-account setup and records</v>
+      </c>
+      <c r="J31" s="125" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="32" ht="31.5" customHeight="1">
+      <c r="A32" s="119" t="s">
+        <v>292</v>
+      </c>
+      <c r="B32" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C32" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D32" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E32" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" s="121">
+        <v>600.0</v>
+      </c>
+      <c r="G32" s="122">
+        <v>1200.0</v>
+      </c>
+      <c r="H32" s="123" t="s">
+        <v>293</v>
+      </c>
+      <c r="I32" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for service agreement support")</f>
+        <v>Legal-consultation benchmark for service agreement support</v>
+      </c>
+      <c r="J32" s="125" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="33" ht="31.5" customHeight="1">
+      <c r="A33" s="119" t="s">
+        <v>295</v>
+      </c>
+      <c r="B33" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C33" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D33" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E33" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F33" s="121">
+        <v>500.0</v>
+      </c>
+      <c r="G33" s="122">
+        <v>1000.0</v>
+      </c>
+      <c r="H33" s="123" t="s">
+        <v>296</v>
+      </c>
+      <c r="I33" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for employment contract change support")</f>
+        <v>Legal-consultation benchmark for employment contract change support</v>
+      </c>
+      <c r="J33" s="125" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="34" ht="31.5" customHeight="1">
+      <c r="A34" s="119" t="s">
+        <v>298</v>
+      </c>
+      <c r="B34" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C34" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D34" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F34" s="121">
+        <v>650.0</v>
+      </c>
+      <c r="G34" s="122">
+        <v>1300.0</v>
+      </c>
+      <c r="H34" s="123" t="s">
+        <v>299</v>
+      </c>
+      <c r="I34" s="124" t="str">
+        <f>HYPERLINK("https://www.firma.de/satzung/","Company-document benchmark for shareholder/subscription document support")</f>
+        <v>Company-document benchmark for shareholder/subscription document support</v>
+      </c>
+      <c r="J34" s="125" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="35" ht="31.5" customHeight="1">
+      <c r="A35" s="119" t="s">
+        <v>301</v>
+      </c>
+      <c r="B35" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="C35" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="D35" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" s="120" t="b">
+        <v>1</v>
+      </c>
+      <c r="F35" s="121">
         <v>300.0</v>
       </c>
-      <c r="G11" s="116" t="s">
-        <v>225</v>
-      </c>
-      <c r="H11" s="116" t="s">
-        <v>235</v>
-      </c>
-      <c r="I11" s="116" t="s">
-        <v>239</v>
-      </c>
-      <c r="J11" s="117" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="12" ht="52.5" customHeight="1">
-      <c r="A12" s="113" t="s">
-        <v>241</v>
-      </c>
-      <c r="B12" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C12" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E12" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" s="115">
-        <v>540.0</v>
-      </c>
-      <c r="G12" s="116" t="s">
-        <v>242</v>
-      </c>
-      <c r="H12" s="118" t="s">
-        <v>230</v>
-      </c>
-      <c r="I12" s="116" t="s">
-        <v>243</v>
-      </c>
-      <c r="J12" s="117" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="13" ht="52.5" customHeight="1">
-      <c r="A13" s="113" t="s">
-        <v>245</v>
-      </c>
-      <c r="B13" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C13" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E13" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" s="115">
-        <v>1949.0</v>
-      </c>
-      <c r="G13" s="116" t="s">
-        <v>246</v>
-      </c>
-      <c r="H13" s="116" t="s">
-        <v>247</v>
-      </c>
-      <c r="I13" s="116" t="s">
-        <v>248</v>
-      </c>
-      <c r="J13" s="117" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="14" ht="52.5" customHeight="1">
-      <c r="A14" s="113" t="s">
-        <v>250</v>
-      </c>
-      <c r="B14" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C14" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E14" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" s="115">
-        <v>240.0</v>
-      </c>
-      <c r="G14" s="116" t="s">
-        <v>251</v>
-      </c>
-      <c r="H14" s="116" t="s">
-        <v>252</v>
-      </c>
-      <c r="I14" s="116" t="s">
-        <v>253</v>
-      </c>
-      <c r="J14" s="117" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="15" ht="52.5" customHeight="1">
-      <c r="A15" s="113" t="s">
-        <v>255</v>
-      </c>
-      <c r="B15" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C15" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="115">
+      <c r="G35" s="122">
+        <v>600.0</v>
+      </c>
+      <c r="H35" s="123" t="s">
+        <v>302</v>
+      </c>
+      <c r="I35" s="124" t="str">
+        <f>HYPERLINK("https://rbo.gov.ie/","RBO Ireland official filing route for relevant Irish incorporated entities")</f>
+        <v>RBO Ireland official filing route for relevant Irish incorporated entities</v>
+      </c>
+      <c r="J35" s="125" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="36" ht="31.5" customHeight="1">
+      <c r="A36" s="119" t="s">
+        <v>304</v>
+      </c>
+      <c r="B36" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C36" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="D36" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36" s="121">
+        <v>750.0</v>
+      </c>
+      <c r="G36" s="122">
+        <v>1500.0</v>
+      </c>
+      <c r="H36" s="123" t="s">
+        <v>305</v>
+      </c>
+      <c r="I36" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV personal tax filing and income-calculation benchmark")</f>
+        <v>StBVV personal tax filing and income-calculation benchmark</v>
+      </c>
+      <c r="J36" s="125" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="37" ht="31.5" customHeight="1">
+      <c r="A37" s="119" t="s">
+        <v>307</v>
+      </c>
+      <c r="B37" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="C37" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="D37" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E37" s="120" t="b">
+        <v>0</v>
+      </c>
+      <c r="F37" s="121">
+        <v>450.0</v>
+      </c>
+      <c r="G37" s="122">
+        <v>900.0</v>
+      </c>
+      <c r="H37" s="123" t="s">
+        <v>308</v>
+      </c>
+      <c r="I37" s="124" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for parental leave and salary-timing planning")</f>
+        <v>Professional support benchmark for parental leave and salary-timing planning</v>
+      </c>
+      <c r="J37" s="125" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="38" ht="31.5" customHeight="1">
+      <c r="A38" s="126" t="s">
+        <v>310</v>
+      </c>
+      <c r="B38" s="127" t="b">
+        <v>0</v>
+      </c>
+      <c r="C38" s="127" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" s="127" t="b">
+        <v>1</v>
+      </c>
+      <c r="E38" s="127" t="b">
+        <v>1</v>
+      </c>
+      <c r="F38" s="128">
         <v>500.0</v>
       </c>
-      <c r="G15" s="116" t="s">
-        <v>256</v>
-      </c>
-      <c r="H15" s="116" t="s">
-        <v>252</v>
-      </c>
-      <c r="I15" s="116" t="s">
-        <v>257</v>
-      </c>
-      <c r="J15" s="117" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="16" ht="52.5" customHeight="1">
-      <c r="A16" s="113" t="s">
-        <v>259</v>
-      </c>
-      <c r="B16" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D16" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E16" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" s="115">
+      <c r="G38" s="129">
+        <v>1000.0</v>
+      </c>
+      <c r="H38" s="130" t="s">
+        <v>311</v>
+      </c>
+      <c r="I38" s="131" t="str">
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for forecast and life-change planning support")</f>
+        <v>Tax-advice benchmark for forecast and life-change planning support</v>
+      </c>
+      <c r="J38" s="132" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="39" ht="31.5" customHeight="1">
+      <c r="A39" s="133" t="s">
+        <v>313</v>
+      </c>
+      <c r="B39" s="110" t="b">
+        <v>0</v>
+      </c>
+      <c r="C39" s="110" t="b">
+        <v>1</v>
+      </c>
+      <c r="D39" s="110" t="b">
+        <v>1</v>
+      </c>
+      <c r="E39" s="110" t="b">
+        <v>1</v>
+      </c>
+      <c r="F39" s="134">
+        <v>600.0</v>
+      </c>
+      <c r="G39" s="134">
         <v>1200.0</v>
       </c>
-      <c r="G16" s="116" t="s">
-        <v>260</v>
-      </c>
-      <c r="H16" s="116" t="s">
-        <v>261</v>
-      </c>
-      <c r="I16" s="116" t="s">
-        <v>262</v>
-      </c>
-      <c r="J16" s="117" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="17" ht="52.5" customHeight="1">
-      <c r="A17" s="113" t="s">
-        <v>264</v>
-      </c>
-      <c r="B17" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D17" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="115">
-        <v>900.0</v>
-      </c>
-      <c r="G17" s="116" t="s">
-        <v>265</v>
-      </c>
-      <c r="H17" s="116" t="s">
-        <v>266</v>
-      </c>
-      <c r="I17" s="116" t="s">
-        <v>267</v>
-      </c>
-      <c r="J17" s="117" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="18" ht="52.5" customHeight="1">
-      <c r="A18" s="113" t="s">
-        <v>269</v>
-      </c>
-      <c r="B18" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C18" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D18" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E18" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" s="115">
-        <v>1200.0</v>
-      </c>
-      <c r="G18" s="116" t="s">
-        <v>270</v>
-      </c>
-      <c r="H18" s="116" t="s">
-        <v>235</v>
-      </c>
-      <c r="I18" s="116" t="s">
-        <v>271</v>
-      </c>
-      <c r="J18" s="117" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="19" ht="52.5" customHeight="1">
-      <c r="A19" s="113" t="s">
-        <v>273</v>
-      </c>
-      <c r="B19" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C19" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D19" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E19" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F19" s="115">
-        <v>300.0</v>
-      </c>
-      <c r="G19" s="116" t="s">
-        <v>242</v>
-      </c>
-      <c r="H19" s="118" t="s">
-        <v>230</v>
-      </c>
-      <c r="I19" s="116" t="s">
-        <v>274</v>
-      </c>
-      <c r="J19" s="117" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="20" ht="52.5" customHeight="1">
-      <c r="A20" s="113" t="s">
-        <v>276</v>
-      </c>
-      <c r="B20" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C20" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D20" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E20" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F20" s="115">
-        <v>350.0</v>
-      </c>
-      <c r="G20" s="116" t="s">
-        <v>256</v>
-      </c>
-      <c r="H20" s="116" t="s">
-        <v>277</v>
-      </c>
-      <c r="I20" s="116" t="s">
-        <v>278</v>
-      </c>
-      <c r="J20" s="117" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="21" ht="52.5" customHeight="1">
-      <c r="A21" s="113" t="s">
-        <v>280</v>
-      </c>
-      <c r="B21" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C21" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D21" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E21" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" s="115">
-        <v>750.0</v>
-      </c>
-      <c r="G21" s="116" t="s">
-        <v>281</v>
-      </c>
-      <c r="H21" s="116" t="s">
-        <v>282</v>
-      </c>
-      <c r="I21" s="116" t="s">
-        <v>283</v>
-      </c>
-      <c r="J21" s="117" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="22" ht="52.5" customHeight="1">
-      <c r="A22" s="113" t="s">
-        <v>285</v>
-      </c>
-      <c r="B22" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C22" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D22" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E22" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F22" s="115">
-        <v>350.0</v>
-      </c>
-      <c r="G22" s="116" t="s">
-        <v>286</v>
-      </c>
-      <c r="H22" s="116" t="s">
-        <v>277</v>
-      </c>
-      <c r="I22" s="116" t="s">
-        <v>287</v>
-      </c>
-      <c r="J22" s="117" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="23" ht="52.5" customHeight="1">
-      <c r="A23" s="113" t="s">
-        <v>289</v>
-      </c>
-      <c r="B23" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C23" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D23" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E23" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F23" s="115">
-        <v>350.0</v>
-      </c>
-      <c r="G23" s="116" t="s">
-        <v>286</v>
-      </c>
-      <c r="H23" s="116" t="s">
-        <v>277</v>
-      </c>
-      <c r="I23" s="116" t="s">
-        <v>290</v>
-      </c>
-      <c r="J23" s="117" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="24" ht="52.5" customHeight="1">
-      <c r="A24" s="113" t="s">
-        <v>292</v>
-      </c>
-      <c r="B24" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C24" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D24" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E24" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24" s="115">
-        <v>250.0</v>
-      </c>
-      <c r="G24" s="116" t="s">
-        <v>225</v>
-      </c>
-      <c r="H24" s="118" t="s">
-        <v>230</v>
-      </c>
-      <c r="I24" s="116" t="s">
-        <v>293</v>
-      </c>
-      <c r="J24" s="117" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="25" ht="52.5" customHeight="1">
-      <c r="A25" s="113" t="s">
-        <v>295</v>
-      </c>
-      <c r="B25" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C25" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="D25" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E25" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="F25" s="115">
-        <v>500.0</v>
-      </c>
-      <c r="G25" s="116" t="s">
-        <v>286</v>
-      </c>
-      <c r="H25" s="116" t="s">
-        <v>277</v>
-      </c>
-      <c r="I25" s="116" t="s">
-        <v>290</v>
-      </c>
-      <c r="J25" s="117" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="26" ht="52.5" customHeight="1">
-      <c r="A26" s="113" t="s">
-        <v>297</v>
-      </c>
-      <c r="B26" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F26" s="115">
-        <v>1000.0</v>
-      </c>
-      <c r="G26" s="116" t="s">
-        <v>286</v>
-      </c>
-      <c r="H26" s="116" t="s">
-        <v>277</v>
-      </c>
-      <c r="I26" s="116" t="s">
-        <v>298</v>
-      </c>
-      <c r="J26" s="117" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="27" ht="52.5" customHeight="1">
-      <c r="A27" s="113" t="s">
-        <v>300</v>
-      </c>
-      <c r="B27" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C27" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="D27" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="E27" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F27" s="115">
-        <v>500.0</v>
-      </c>
-      <c r="G27" s="116" t="s">
-        <v>286</v>
-      </c>
-      <c r="H27" s="116" t="s">
-        <v>301</v>
-      </c>
-      <c r="I27" s="116" t="s">
-        <v>302</v>
-      </c>
-      <c r="J27" s="117" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="28" ht="52.5" customHeight="1">
-      <c r="A28" s="113" t="s">
-        <v>304</v>
-      </c>
-      <c r="B28" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C28" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D28" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E28" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="F28" s="115">
-        <v>300.0</v>
-      </c>
-      <c r="G28" s="116" t="s">
-        <v>225</v>
-      </c>
-      <c r="H28" s="116" t="s">
-        <v>305</v>
-      </c>
-      <c r="I28" s="116" t="s">
-        <v>306</v>
-      </c>
-      <c r="J28" s="117" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="29" ht="52.5" customHeight="1">
-      <c r="A29" s="113" t="s">
-        <v>308</v>
-      </c>
-      <c r="B29" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C29" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D29" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E29" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="F29" s="115">
-        <v>250.0</v>
-      </c>
-      <c r="G29" s="116" t="s">
-        <v>225</v>
-      </c>
-      <c r="H29" s="116" t="s">
-        <v>309</v>
-      </c>
-      <c r="I29" s="116" t="s">
-        <v>310</v>
-      </c>
-      <c r="J29" s="117" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="30" ht="52.5" customHeight="1">
-      <c r="A30" s="113" t="s">
-        <v>312</v>
-      </c>
-      <c r="B30" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C30" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D30" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E30" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F30" s="115">
-        <v>250.0</v>
-      </c>
-      <c r="G30" s="116" t="s">
-        <v>225</v>
-      </c>
-      <c r="H30" s="118" t="s">
-        <v>230</v>
-      </c>
-      <c r="I30" s="116" t="s">
-        <v>313</v>
-      </c>
-      <c r="J30" s="117" t="s">
+      <c r="H39" s="110" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="31" ht="52.5" customHeight="1">
-      <c r="A31" s="113" t="s">
+      <c r="I39" s="135" t="str">
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for recurring client support")</f>
+        <v>StBVV-style time-fee benchmark for recurring client support</v>
+      </c>
+      <c r="J39" s="110" t="s">
         <v>315</v>
       </c>
-      <c r="B31" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C31" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D31" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E31" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F31" s="115">
-        <v>600.0</v>
-      </c>
-      <c r="G31" s="116" t="s">
-        <v>316</v>
-      </c>
-      <c r="H31" s="116" t="s">
-        <v>317</v>
-      </c>
-      <c r="I31" s="116" t="s">
-        <v>318</v>
-      </c>
-      <c r="J31" s="117" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="32" ht="52.5" customHeight="1">
-      <c r="A32" s="113" t="s">
-        <v>320</v>
-      </c>
-      <c r="B32" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C32" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D32" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E32" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F32" s="115">
-        <v>500.0</v>
-      </c>
-      <c r="G32" s="116" t="s">
-        <v>321</v>
-      </c>
-      <c r="H32" s="116" t="s">
-        <v>322</v>
-      </c>
-      <c r="I32" s="116" t="s">
-        <v>323</v>
-      </c>
-      <c r="J32" s="117" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="33" ht="52.5" customHeight="1">
-      <c r="A33" s="113" t="s">
-        <v>325</v>
-      </c>
-      <c r="B33" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C33" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D33" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E33" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F33" s="115">
-        <v>650.0</v>
-      </c>
-      <c r="G33" s="116" t="s">
-        <v>326</v>
-      </c>
-      <c r="H33" s="116" t="s">
-        <v>317</v>
-      </c>
-      <c r="I33" s="116" t="s">
-        <v>318</v>
-      </c>
-      <c r="J33" s="117" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="34" ht="52.5" customHeight="1">
-      <c r="A34" s="113" t="s">
-        <v>328</v>
-      </c>
-      <c r="B34" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C34" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="D34" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="E34" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F34" s="115">
-        <v>300.0</v>
-      </c>
-      <c r="G34" s="116" t="s">
-        <v>329</v>
-      </c>
-      <c r="H34" s="116" t="s">
-        <v>330</v>
-      </c>
-      <c r="I34" s="116" t="s">
-        <v>331</v>
-      </c>
-      <c r="J34" s="117" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="35" ht="52.5" customHeight="1">
-      <c r="A35" s="113" t="s">
-        <v>333</v>
-      </c>
-      <c r="B35" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C35" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="D35" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="E35" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="F35" s="115">
-        <v>750.0</v>
-      </c>
-      <c r="G35" s="116" t="s">
-        <v>334</v>
-      </c>
-      <c r="H35" s="118" t="s">
-        <v>230</v>
-      </c>
-      <c r="I35" s="116" t="s">
-        <v>335</v>
-      </c>
-      <c r="J35" s="117" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="36" ht="52.5" customHeight="1">
-      <c r="A36" s="113" t="s">
-        <v>337</v>
-      </c>
-      <c r="B36" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C36" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="D36" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="E36" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="F36" s="115">
-        <v>450.0</v>
-      </c>
-      <c r="G36" s="116" t="s">
-        <v>338</v>
-      </c>
-      <c r="H36" s="118" t="s">
-        <v>230</v>
-      </c>
-      <c r="I36" s="116" t="s">
-        <v>339</v>
-      </c>
-      <c r="J36" s="117" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="37" ht="52.5" customHeight="1">
-      <c r="A37" s="113" t="s">
-        <v>341</v>
-      </c>
-      <c r="B37" s="114" t="b">
-        <v>0</v>
-      </c>
-      <c r="C37" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="D37" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="E37" s="114" t="b">
-        <v>1</v>
-      </c>
-      <c r="F37" s="115">
-        <v>500.0</v>
-      </c>
-      <c r="G37" s="116" t="s">
-        <v>242</v>
-      </c>
-      <c r="H37" s="116" t="s">
-        <v>277</v>
-      </c>
-      <c r="I37" s="116" t="s">
-        <v>342</v>
-      </c>
-      <c r="J37" s="117" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="38" ht="52.5" customHeight="1">
-      <c r="A38" s="119" t="s">
-        <v>344</v>
-      </c>
-      <c r="B38" s="120" t="b">
-        <v>0</v>
-      </c>
-      <c r="C38" s="120" t="b">
-        <v>1</v>
-      </c>
-      <c r="D38" s="120" t="b">
-        <v>1</v>
-      </c>
-      <c r="E38" s="120" t="b">
-        <v>1</v>
-      </c>
-      <c r="F38" s="121">
-        <v>600.0</v>
-      </c>
-      <c r="G38" s="122" t="s">
-        <v>242</v>
-      </c>
-      <c r="H38" s="123" t="s">
-        <v>230</v>
-      </c>
-      <c r="I38" s="122" t="s">
-        <v>345</v>
-      </c>
-      <c r="J38" s="124" t="s">
-        <v>346</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$6:$J$38"/>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="H9"/>
-    <hyperlink r:id="rId2" ref="H12"/>
-    <hyperlink r:id="rId3" ref="H19"/>
-    <hyperlink r:id="rId4" ref="H24"/>
-    <hyperlink r:id="rId5" ref="H30"/>
-    <hyperlink r:id="rId6" ref="H35"/>
-    <hyperlink r:id="rId7" ref="H36"/>
-    <hyperlink r:id="rId8" ref="H38"/>
-  </hyperlinks>
-  <drawing r:id="rId9"/>
+  <autoFilter ref="$A$7:$J$39"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
+  </mergeCells>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add savings estimate timing column
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -9,14 +9,14 @@
     <sheet state="visible" name="Services checklist" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Services checklist'!$A$7:$J$39</definedName>
+    <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Services checklist'!$A$7:$K$39</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="331">
   <si>
     <t>Savings Calculation Template</t>
   </si>
@@ -669,6 +669,9 @@
     <t>Mid-end DE estimate</t>
   </si>
   <si>
+    <t>Timing</t>
+  </si>
+  <si>
     <t>Basis / cost components</t>
   </si>
   <si>
@@ -681,6 +684,9 @@
     <t>Basic operating entity review</t>
   </si>
   <si>
+    <t>One-off</t>
+  </si>
+  <si>
     <t>Initial entity and accounting review; low uses public tax-advice plus basic support, mid includes deeper bookkeeping/accounting scoping</t>
   </si>
   <si>
@@ -708,6 +714,9 @@
     <t>Monthly bookkeeping/accounting package</t>
   </si>
   <si>
+    <t>Annual</t>
+  </si>
+  <si>
     <t>Recurring accounting package; low uses 99/month plus DATEV 15/month, mid uses 169/month plus DATEV 15/month</t>
   </si>
   <si>
@@ -717,6 +726,9 @@
     <t>Bookkeeping software setup and filing calendar setup</t>
   </si>
   <si>
+    <t>One-off setup</t>
+  </si>
+  <si>
     <t>Software setup, chart of accounts, filing calendar, access permissions, and recurring tool configuration; excludes monthly bookkeeping above</t>
   </si>
   <si>
@@ -753,6 +765,9 @@
     <t>Payroll setup, retroactive payslips and filings</t>
   </si>
   <si>
+    <t>One-off / catch-up</t>
+  </si>
+  <si>
     <t>Setup or correction project for payroll history, retroactive payslips, registrations, filings and payment reconciliation</t>
   </si>
   <si>
@@ -762,6 +777,9 @@
     <t>Office rent / company-address optimisation</t>
   </si>
   <si>
+    <t>Annual recurring</t>
+  </si>
+  <si>
     <t>Advisory plus benchmark analysis, company/person rent contract, and recurring monthly rent payment administration</t>
   </si>
   <si>
@@ -807,6 +825,9 @@
     <t>Authority, health insurer and penalty/fine resolution</t>
   </si>
   <si>
+    <t>Case-based</t>
+  </si>
+  <si>
     <t>Active case management: calls, letters, objections, escalation and chasing with Finanzamt, health insurers, payroll/social bodies and fine issuers</t>
   </si>
   <si>
@@ -816,6 +837,9 @@
     <t>Car purchase / depreciation planning</t>
   </si>
   <si>
+    <t>One-off planning</t>
+  </si>
+  <si>
     <t>Vehicle purchase, depreciation, benefit-in-kind and accounting treatment analysis; support estimate only, no vehicle cost included</t>
   </si>
   <si>
@@ -852,6 +876,9 @@
     <t>Dual tax jurisdiction / IE-DE tax residence review</t>
   </si>
   <si>
+    <t>One-off review</t>
+  </si>
+  <si>
     <t>Cross-border tax-residence review and dual-jurisdiction coordination estimate; excludes actual director service below</t>
   </si>
   <si>
@@ -897,6 +924,9 @@
     <t>Service agreement contracts with client customers</t>
   </si>
   <si>
+    <t>One-off / contract</t>
+  </si>
+  <si>
     <t>Contract preparation/review support estimate for customer service agreements and accounting/legal alignment</t>
   </si>
   <si>
@@ -906,6 +936,9 @@
     <t>Employment contract changes</t>
   </si>
   <si>
+    <t>One-off / change</t>
+  </si>
+  <si>
     <t>Employment/director contract change support plus payroll/accounting alignment and recurring payroll handover</t>
   </si>
   <si>
@@ -915,6 +948,9 @@
     <t>Share subscription agreements</t>
   </si>
   <si>
+    <t>One-off / document</t>
+  </si>
+  <si>
     <t>Share subscription agreement support estimate, including legal document review and company-record alignment</t>
   </si>
   <si>
@@ -924,6 +960,9 @@
     <t>RBO / beneficial-owner filing where applicable</t>
   </si>
   <si>
+    <t>Annual / event-based</t>
+  </si>
+  <si>
     <t>Beneficial-owner filing and annual/trigger-event monitoring support; checked in all options for IE company structures</t>
   </si>
   <si>
@@ -933,6 +972,9 @@
     <t>Personal tax bookkeeping and filing add-on</t>
   </si>
   <si>
+    <t>Optional annual</t>
+  </si>
+  <si>
     <t>Optional annual personal tax bookkeeping and filing estimate; separate from company operating entity services</t>
   </si>
   <si>
@@ -940,6 +982,9 @@
   </si>
   <si>
     <t>Parental leave planning</t>
+  </si>
+  <si>
+    <t>Optional planning</t>
   </si>
   <si>
     <t>Optional planning estimate for parental leave, owner salary timing, payroll impact and benefit timing</t>
@@ -1469,7 +1514,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="139">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1793,6 +1838,9 @@
     <xf borderId="21" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="21" fillId="8" fontId="15" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="21" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1814,6 +1862,9 @@
     <xf borderId="24" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="24" fillId="8" fontId="15" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="24" fillId="8" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1827,6 +1878,9 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="8" fontId="15" numFmtId="169" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="15" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="8" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -7321,9 +7375,10 @@
     <col customWidth="1" min="1" max="1" width="33.88"/>
     <col customWidth="1" min="2" max="5" width="15.13"/>
     <col customWidth="1" min="6" max="7" width="15.75"/>
-    <col customWidth="1" min="8" max="8" width="30.75"/>
-    <col customWidth="1" min="9" max="9" width="45.13"/>
-    <col customWidth="1" min="10" max="10" width="57.63"/>
+    <col customWidth="1" min="8" max="8" width="14.5"/>
+    <col customWidth="1" min="9" max="9" width="30.75"/>
+    <col customWidth="1" min="10" max="10" width="45.13"/>
+    <col customWidth="1" min="11" max="11" width="57.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.0" customHeight="1">
@@ -7356,6 +7411,7 @@
       <c r="H2" s="108"/>
       <c r="I2" s="108"/>
       <c r="J2" s="108"/>
+      <c r="K2" s="108"/>
     </row>
     <row r="3">
       <c r="A3" s="106" t="s">
@@ -7382,6 +7438,7 @@
       <c r="H3" s="108"/>
       <c r="I3" s="108"/>
       <c r="J3" s="108"/>
+      <c r="K3" s="108"/>
     </row>
     <row r="4">
       <c r="A4" s="106" t="s">
@@ -7408,6 +7465,7 @@
       <c r="H4" s="110"/>
       <c r="I4" s="110"/>
       <c r="J4" s="110"/>
+      <c r="K4" s="110"/>
     </row>
     <row r="5">
       <c r="A5" s="111" t="s">
@@ -7424,7 +7482,8 @@
       <c r="G6" s="113"/>
       <c r="H6" s="113"/>
       <c r="I6" s="113"/>
-      <c r="J6" s="114"/>
+      <c r="J6" s="113"/>
+      <c r="K6" s="114"/>
     </row>
     <row r="7" ht="37.5" customHeight="1">
       <c r="A7" s="115" t="s">
@@ -7454,13 +7513,16 @@
       <c r="I7" s="116" t="s">
         <v>218</v>
       </c>
-      <c r="J7" s="118" t="s">
+      <c r="J7" s="116" t="s">
         <v>219</v>
+      </c>
+      <c r="K7" s="118" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
       <c r="A8" s="119" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B8" s="120" t="b">
         <v>1</v>
@@ -7481,19 +7543,22 @@
         <v>1223.0</v>
       </c>
       <c r="H8" s="123" t="s">
-        <v>221</v>
-      </c>
-      <c r="I8" s="124" t="str">
+        <v>222</v>
+      </c>
+      <c r="I8" s="124" t="s">
+        <v>223</v>
+      </c>
+      <c r="J8" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","firma.de tax-advice benchmark plus professional-support estimate")</f>
         <v>firma.de tax-advice benchmark plus professional-support estimate</v>
       </c>
-      <c r="J8" s="125" t="s">
-        <v>222</v>
+      <c r="K8" s="126" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1">
       <c r="A9" s="119" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B9" s="120" t="b">
         <v>1</v>
@@ -7514,19 +7579,22 @@
         <v>1500.0</v>
       </c>
       <c r="H9" s="123" t="s">
-        <v>224</v>
-      </c>
-      <c r="I9" s="124" t="str">
+        <v>222</v>
+      </c>
+      <c r="I9" s="124" t="s">
+        <v>226</v>
+      </c>
+      <c r="J9" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/satzung/","firma.de company-document benchmark plus incorporation support estimate")</f>
         <v>firma.de company-document benchmark plus incorporation support estimate</v>
       </c>
-      <c r="J9" s="125" t="s">
-        <v>225</v>
+      <c r="K9" s="126" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="10" ht="31.5" customHeight="1">
       <c r="A10" s="119" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B10" s="120" t="b">
         <v>1</v>
@@ -7547,19 +7615,22 @@
         <v>600.0</v>
       </c>
       <c r="H10" s="123" t="s">
-        <v>227</v>
-      </c>
-      <c r="I10" s="124" t="str">
+        <v>222</v>
+      </c>
+      <c r="I10" s="124" t="s">
+        <v>229</v>
+      </c>
+      <c r="J10" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for document intake and admin support")</f>
         <v>StBVV-style time-fee benchmark for document intake and admin support</v>
       </c>
-      <c r="J10" s="125" t="s">
-        <v>228</v>
+      <c r="K10" s="126" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="11" ht="31.5" customHeight="1">
       <c r="A11" s="119" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B11" s="120" t="b">
         <v>1</v>
@@ -7580,19 +7651,22 @@
         <v>2208.0</v>
       </c>
       <c r="H11" s="123" t="s">
-        <v>230</v>
-      </c>
-      <c r="I11" s="124" t="str">
+        <v>232</v>
+      </c>
+      <c r="I11" s="124" t="s">
+        <v>233</v>
+      </c>
+      <c r="J11" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/buchhaltung/","firma.de bookkeeping package prices including DATEV software add-on")</f>
         <v>firma.de bookkeeping package prices including DATEV software add-on</v>
       </c>
-      <c r="J11" s="125" t="s">
-        <v>231</v>
+      <c r="K11" s="126" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="12" ht="31.5" customHeight="1">
       <c r="A12" s="119" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B12" s="120" t="b">
         <v>1</v>
@@ -7613,19 +7687,22 @@
         <v>600.0</v>
       </c>
       <c r="H12" s="123" t="s">
-        <v>233</v>
-      </c>
-      <c r="I12" s="124" t="str">
+        <v>236</v>
+      </c>
+      <c r="I12" s="124" t="s">
+        <v>237</v>
+      </c>
+      <c r="J12" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware Office software prices used where a tool cost is needed")</f>
         <v>Lexware Office software prices used where a tool cost is needed</v>
       </c>
-      <c r="J12" s="125" t="s">
-        <v>234</v>
+      <c r="K12" s="126" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="13" ht="31.5" customHeight="1">
       <c r="A13" s="119" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B13" s="120" t="b">
         <v>1</v>
@@ -7646,19 +7723,22 @@
         <v>1200.0</v>
       </c>
       <c r="H13" s="123" t="s">
-        <v>236</v>
-      </c>
-      <c r="I13" s="124" t="str">
+        <v>232</v>
+      </c>
+      <c r="I13" s="124" t="s">
+        <v>240</v>
+      </c>
+      <c r="J13" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware VAT filing and software-pricing reference for tool costs")</f>
         <v>Lexware VAT filing and software-pricing reference for tool costs</v>
       </c>
-      <c r="J13" s="125" t="s">
-        <v>237</v>
+      <c r="K13" s="126" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="14" ht="31.5" customHeight="1">
       <c r="A14" s="119" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B14" s="120" t="b">
         <v>1</v>
@@ -7679,19 +7759,22 @@
         <v>2048.0</v>
       </c>
       <c r="H14" s="123" t="s">
-        <v>239</v>
-      </c>
-      <c r="I14" s="124" t="str">
+        <v>232</v>
+      </c>
+      <c r="I14" s="124" t="s">
+        <v>243</v>
+      </c>
+      <c r="J14" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/jahresabschluss-kapitalgesellschaft/","firma.de annual accounts prices plus disclosure filing add-on")</f>
         <v>firma.de annual accounts prices plus disclosure filing add-on</v>
       </c>
-      <c r="J14" s="125" t="s">
-        <v>240</v>
+      <c r="K14" s="126" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="15" ht="31.5" customHeight="1">
       <c r="A15" s="119" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B15" s="120" t="b">
         <v>1</v>
@@ -7712,19 +7795,22 @@
         <v>395.0</v>
       </c>
       <c r="H15" s="123" t="s">
-        <v>242</v>
-      </c>
-      <c r="I15" s="124" t="str">
+        <v>232</v>
+      </c>
+      <c r="I15" s="124" t="s">
+        <v>246</v>
+      </c>
+      <c r="J15" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/lohnabrechnung/","firma.de payroll benchmark; mid estimate also includes payroll tool cost")</f>
         <v>firma.de payroll benchmark; mid estimate also includes payroll tool cost</v>
       </c>
-      <c r="J15" s="125" t="s">
-        <v>243</v>
+      <c r="K15" s="126" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="16" ht="31.5" customHeight="1">
       <c r="A16" s="119" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B16" s="120" t="b">
         <v>1</v>
@@ -7745,19 +7831,22 @@
         <v>1000.0</v>
       </c>
       <c r="H16" s="123" t="s">
-        <v>245</v>
-      </c>
-      <c r="I16" s="124" t="str">
+        <v>249</v>
+      </c>
+      <c r="I16" s="124" t="s">
+        <v>250</v>
+      </c>
+      <c r="J16" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware payroll filing/tool reference plus setup-support estimate")</f>
         <v>Lexware payroll filing/tool reference plus setup-support estimate</v>
       </c>
-      <c r="J16" s="125" t="s">
-        <v>246</v>
+      <c r="K16" s="126" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="17" ht="31.5" customHeight="1">
       <c r="A17" s="119" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B17" s="120" t="b">
         <v>0</v>
@@ -7778,19 +7867,22 @@
         <v>2400.0</v>
       </c>
       <c r="H17" s="123" t="s">
-        <v>248</v>
-      </c>
-      <c r="I17" s="124" t="str">
+        <v>253</v>
+      </c>
+      <c r="I17" s="124" t="s">
+        <v>254</v>
+      </c>
+      <c r="J17" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for rent analysis, contract and recurring payment work")</f>
         <v>Professional time-fee benchmark for rent analysis, contract and recurring payment work</v>
       </c>
-      <c r="J17" s="125" t="s">
-        <v>249</v>
+      <c r="K17" s="126" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="18" ht="31.5" customHeight="1">
       <c r="A18" s="119" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="B18" s="120" t="b">
         <v>0</v>
@@ -7811,19 +7903,22 @@
         <v>1800.0</v>
       </c>
       <c r="H18" s="123" t="s">
-        <v>251</v>
-      </c>
-      <c r="I18" s="124" t="str">
+        <v>253</v>
+      </c>
+      <c r="I18" s="124" t="s">
+        <v>257</v>
+      </c>
+      <c r="J18" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for recurring expense and travel-support work")</f>
         <v>Professional time-fee benchmark for recurring expense and travel-support work</v>
       </c>
-      <c r="J18" s="125" t="s">
-        <v>252</v>
+      <c r="K18" s="126" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
       <c r="A19" s="119" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B19" s="120" t="b">
         <v>0</v>
@@ -7844,19 +7939,22 @@
         <v>2663.0</v>
       </c>
       <c r="H19" s="123" t="s">
-        <v>254</v>
-      </c>
-      <c r="I19" s="124" t="str">
+        <v>253</v>
+      </c>
+      <c r="I19" s="124" t="s">
+        <v>260</v>
+      </c>
+      <c r="J19" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware invoicing, banking, payment and bookkeeping tool-cost reference")</f>
         <v>Lexware invoicing, banking, payment and bookkeeping tool-cost reference</v>
       </c>
-      <c r="J19" s="125" t="s">
-        <v>255</v>
+      <c r="K19" s="126" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="20" ht="31.5" customHeight="1">
       <c r="A20" s="119" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B20" s="120" t="b">
         <v>1</v>
@@ -7877,19 +7975,22 @@
         <v>1200.0</v>
       </c>
       <c r="H20" s="123" t="s">
-        <v>257</v>
-      </c>
-      <c r="I20" s="124" t="str">
+        <v>253</v>
+      </c>
+      <c r="I20" s="124" t="s">
+        <v>263</v>
+      </c>
+      <c r="J20" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style recurring support benchmark for tax-payment tracking")</f>
         <v>StBVV-style recurring support benchmark for tax-payment tracking</v>
       </c>
-      <c r="J20" s="125" t="s">
-        <v>258</v>
+      <c r="K20" s="126" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="21" ht="31.5" customHeight="1">
       <c r="A21" s="119" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B21" s="120" t="b">
         <v>1</v>
@@ -7910,19 +8011,22 @@
         <v>1800.0</v>
       </c>
       <c r="H21" s="123" t="s">
-        <v>260</v>
-      </c>
-      <c r="I21" s="124" t="str">
+        <v>253</v>
+      </c>
+      <c r="I21" s="124" t="s">
+        <v>266</v>
+      </c>
+      <c r="J21" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for correspondence support and authority letters")</f>
         <v>Tax-advice benchmark for correspondence support and authority letters</v>
       </c>
-      <c r="J21" s="125" t="s">
-        <v>261</v>
+      <c r="K21" s="126" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="22" ht="31.5" customHeight="1">
       <c r="A22" s="119" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B22" s="120" t="b">
         <v>1</v>
@@ -7943,19 +8047,22 @@
         <v>1500.0</v>
       </c>
       <c r="H22" s="123" t="s">
-        <v>263</v>
-      </c>
-      <c r="I22" s="124" t="str">
+        <v>269</v>
+      </c>
+      <c r="I22" s="124" t="s">
+        <v>270</v>
+      </c>
+      <c r="J22" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for authority correspondence and case work")</f>
         <v>Professional time-fee benchmark for authority correspondence and case work</v>
       </c>
-      <c r="J22" s="125" t="s">
-        <v>264</v>
+      <c r="K22" s="126" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="23" ht="31.5" customHeight="1">
       <c r="A23" s="119" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B23" s="120" t="b">
         <v>0</v>
@@ -7976,19 +8083,22 @@
         <v>700.0</v>
       </c>
       <c r="H23" s="123" t="s">
-        <v>266</v>
-      </c>
-      <c r="I23" s="124" t="str">
+        <v>273</v>
+      </c>
+      <c r="I23" s="124" t="s">
+        <v>274</v>
+      </c>
+      <c r="J23" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for depreciation and tax-planning analysis")</f>
         <v>Professional benchmark for depreciation and tax-planning analysis</v>
       </c>
-      <c r="J23" s="125" t="s">
-        <v>267</v>
+      <c r="K23" s="126" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="24" ht="31.5" customHeight="1">
       <c r="A24" s="119" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="B24" s="120" t="b">
         <v>0</v>
@@ -8009,19 +8119,22 @@
         <v>700.0</v>
       </c>
       <c r="H24" s="123" t="s">
-        <v>269</v>
-      </c>
-      <c r="I24" s="124" t="str">
+        <v>273</v>
+      </c>
+      <c r="I24" s="124" t="s">
+        <v>277</v>
+      </c>
+      <c r="J24" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for retained-profit and investment planning")</f>
         <v>Tax-advice benchmark for retained-profit and investment planning</v>
       </c>
-      <c r="J24" s="125" t="s">
-        <v>270</v>
+      <c r="K24" s="126" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="25" ht="31.5" customHeight="1">
       <c r="A25" s="119" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="B25" s="120" t="b">
         <v>0</v>
@@ -8042,19 +8155,22 @@
         <v>500.0</v>
       </c>
       <c r="H25" s="123" t="s">
-        <v>272</v>
-      </c>
-      <c r="I25" s="124" t="str">
+        <v>236</v>
+      </c>
+      <c r="I25" s="124" t="s">
+        <v>280</v>
+      </c>
+      <c r="J25" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for setup and evidence handling")</f>
         <v>Professional support benchmark for setup and evidence handling</v>
       </c>
-      <c r="J25" s="125" t="s">
-        <v>273</v>
+      <c r="K25" s="126" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="26" ht="31.5" customHeight="1">
       <c r="A26" s="119" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="B26" s="120" t="b">
         <v>0</v>
@@ -8075,19 +8191,22 @@
         <v>1000.0</v>
       </c>
       <c r="H26" s="123" t="s">
-        <v>275</v>
-      </c>
-      <c r="I26" s="124" t="str">
+        <v>273</v>
+      </c>
+      <c r="I26" s="124" t="s">
+        <v>283</v>
+      </c>
+      <c r="J26" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for pension reserve planning support")</f>
         <v>Tax-advice benchmark for pension reserve planning support</v>
       </c>
-      <c r="J26" s="125" t="s">
-        <v>276</v>
+      <c r="K26" s="126" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="27" ht="31.5" customHeight="1">
       <c r="A27" s="119" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="B27" s="120" t="b">
         <v>0</v>
@@ -8108,19 +8227,22 @@
         <v>2000.0</v>
       </c>
       <c r="H27" s="123" t="s">
-        <v>278</v>
-      </c>
-      <c r="I27" s="124" t="str">
+        <v>286</v>
+      </c>
+      <c r="I27" s="124" t="s">
+        <v>287</v>
+      </c>
+      <c r="J27" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for complex cross-border tax and accounting work")</f>
         <v>Professional benchmark for complex cross-border tax and accounting work</v>
       </c>
-      <c r="J27" s="125" t="s">
-        <v>279</v>
+      <c r="K27" s="126" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="28" ht="31.5" customHeight="1">
       <c r="A28" s="119" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="B28" s="120" t="b">
         <v>0</v>
@@ -8141,19 +8263,22 @@
         <v>6000.0</v>
       </c>
       <c r="H28" s="123" t="s">
-        <v>281</v>
-      </c>
-      <c r="I28" s="124" t="str">
+        <v>253</v>
+      </c>
+      <c r="I28" s="124" t="s">
+        <v>290</v>
+      </c>
+      <c r="J28" s="125" t="str">
         <f>HYPERLINK("https://www.irishstatutebook.ie/eli/2014/act/38/section/137/enacted/en/html","Irish Companies Act director-residence reference plus annual director-service estimate")</f>
         <v>Irish Companies Act director-residence reference plus annual director-service estimate</v>
       </c>
-      <c r="J28" s="125" t="s">
-        <v>282</v>
+      <c r="K28" s="126" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="29" ht="31.5" customHeight="1">
       <c r="A29" s="119" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="B29" s="120" t="b">
         <v>1</v>
@@ -8174,19 +8299,22 @@
         <v>600.0</v>
       </c>
       <c r="H29" s="123" t="s">
-        <v>284</v>
-      </c>
-      <c r="I29" s="124" t="str">
+        <v>236</v>
+      </c>
+      <c r="I29" s="124" t="s">
+        <v>293</v>
+      </c>
+      <c r="J29" s="125" t="str">
         <f>HYPERLINK("https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service","Bundesagentur employer-number service plus employer registration support estimate")</f>
         <v>Bundesagentur employer-number service plus employer registration support estimate</v>
       </c>
-      <c r="J29" s="125" t="s">
-        <v>285</v>
+      <c r="K29" s="126" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="30" ht="31.5" customHeight="1">
       <c r="A30" s="119" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="B30" s="120" t="b">
         <v>1</v>
@@ -8207,19 +8335,22 @@
         <v>531.0</v>
       </c>
       <c r="H30" s="123" t="s">
-        <v>287</v>
-      </c>
-      <c r="I30" s="124" t="str">
+        <v>222</v>
+      </c>
+      <c r="I30" s="124" t="s">
+        <v>296</v>
+      </c>
+      <c r="J30" s="125" t="str">
         <f>HYPERLINK("https://service.berlin.de/dienstleistung/121921/","Berlin Gewerbeanmeldung fee reference plus registration support estimate")</f>
         <v>Berlin Gewerbeanmeldung fee reference plus registration support estimate</v>
       </c>
-      <c r="J30" s="125" t="s">
-        <v>288</v>
+      <c r="K30" s="126" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="31" ht="31.5" customHeight="1">
       <c r="A31" s="119" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="B31" s="120" t="b">
         <v>0</v>
@@ -8240,19 +8371,22 @@
         <v>500.0</v>
       </c>
       <c r="H31" s="123" t="s">
-        <v>290</v>
-      </c>
-      <c r="I31" s="124" t="str">
+        <v>236</v>
+      </c>
+      <c r="I31" s="124" t="s">
+        <v>299</v>
+      </c>
+      <c r="J31" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for bank-account setup and records")</f>
         <v>Professional support benchmark for bank-account setup and records</v>
       </c>
-      <c r="J31" s="125" t="s">
-        <v>291</v>
+      <c r="K31" s="126" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="32" ht="31.5" customHeight="1">
       <c r="A32" s="119" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="B32" s="120" t="b">
         <v>0</v>
@@ -8273,19 +8407,22 @@
         <v>1200.0</v>
       </c>
       <c r="H32" s="123" t="s">
-        <v>293</v>
-      </c>
-      <c r="I32" s="124" t="str">
+        <v>302</v>
+      </c>
+      <c r="I32" s="124" t="s">
+        <v>303</v>
+      </c>
+      <c r="J32" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for service agreement support")</f>
         <v>Legal-consultation benchmark for service agreement support</v>
       </c>
-      <c r="J32" s="125" t="s">
-        <v>294</v>
+      <c r="K32" s="126" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
       <c r="A33" s="119" t="s">
-        <v>295</v>
+        <v>305</v>
       </c>
       <c r="B33" s="120" t="b">
         <v>0</v>
@@ -8306,19 +8443,22 @@
         <v>1000.0</v>
       </c>
       <c r="H33" s="123" t="s">
-        <v>296</v>
-      </c>
-      <c r="I33" s="124" t="str">
+        <v>306</v>
+      </c>
+      <c r="I33" s="124" t="s">
+        <v>307</v>
+      </c>
+      <c r="J33" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for employment contract change support")</f>
         <v>Legal-consultation benchmark for employment contract change support</v>
       </c>
-      <c r="J33" s="125" t="s">
-        <v>297</v>
+      <c r="K33" s="126" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
       <c r="A34" s="119" t="s">
-        <v>298</v>
+        <v>309</v>
       </c>
       <c r="B34" s="120" t="b">
         <v>0</v>
@@ -8339,19 +8479,22 @@
         <v>1300.0</v>
       </c>
       <c r="H34" s="123" t="s">
-        <v>299</v>
-      </c>
-      <c r="I34" s="124" t="str">
+        <v>310</v>
+      </c>
+      <c r="I34" s="124" t="s">
+        <v>311</v>
+      </c>
+      <c r="J34" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/satzung/","Company-document benchmark for shareholder/subscription document support")</f>
         <v>Company-document benchmark for shareholder/subscription document support</v>
       </c>
-      <c r="J34" s="125" t="s">
-        <v>300</v>
+      <c r="K34" s="126" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
       <c r="A35" s="119" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="B35" s="120" t="b">
         <v>1</v>
@@ -8372,19 +8515,22 @@
         <v>600.0</v>
       </c>
       <c r="H35" s="123" t="s">
-        <v>302</v>
-      </c>
-      <c r="I35" s="124" t="str">
+        <v>314</v>
+      </c>
+      <c r="I35" s="124" t="s">
+        <v>315</v>
+      </c>
+      <c r="J35" s="125" t="str">
         <f>HYPERLINK("https://rbo.gov.ie/","RBO Ireland official filing route for relevant Irish incorporated entities")</f>
         <v>RBO Ireland official filing route for relevant Irish incorporated entities</v>
       </c>
-      <c r="J35" s="125" t="s">
-        <v>303</v>
+      <c r="K35" s="126" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
       <c r="A36" s="119" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="B36" s="120" t="b">
         <v>0</v>
@@ -8405,19 +8551,22 @@
         <v>1500.0</v>
       </c>
       <c r="H36" s="123" t="s">
-        <v>305</v>
-      </c>
-      <c r="I36" s="124" t="str">
+        <v>318</v>
+      </c>
+      <c r="I36" s="124" t="s">
+        <v>319</v>
+      </c>
+      <c r="J36" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV personal tax filing and income-calculation benchmark")</f>
         <v>StBVV personal tax filing and income-calculation benchmark</v>
       </c>
-      <c r="J36" s="125" t="s">
-        <v>306</v>
+      <c r="K36" s="126" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="37" ht="31.5" customHeight="1">
       <c r="A37" s="119" t="s">
-        <v>307</v>
+        <v>321</v>
       </c>
       <c r="B37" s="120" t="b">
         <v>0</v>
@@ -8438,52 +8587,58 @@
         <v>900.0</v>
       </c>
       <c r="H37" s="123" t="s">
-        <v>308</v>
-      </c>
-      <c r="I37" s="124" t="str">
+        <v>322</v>
+      </c>
+      <c r="I37" s="124" t="s">
+        <v>323</v>
+      </c>
+      <c r="J37" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for parental leave and salary-timing planning")</f>
         <v>Professional support benchmark for parental leave and salary-timing planning</v>
       </c>
-      <c r="J37" s="125" t="s">
-        <v>309</v>
+      <c r="K37" s="126" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="38" ht="31.5" customHeight="1">
-      <c r="A38" s="126" t="s">
-        <v>310</v>
-      </c>
-      <c r="B38" s="127" t="b">
+      <c r="A38" s="127" t="s">
+        <v>325</v>
+      </c>
+      <c r="B38" s="128" t="b">
         <v>0</v>
       </c>
-      <c r="C38" s="127" t="b">
-        <v>1</v>
-      </c>
-      <c r="D38" s="127" t="b">
-        <v>1</v>
-      </c>
-      <c r="E38" s="127" t="b">
-        <v>1</v>
-      </c>
-      <c r="F38" s="128">
+      <c r="C38" s="128" t="b">
+        <v>1</v>
+      </c>
+      <c r="D38" s="128" t="b">
+        <v>1</v>
+      </c>
+      <c r="E38" s="128" t="b">
+        <v>1</v>
+      </c>
+      <c r="F38" s="129">
         <v>500.0</v>
       </c>
-      <c r="G38" s="129">
+      <c r="G38" s="130">
         <v>1000.0</v>
       </c>
-      <c r="H38" s="130" t="s">
-        <v>311</v>
-      </c>
-      <c r="I38" s="131" t="str">
+      <c r="H38" s="131" t="s">
+        <v>314</v>
+      </c>
+      <c r="I38" s="132" t="s">
+        <v>326</v>
+      </c>
+      <c r="J38" s="133" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for forecast and life-change planning support")</f>
         <v>Tax-advice benchmark for forecast and life-change planning support</v>
       </c>
-      <c r="J38" s="132" t="s">
-        <v>312</v>
+      <c r="K38" s="134" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
-      <c r="A39" s="133" t="s">
-        <v>313</v>
+      <c r="A39" s="135" t="s">
+        <v>328</v>
       </c>
       <c r="B39" s="110" t="b">
         <v>0</v>
@@ -8497,28 +8652,31 @@
       <c r="E39" s="110" t="b">
         <v>1</v>
       </c>
-      <c r="F39" s="134">
+      <c r="F39" s="136">
         <v>600.0</v>
       </c>
-      <c r="G39" s="134">
+      <c r="G39" s="136">
         <v>1200.0</v>
       </c>
-      <c r="H39" s="110" t="s">
-        <v>314</v>
-      </c>
-      <c r="I39" s="135" t="str">
+      <c r="H39" s="137" t="s">
+        <v>253</v>
+      </c>
+      <c r="I39" s="110" t="s">
+        <v>329</v>
+      </c>
+      <c r="J39" s="138" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for recurring client support")</f>
         <v>StBVV-style time-fee benchmark for recurring client support</v>
       </c>
-      <c r="J39" s="110" t="s">
-        <v>315</v>
+      <c r="K39" s="110" t="s">
+        <v>330</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$7:$J$39"/>
+  <autoFilter ref="$A$7:$K$39"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Clarify recurring filing and payment scope
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="333">
   <si>
     <t>Savings Calculation Template</t>
   </si>
@@ -501,7 +501,7 @@
     <t>Applies to optimisation options when employee count exceeds threshold</t>
   </si>
   <si>
-    <t>Shown as separate line in Option 3</t>
+    <t>Annual surcharge shown as separate line in Option 3 for pension reserve planning plus recurring reserve accounting/year-end support</t>
   </si>
   <si>
     <t>Shown as separate line in Option 4</t>
@@ -525,13 +525,13 @@
     <t>1000 plus employee surcharge</t>
   </si>
   <si>
-    <t>Office rent, business travel, eligible expenses, car depreciation, and investment planning; pension reserve excluded</t>
+    <t>Office rent, business travel, eligible expenses, car depreciation, and investment/startup shareholding planning, including recurring accounting uplift where those structures are used; pension reserve excluded</t>
   </si>
   <si>
     <t>1000 plus pension surcharge plus employee surcharge if applicable</t>
   </si>
   <si>
-    <t>Option 2 scope plus pension reserve planning</t>
+    <t>Option 2 scope plus pension reserve planning and annual reserve accounting/year-end support</t>
   </si>
   <si>
     <t>1000 plus dual tax jurisdiction and discounted director surcharge plus employee surcharge if applicable</t>
@@ -657,7 +657,7 @@
     <t>Standalone DE market value checked - mid</t>
   </si>
   <si>
-    <t>Status: provisional. Source: RB service-list work, user corrections, and public pricing/statutory references checked 2026-06-15. Low/mid estimates include advisory support plus third-party software, filing, and public-authority costs where relevant; review before client reliance.</t>
+    <t>Status: provisional. Source: RB service-list work, user corrections, ELSTER official filing-form list, and public pricing/statutory references checked 2026-06-15. Low/mid estimates include advisory support plus third-party software, filing, payment administration and recurring accounting uplift where relevant; review before client reliance.</t>
   </si>
   <si>
     <t>Service</t>
@@ -735,31 +735,37 @@
     <t>Make the operating calendar and software stack explicit before the client chooses the option</t>
   </si>
   <si>
-    <t>VAT compliance / VAT filings</t>
-  </si>
-  <si>
-    <t>Recurring VAT filing support plus filing-software/transmission setup where needed; low assumes lighter filing volume, mid assumes monthly complexity</t>
-  </si>
-  <si>
-    <t>Track VAT deadlines, prepare filings, submit returns, and retain filing/payment evidence</t>
-  </si>
-  <si>
-    <t>Annual accounts and corporate tax filings</t>
-  </si>
-  <si>
-    <t>Annual accounts plus disclosure/filing; low uses 1249 plus 99 disclosure, mid uses 1949 plus 99 disclosure</t>
-  </si>
-  <si>
-    <t>Annual compliance is separate from monthly bookkeeping and should stay visible in the service comparison</t>
+    <t>VAT compliance / quarterly VAT filings</t>
+  </si>
+  <si>
+    <t>Quarterly + annual</t>
+  </si>
+  <si>
+    <t>Quarterly VAT pre-returns (monthly where required), annual VAT return, filing-software/transmission setup, deadline/payment tracking and evidence retention</t>
+  </si>
+  <si>
+    <t>VAT estimate includes quarterly pre-returns and annual VAT return, not only year-end filing</t>
+  </si>
+  <si>
+    <t>Annual accounts, e-Bilanz and corporate/trade tax filings</t>
+  </si>
+  <si>
+    <t>Annual accounts, disclosure/filing, e-Bilanz transmission, corporate tax return and trade tax return; VAT filings are costed in the VAT row</t>
+  </si>
+  <si>
+    <t>Annual filing scope should cover accounts, e-Bilanz, corporation tax and trade tax; VAT is shown separately</t>
   </si>
   <si>
     <t>Payroll for one employee</t>
   </si>
   <si>
-    <t>Recurring payroll plus payroll-software/filing component; low uses payroll service benchmark, mid adds Lexware payroll add-on at 12.90/month</t>
-  </si>
-  <si>
-    <t>Run payroll, social-insurance and wage-tax filings, payments, and evidence capture for the employee</t>
+    <t>Monthly / annual</t>
+  </si>
+  <si>
+    <t>Monthly payroll calculations, payslips, wage-tax/social filings, net salary payment, wage-tax payment, social-charge payment coordination/execution, payroll software and evidence capture</t>
+  </si>
+  <si>
+    <t>Yes: payroll service should include making the net salary, wage-tax and social-insurance payments on time, not just producing payslips</t>
   </si>
   <si>
     <t>Payroll setup, retroactive payslips and filings</t>
@@ -834,43 +840,43 @@
     <t>Call Finanzamt and health insurers, fight fines, and keep issue ownership until resolved</t>
   </si>
   <si>
-    <t>Car purchase / depreciation planning</t>
-  </si>
-  <si>
-    <t>One-off planning</t>
-  </si>
-  <si>
-    <t>Vehicle purchase, depreciation, benefit-in-kind and accounting treatment analysis; support estimate only, no vehicle cost included</t>
-  </si>
-  <si>
-    <t>Analyse car purchase and depreciation treatment before committing to the company purchase</t>
-  </si>
-  <si>
-    <t>Investment / retained-profit planning</t>
-  </si>
-  <si>
-    <t>Retained-profit investment planning and accounting/tax treatment review; advisory support estimate, not investment-management fees</t>
-  </si>
-  <si>
-    <t>Help decide whether retained profits should be invested or held for taxes, salary and reserve planning</t>
+    <t>Car purchase / depreciation planning and annual accounting</t>
+  </si>
+  <si>
+    <t>One-off + annual</t>
+  </si>
+  <si>
+    <t>Car purchase/depreciation planning plus annual fixed-asset register, depreciation postings, private-use/accounting reconciliation and year-end tax support; vehicle cost excluded</t>
+  </si>
+  <si>
+    <t>Include both the decision/planning work and the recurring depreciation accounting uplift</t>
+  </si>
+  <si>
+    <t>Investment / retained-profit and startup shareholding planning</t>
+  </si>
+  <si>
+    <t>Retained-profit investment planning, startup shareholding transfer planning, accounting/tax treatment review and annual investment/valuation/accounting support; investment-management fees excluded</t>
+  </si>
+  <si>
+    <t>For startup investments, include the annual accounting/tax uplift after the structure is set up</t>
   </si>
   <si>
     <t>Investment account setup</t>
   </si>
   <si>
-    <t>Administrative setup estimate for investment account documents, evidence, accounting treatment and source-record workflow</t>
-  </si>
-  <si>
-    <t>Set up the investment-account records correctly if the client decides to invest retained profits</t>
-  </si>
-  <si>
-    <t>Pension reserve planning</t>
-  </si>
-  <si>
-    <t>Additional pension reserve analysis and documentation; reflected as the separate RB pension surcharge line in option 3</t>
-  </si>
-  <si>
-    <t>Only included when the client chooses the pension reserve add-on</t>
+    <t>Administrative setup estimate for investment account documents, evidence, accounting treatment and source-record workflow; recurring investment accounting is captured in the investment planning row</t>
+  </si>
+  <si>
+    <t>Set up the account/evidence workflow; do not treat this as the full recurring investment-accounting cost</t>
+  </si>
+  <si>
+    <t>Pension reserve planning and annual accounting</t>
+  </si>
+  <si>
+    <t>Pension reserve analysis plus recurring annual accounting, documentation, reserve movement review and year-end tax support; reflected as RB pension surcharge in option 3 but standalone DE estimate includes annual uplift</t>
+  </si>
+  <si>
+    <t>Planning is not enough; pension reserve creates recurring accounting/year-end work</t>
   </si>
   <si>
     <t>Dual tax jurisdiction / IE-DE tax residence review</t>
@@ -945,16 +951,16 @@
     <t>Change employment or director contracts and align payroll/accounting treatment</t>
   </si>
   <si>
-    <t>Share subscription agreements</t>
-  </si>
-  <si>
-    <t>One-off / document</t>
-  </si>
-  <si>
-    <t>Share subscription agreement support estimate, including legal document review and company-record alignment</t>
-  </si>
-  <si>
-    <t>Prepare share subscription agreements where the structure needs them</t>
+    <t>Share subscription / personal shareholding transfer agreements and filings</t>
+  </si>
+  <si>
+    <t>One-off + filings</t>
+  </si>
+  <si>
+    <t>Agreement drafting/review plus shareholder/company approvals, share-capital/cap-table updates, corporate-register filings and notary coordination where required; external notary/statutory fees may be extra</t>
+  </si>
+  <si>
+    <t>For moving a personal startup shareholding into a company, check filings, notary route, share-capital changes and external fees</t>
   </si>
   <si>
     <t>RBO / beneficial-owner filing where applicable</t>
@@ -7419,19 +7425,19 @@
       </c>
       <c r="B3" s="107">
         <f t="shared" ref="B3:E3" si="1">SUMIF(B8:B39,TRUE,$F$8:$F$39)</f>
-        <v>9511</v>
+        <v>10743</v>
       </c>
       <c r="C3" s="107">
         <f t="shared" si="1"/>
-        <v>17016</v>
+        <v>19998</v>
       </c>
       <c r="D3" s="107">
         <f t="shared" si="1"/>
-        <v>17516</v>
+        <v>20898</v>
       </c>
       <c r="E3" s="107">
         <f t="shared" si="1"/>
-        <v>21016</v>
+        <v>23998</v>
       </c>
       <c r="F3" s="108"/>
       <c r="G3" s="108"/>
@@ -7446,19 +7452,19 @@
       </c>
       <c r="B4" s="109">
         <f t="shared" ref="B4:E4" si="2">SUMIF(B8:B39,TRUE,$G$8:$G$39)</f>
-        <v>17005</v>
+        <v>19802</v>
       </c>
       <c r="C4" s="109">
         <f t="shared" si="2"/>
-        <v>31968</v>
+        <v>38265</v>
       </c>
       <c r="D4" s="109">
         <f t="shared" si="2"/>
-        <v>32968</v>
+        <v>40065</v>
       </c>
       <c r="E4" s="109">
         <f t="shared" si="2"/>
-        <v>39968</v>
+        <v>46265</v>
       </c>
       <c r="F4" s="110"/>
       <c r="G4" s="110"/>
@@ -7717,28 +7723,28 @@
         <v>1</v>
       </c>
       <c r="F13" s="121">
-        <v>600.0</v>
+        <v>1000.0</v>
       </c>
       <c r="G13" s="122">
-        <v>1200.0</v>
+        <v>2200.0</v>
       </c>
       <c r="H13" s="123" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="I13" s="124" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J13" s="125" t="str">
-        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware VAT filing and software-pricing reference for tool costs")</f>
-        <v>Lexware VAT filing and software-pricing reference for tool costs</v>
+        <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Umsatzsteuer-Voranmeldung and Umsatzsteuererklärung forms")</f>
+        <v>ELSTER lists Umsatzsteuer-Voranmeldung and Umsatzsteuererklärung forms</v>
       </c>
       <c r="K13" s="126" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" ht="31.5" customHeight="1">
       <c r="A14" s="119" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B14" s="120" t="b">
         <v>1</v>
@@ -7753,28 +7759,28 @@
         <v>1</v>
       </c>
       <c r="F14" s="121">
-        <v>1348.0</v>
+        <v>1700.0</v>
       </c>
       <c r="G14" s="122">
-        <v>2048.0</v>
+        <v>2800.0</v>
       </c>
       <c r="H14" s="123" t="s">
         <v>232</v>
       </c>
       <c r="I14" s="124" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="J14" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/jahresabschluss-kapitalgesellschaft/","firma.de annual accounts prices plus disclosure filing add-on")</f>
-        <v>firma.de annual accounts prices plus disclosure filing add-on</v>
+        <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Körperschaftsteuererklärung and Gewerbesteuererklärung; annual accounts benchmark added separately")</f>
+        <v>ELSTER lists Körperschaftsteuererklärung and Gewerbesteuererklärung; annual accounts benchmark added separately</v>
       </c>
       <c r="K14" s="126" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15" ht="31.5" customHeight="1">
       <c r="A15" s="119" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B15" s="120" t="b">
         <v>1</v>
@@ -7789,28 +7795,28 @@
         <v>1</v>
       </c>
       <c r="F15" s="121">
-        <v>240.0</v>
+        <v>720.0</v>
       </c>
       <c r="G15" s="122">
-        <v>395.0</v>
+        <v>1440.0</v>
       </c>
       <c r="H15" s="123" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="I15" s="124" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="J15" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/lohnabrechnung/","firma.de payroll benchmark; mid estimate also includes payroll tool cost")</f>
-        <v>firma.de payroll benchmark; mid estimate also includes payroll tool cost</v>
+        <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Lohnsteuer-Anmeldung; estimate includes payment-run administration")</f>
+        <v>ELSTER lists Lohnsteuer-Anmeldung; estimate includes payment-run administration</v>
       </c>
       <c r="K15" s="126" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" ht="31.5" customHeight="1">
       <c r="A16" s="119" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B16" s="120" t="b">
         <v>1</v>
@@ -7831,22 +7837,22 @@
         <v>1000.0</v>
       </c>
       <c r="H16" s="123" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="I16" s="124" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="J16" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware payroll filing/tool reference plus setup-support estimate")</f>
         <v>Lexware payroll filing/tool reference plus setup-support estimate</v>
       </c>
       <c r="K16" s="126" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" ht="31.5" customHeight="1">
       <c r="A17" s="119" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B17" s="120" t="b">
         <v>0</v>
@@ -7867,22 +7873,22 @@
         <v>2400.0</v>
       </c>
       <c r="H17" s="123" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I17" s="124" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="J17" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for rent analysis, contract and recurring payment work")</f>
         <v>Professional time-fee benchmark for rent analysis, contract and recurring payment work</v>
       </c>
       <c r="K17" s="126" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="18" ht="31.5" customHeight="1">
       <c r="A18" s="119" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B18" s="120" t="b">
         <v>0</v>
@@ -7903,22 +7909,22 @@
         <v>1800.0</v>
       </c>
       <c r="H18" s="123" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I18" s="124" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="J18" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for recurring expense and travel-support work")</f>
         <v>Professional time-fee benchmark for recurring expense and travel-support work</v>
       </c>
       <c r="K18" s="126" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
       <c r="A19" s="119" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B19" s="120" t="b">
         <v>0</v>
@@ -7939,22 +7945,22 @@
         <v>2663.0</v>
       </c>
       <c r="H19" s="123" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I19" s="124" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="J19" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware invoicing, banking, payment and bookkeeping tool-cost reference")</f>
         <v>Lexware invoicing, banking, payment and bookkeeping tool-cost reference</v>
       </c>
       <c r="K19" s="126" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" ht="31.5" customHeight="1">
       <c r="A20" s="119" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B20" s="120" t="b">
         <v>1</v>
@@ -7975,22 +7981,22 @@
         <v>1200.0</v>
       </c>
       <c r="H20" s="123" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I20" s="124" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="J20" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style recurring support benchmark for tax-payment tracking")</f>
         <v>StBVV-style recurring support benchmark for tax-payment tracking</v>
       </c>
       <c r="K20" s="126" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" ht="31.5" customHeight="1">
       <c r="A21" s="119" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B21" s="120" t="b">
         <v>1</v>
@@ -8011,22 +8017,22 @@
         <v>1800.0</v>
       </c>
       <c r="H21" s="123" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I21" s="124" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="J21" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for correspondence support and authority letters")</f>
         <v>Tax-advice benchmark for correspondence support and authority letters</v>
       </c>
       <c r="K21" s="126" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" ht="31.5" customHeight="1">
       <c r="A22" s="119" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B22" s="120" t="b">
         <v>1</v>
@@ -8047,22 +8053,22 @@
         <v>1500.0</v>
       </c>
       <c r="H22" s="123" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="I22" s="124" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="J22" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for authority correspondence and case work")</f>
         <v>Professional time-fee benchmark for authority correspondence and case work</v>
       </c>
       <c r="K22" s="126" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" ht="31.5" customHeight="1">
       <c r="A23" s="119" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B23" s="120" t="b">
         <v>0</v>
@@ -8077,28 +8083,28 @@
         <v>1</v>
       </c>
       <c r="F23" s="121">
-        <v>350.0</v>
+        <v>650.0</v>
       </c>
       <c r="G23" s="122">
-        <v>700.0</v>
+        <v>1300.0</v>
       </c>
       <c r="H23" s="123" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I23" s="124" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="J23" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for depreciation and tax-planning analysis")</f>
-        <v>Professional benchmark for depreciation and tax-planning analysis</v>
+        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for depreciation, recurring accounting and tax-planning support")</f>
+        <v>Professional benchmark for depreciation, recurring accounting and tax-planning support</v>
       </c>
       <c r="K23" s="126" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24" ht="31.5" customHeight="1">
       <c r="A24" s="119" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B24" s="120" t="b">
         <v>0</v>
@@ -8113,28 +8119,28 @@
         <v>1</v>
       </c>
       <c r="F24" s="121">
-        <v>350.0</v>
+        <v>900.0</v>
       </c>
       <c r="G24" s="122">
-        <v>700.0</v>
+        <v>1800.0</v>
       </c>
       <c r="H24" s="123" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I24" s="124" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="J24" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for retained-profit and investment planning")</f>
-        <v>Tax-advice benchmark for retained-profit and investment planning</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for retained-profit, investment and recurring accounting support")</f>
+        <v>Tax-advice benchmark for retained-profit, investment and recurring accounting support</v>
       </c>
       <c r="K24" s="126" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="25" ht="31.5" customHeight="1">
       <c r="A25" s="119" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B25" s="120" t="b">
         <v>0</v>
@@ -8149,28 +8155,28 @@
         <v>1</v>
       </c>
       <c r="F25" s="121">
-        <v>250.0</v>
+        <v>300.0</v>
       </c>
       <c r="G25" s="122">
-        <v>500.0</v>
+        <v>600.0</v>
       </c>
       <c r="H25" s="123" t="s">
         <v>236</v>
       </c>
       <c r="I25" s="124" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="J25" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for setup and evidence handling")</f>
         <v>Professional support benchmark for setup and evidence handling</v>
       </c>
       <c r="K25" s="126" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="26" ht="31.5" customHeight="1">
       <c r="A26" s="119" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B26" s="120" t="b">
         <v>0</v>
@@ -8185,28 +8191,28 @@
         <v>0</v>
       </c>
       <c r="F26" s="121">
-        <v>500.0</v>
+        <v>900.0</v>
       </c>
       <c r="G26" s="122">
-        <v>1000.0</v>
+        <v>1800.0</v>
       </c>
       <c r="H26" s="123" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I26" s="124" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="J26" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for pension reserve planning support")</f>
-        <v>Tax-advice benchmark for pension reserve planning support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for pension reserve planning and annual accounting support")</f>
+        <v>Tax-advice benchmark for pension reserve planning and annual accounting support</v>
       </c>
       <c r="K26" s="126" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="27" ht="31.5" customHeight="1">
       <c r="A27" s="119" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B27" s="120" t="b">
         <v>0</v>
@@ -8227,22 +8233,22 @@
         <v>2000.0</v>
       </c>
       <c r="H27" s="123" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="I27" s="124" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="J27" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for complex cross-border tax and accounting work")</f>
         <v>Professional benchmark for complex cross-border tax and accounting work</v>
       </c>
       <c r="K27" s="126" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="28" ht="31.5" customHeight="1">
       <c r="A28" s="119" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B28" s="120" t="b">
         <v>0</v>
@@ -8263,22 +8269,22 @@
         <v>6000.0</v>
       </c>
       <c r="H28" s="123" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I28" s="124" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="J28" s="125" t="str">
         <f>HYPERLINK("https://www.irishstatutebook.ie/eli/2014/act/38/section/137/enacted/en/html","Irish Companies Act director-residence reference plus annual director-service estimate")</f>
         <v>Irish Companies Act director-residence reference plus annual director-service estimate</v>
       </c>
       <c r="K28" s="126" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29" ht="31.5" customHeight="1">
       <c r="A29" s="119" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B29" s="120" t="b">
         <v>1</v>
@@ -8302,19 +8308,19 @@
         <v>236</v>
       </c>
       <c r="I29" s="124" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="J29" s="125" t="str">
         <f>HYPERLINK("https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service","Bundesagentur employer-number service plus employer registration support estimate")</f>
         <v>Bundesagentur employer-number service plus employer registration support estimate</v>
       </c>
       <c r="K29" s="126" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="30" ht="31.5" customHeight="1">
       <c r="A30" s="119" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B30" s="120" t="b">
         <v>1</v>
@@ -8338,19 +8344,19 @@
         <v>222</v>
       </c>
       <c r="I30" s="124" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="J30" s="125" t="str">
         <f>HYPERLINK("https://service.berlin.de/dienstleistung/121921/","Berlin Gewerbeanmeldung fee reference plus registration support estimate")</f>
         <v>Berlin Gewerbeanmeldung fee reference plus registration support estimate</v>
       </c>
       <c r="K30" s="126" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="31" ht="31.5" customHeight="1">
       <c r="A31" s="119" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B31" s="120" t="b">
         <v>0</v>
@@ -8374,19 +8380,19 @@
         <v>236</v>
       </c>
       <c r="I31" s="124" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="J31" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for bank-account setup and records")</f>
         <v>Professional support benchmark for bank-account setup and records</v>
       </c>
       <c r="K31" s="126" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="32" ht="31.5" customHeight="1">
       <c r="A32" s="119" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B32" s="120" t="b">
         <v>0</v>
@@ -8407,22 +8413,22 @@
         <v>1200.0</v>
       </c>
       <c r="H32" s="123" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="I32" s="124" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="J32" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for service agreement support")</f>
         <v>Legal-consultation benchmark for service agreement support</v>
       </c>
       <c r="K32" s="126" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
       <c r="A33" s="119" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B33" s="120" t="b">
         <v>0</v>
@@ -8443,22 +8449,22 @@
         <v>1000.0</v>
       </c>
       <c r="H33" s="123" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="I33" s="124" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="J33" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for employment contract change support")</f>
         <v>Legal-consultation benchmark for employment contract change support</v>
       </c>
       <c r="K33" s="126" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
       <c r="A34" s="119" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B34" s="120" t="b">
         <v>0</v>
@@ -8473,28 +8479,28 @@
         <v>1</v>
       </c>
       <c r="F34" s="121">
-        <v>650.0</v>
+        <v>1500.0</v>
       </c>
       <c r="G34" s="122">
-        <v>1300.0</v>
+        <v>3000.0</v>
       </c>
       <c r="H34" s="123" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="I34" s="124" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="J34" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/satzung/","Company-document benchmark for shareholder/subscription document support")</f>
-        <v>Company-document benchmark for shareholder/subscription document support</v>
+        <f>HYPERLINK("https://www.firma.de/satzung/","Company-document benchmark plus filing and notary-coordination estimate")</f>
+        <v>Company-document benchmark plus filing and notary-coordination estimate</v>
       </c>
       <c r="K34" s="126" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
       <c r="A35" s="119" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B35" s="120" t="b">
         <v>1</v>
@@ -8515,22 +8521,22 @@
         <v>600.0</v>
       </c>
       <c r="H35" s="123" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="I35" s="124" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J35" s="125" t="str">
         <f>HYPERLINK("https://rbo.gov.ie/","RBO Ireland official filing route for relevant Irish incorporated entities")</f>
         <v>RBO Ireland official filing route for relevant Irish incorporated entities</v>
       </c>
       <c r="K35" s="126" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
       <c r="A36" s="119" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B36" s="120" t="b">
         <v>0</v>
@@ -8551,22 +8557,22 @@
         <v>1500.0</v>
       </c>
       <c r="H36" s="123" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="I36" s="124" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="J36" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV personal tax filing and income-calculation benchmark")</f>
         <v>StBVV personal tax filing and income-calculation benchmark</v>
       </c>
       <c r="K36" s="126" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="37" ht="31.5" customHeight="1">
       <c r="A37" s="119" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B37" s="120" t="b">
         <v>0</v>
@@ -8587,22 +8593,22 @@
         <v>900.0</v>
       </c>
       <c r="H37" s="123" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="I37" s="124" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J37" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for parental leave and salary-timing planning")</f>
         <v>Professional support benchmark for parental leave and salary-timing planning</v>
       </c>
       <c r="K37" s="126" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="38" ht="31.5" customHeight="1">
       <c r="A38" s="127" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B38" s="128" t="b">
         <v>0</v>
@@ -8623,22 +8629,22 @@
         <v>1000.0</v>
       </c>
       <c r="H38" s="131" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="I38" s="132" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="J38" s="133" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for forecast and life-change planning support")</f>
         <v>Tax-advice benchmark for forecast and life-change planning support</v>
       </c>
       <c r="K38" s="134" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
       <c r="A39" s="135" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B39" s="110" t="b">
         <v>0</v>
@@ -8659,17 +8665,17 @@
         <v>1200.0</v>
       </c>
       <c r="H39" s="137" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I39" s="110" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J39" s="138" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for recurring client support")</f>
         <v>StBVV-style time-fee benchmark for recurring client support</v>
       </c>
       <c r="K39" s="110" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Narrow option 1 and add startup execution costs
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="336">
   <si>
     <t>Savings Calculation Template</t>
   </si>
@@ -30,502 +30,505 @@
     <t>Before analysis</t>
   </si>
   <si>
+    <t>Basic operating entity; no optimisation, payroll setup, registrations, authority case work or RBO</t>
+  </si>
+  <si>
+    <t>Option 2 - Full optimisation</t>
+  </si>
+  <si>
+    <t>Option 3 - Pension reserve</t>
+  </si>
+  <si>
+    <t>Option 4 - IE tax residence</t>
+  </si>
+  <si>
+    <t>Service scope</t>
+  </si>
+  <si>
+    <t>Current position</t>
+  </si>
+  <si>
+    <t>Basic operating entity; no optimisation</t>
+  </si>
+  <si>
+    <t>Full optimisation excl. pension reserve</t>
+  </si>
+  <si>
+    <t>Full optimisation + pension reserve</t>
+  </si>
+  <si>
+    <t>IE tax residence + director support</t>
+  </si>
+  <si>
+    <t>Tax residence</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>Optimises office rent</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Optimises business travel / other expenses</t>
+  </si>
+  <si>
+    <t>Car depreciation support</t>
+  </si>
+  <si>
+    <t>Investment planning support</t>
+  </si>
+  <si>
+    <t>Pension reserve included</t>
+  </si>
+  <si>
+    <t>Director fee required</t>
+  </si>
+  <si>
+    <t>Previous accounting fee</t>
+  </si>
+  <si>
+    <t>RB Accounting, Legal, Structuring</t>
+  </si>
+  <si>
+    <t>Employee surcharge</t>
+  </si>
+  <si>
+    <t>Pension surcharge</t>
+  </si>
+  <si>
+    <t>Dual tax jurisdiction surcharge</t>
+  </si>
+  <si>
+    <t>Director surcharge (discounted)</t>
+  </si>
+  <si>
+    <t>Total RB fee</t>
+  </si>
+  <si>
+    <t>Company model</t>
+  </si>
+  <si>
+    <t>Estimated status quo profit</t>
+  </si>
+  <si>
+    <t>Office rent deductible</t>
+  </si>
+  <si>
+    <t>Business travel / other deductible</t>
+  </si>
+  <si>
+    <t>Other investment planning benefit</t>
+  </si>
+  <si>
+    <t>Annual car depreciation deductible</t>
+  </si>
+  <si>
+    <t>Pension reserve contribution</t>
+  </si>
+  <si>
+    <t>IE director fee deductible</t>
+  </si>
+  <si>
+    <t>RB fee deductible</t>
+  </si>
+  <si>
+    <t>Total additional deductions</t>
+  </si>
+  <si>
+    <t>Estimated taxable profit after scenario</t>
+  </si>
+  <si>
+    <t>Corporation tax rate</t>
+  </si>
+  <si>
+    <t>Corporation tax payable</t>
+  </si>
+  <si>
+    <t>Corporation tax saved vs before</t>
+  </si>
+  <si>
+    <t>Personal / owner value</t>
+  </si>
+  <si>
+    <t>Office rent net owner benefit</t>
+  </si>
+  <si>
+    <t>Travel / other costs shifted from personal</t>
+  </si>
+  <si>
+    <t>Investment planning benefit</t>
+  </si>
+  <si>
+    <t>Pension reserve value</t>
+  </si>
+  <si>
+    <t>Director fee net owner benefit</t>
+  </si>
+  <si>
+    <t>Outcome</t>
+  </si>
+  <si>
+    <t>Incremental value before RB fee</t>
+  </si>
+  <si>
+    <t>Avoided previous accounting fee</t>
+  </si>
+  <si>
+    <t>Net savings after RB fee</t>
+  </si>
+  <si>
+    <t>Net savings multiple of fee</t>
+  </si>
+  <si>
+    <t>Review note</t>
+  </si>
+  <si>
+    <t>Baseline only</t>
+  </si>
+  <si>
+    <t>Basic operating entity only</t>
+  </si>
+  <si>
+    <t>Full optimisation, pension reserve excluded</t>
+  </si>
+  <si>
+    <t>Pension surcharge shown separately</t>
+  </si>
+  <si>
+    <t>IE tax residence, dual jurisdiction and director split</t>
+  </si>
+  <si>
+    <t>Model checks</t>
+  </si>
+  <si>
+    <t>Taxable profit not negative?</t>
+  </si>
+  <si>
+    <t>Net savings positive?</t>
+  </si>
+  <si>
+    <t>Baseline</t>
+  </si>
+  <si>
+    <t>Fee rule status</t>
+  </si>
+  <si>
+    <t>Basic operating entity fee fixed at 500</t>
+  </si>
+  <si>
+    <t>Base plus employee surcharge if over threshold</t>
+  </si>
+  <si>
+    <t>Base plus pension surcharge and employee surcharge if over threshold</t>
+  </si>
+  <si>
+    <t>Base plus dual tax jurisdiction and discounted director surcharge</t>
+  </si>
+  <si>
+    <t>Assumptions</t>
+  </si>
+  <si>
+    <t>Status: provisional. Source: user instruction, RB internal service lists, and public DE pricing references imported 2026-06-12. Review before client reliance.</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Client / company name</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>Client-facing display name</t>
+  </si>
+  <si>
+    <t>Prepared for</t>
+  </si>
+  <si>
+    <t>Contact or stakeholder</t>
+  </si>
+  <si>
+    <t>Selected scenario</t>
+  </si>
+  <si>
+    <t>Client choice pending</t>
+  </si>
+  <si>
+    <t>choice</t>
+  </si>
+  <si>
+    <t>P&amp;L add-on stays pending until a client choice is made</t>
+  </si>
+  <si>
+    <t>Total employees</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>Employee surcharge applies above the threshold below</t>
+  </si>
+  <si>
+    <t>Employee notes</t>
+  </si>
+  <si>
+    <t>Use for part-time or payroll complexity notes</t>
+  </si>
+  <si>
+    <t>Current tax residence</t>
+  </si>
+  <si>
+    <t>Option 4 models IE tax residence</t>
+  </si>
+  <si>
+    <t>Tax rates</t>
+  </si>
+  <si>
+    <t>Tax rate note</t>
+  </si>
+  <si>
+    <t>Replace rates with client-specific values</t>
+  </si>
+  <si>
+    <t>Planning rates only</t>
+  </si>
+  <si>
+    <t>DE corporation tax rate</t>
+  </si>
+  <si>
+    <t>% incl. trade tax</t>
+  </si>
+  <si>
+    <t>Planning assumption; replace with client-specific rate</t>
+  </si>
+  <si>
+    <t>IE corporation tax rate</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Trading-rate planning assumption; confirm applicability</t>
+  </si>
+  <si>
+    <t>Owner marginal personal tax rate</t>
+  </si>
+  <si>
+    <t>Review-only rate used for net owner benefit estimates; not a client data input</t>
+  </si>
+  <si>
+    <t>Operating model</t>
+  </si>
+  <si>
+    <t>Operating model note</t>
+  </si>
+  <si>
+    <t>Status quo estimated from earnings and spend</t>
+  </si>
+  <si>
+    <t>Future gross-net calculator workflow can use https://www.brutto-netto-rechner.info/gehalt/gehaltsrechner-arbeitgeber.php</t>
+  </si>
+  <si>
+    <t>Annual revenue</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>Before optimisation</t>
+  </si>
+  <si>
+    <t>Current operating costs before owner planning</t>
+  </si>
+  <si>
+    <t>Exclude RB fee and optimisation items below</t>
+  </si>
+  <si>
+    <t>Baseline profit already includes current accounting fee?</t>
+  </si>
+  <si>
+    <t>Set previous accounting fee below to 0 if already embedded and not replaced</t>
+  </si>
+  <si>
+    <t>Estimated status quo profit (calculated)</t>
+  </si>
+  <si>
+    <t>Calculated from annual revenue minus current operating costs; not a client input</t>
+  </si>
+  <si>
+    <t>Office rent and expense optimisation</t>
+  </si>
+  <si>
+    <t>Office rent note</t>
+  </si>
+  <si>
+    <t>Use conservative eligible amounts</t>
+  </si>
+  <si>
+    <t>Company-paid office rent or home-office arrangement</t>
+  </si>
+  <si>
+    <t>Annual office rent company can rent to owner</t>
+  </si>
+  <si>
+    <t>Eligible office rent deductible</t>
+  </si>
+  <si>
+    <t>Used in comparison tab</t>
+  </si>
+  <si>
+    <t>Taxable share of company-paid office rent</t>
+  </si>
+  <si>
+    <t>Use 0 if tax-free and 1 if fully taxable to the owner; review case by case</t>
+  </si>
+  <si>
+    <t>Business travel deductible</t>
+  </si>
+  <si>
+    <t>Business travel moved into company</t>
+  </si>
+  <si>
+    <t>Other eligible business expenses deductible</t>
+  </si>
+  <si>
+    <t>Software, training, conferences, equipment, etc.</t>
+  </si>
+  <si>
+    <t>Car purchase / depreciation</t>
+  </si>
+  <si>
+    <t>Car purchase price</t>
+  </si>
+  <si>
+    <t>Gross planning amount</t>
+  </si>
+  <si>
+    <t>Useful life years</t>
+  </si>
+  <si>
+    <t>years</t>
+  </si>
+  <si>
+    <t>Replace with client-specific depreciation method</t>
+  </si>
+  <si>
+    <t>Business-use share</t>
+  </si>
+  <si>
+    <t>Planning share</t>
+  </si>
+  <si>
+    <t>Annual depreciation before business-use share</t>
+  </si>
+  <si>
+    <t>Straight-line placeholder</t>
+  </si>
+  <si>
+    <t>Eligible annual car depreciation</t>
+  </si>
+  <si>
+    <t>Investment and pension reserve</t>
+  </si>
+  <si>
+    <t>Retained-profit or investment planning value</t>
+  </si>
+  <si>
+    <t>Only included in Option 3</t>
+  </si>
+  <si>
+    <t>IE tax residence / director</t>
+  </si>
+  <si>
+    <t>Annual director fee deductible</t>
+  </si>
+  <si>
+    <t>Only included in Option 4</t>
+  </si>
+  <si>
+    <t>Estimated tax on director fee</t>
+  </si>
+  <si>
+    <t>Applied to director fee only to estimate after-tax owner benefit; review case by case</t>
+  </si>
+  <si>
+    <t>Current annual accounting, legal, or advisory fee that RB replaces</t>
+  </si>
+  <si>
+    <t>Option 1 Basic operating entity fee</t>
+  </si>
+  <si>
+    <t>No software/calendar setup, payroll, employer/local registrations, tax payment/correspondence/fine resolution, RBO, office rent, travel, investment, car, or pension optimisation</t>
+  </si>
+  <si>
+    <t>RB Accounting, Legal, Structuring base fee</t>
+  </si>
+  <si>
+    <t>Base fee for Options 2-4 before surcharges</t>
+  </si>
+  <si>
+    <t>Employee surcharge threshold</t>
+  </si>
+  <si>
+    <t>employees</t>
+  </si>
+  <si>
+    <t>Total employees above this threshold trigger surcharge</t>
+  </si>
+  <si>
+    <t>Employee surcharge if over threshold</t>
+  </si>
+  <si>
+    <t>Applies to optimisation options when employee count exceeds threshold</t>
+  </si>
+  <si>
+    <t>Annual surcharge shown as separate line in Option 3 for pension reserve planning plus recurring reserve accounting/year-end support</t>
+  </si>
+  <si>
+    <t>Shown as separate line in Option 4</t>
+  </si>
+  <si>
+    <t>Director surcharge discounted</t>
+  </si>
+  <si>
+    <t>Discounted director support surcharge in Option 4</t>
+  </si>
+  <si>
+    <t>Fee definitions</t>
+  </si>
+  <si>
+    <t>Current position before RB analysis</t>
+  </si>
+  <si>
     <t>Option 1 - Basic operating entity</t>
   </si>
   <si>
-    <t>Option 2 - Full optimisation</t>
-  </si>
-  <si>
-    <t>Option 3 - Pension reserve</t>
-  </si>
-  <si>
-    <t>Option 4 - IE tax residence</t>
-  </si>
-  <si>
-    <t>Service scope</t>
-  </si>
-  <si>
-    <t>Current position</t>
-  </si>
-  <si>
-    <t>Basic operating entity; no optimisation</t>
-  </si>
-  <si>
-    <t>Full optimisation excl. pension reserve</t>
-  </si>
-  <si>
-    <t>Full optimisation + pension reserve</t>
-  </si>
-  <si>
-    <t>IE tax residence + director support</t>
-  </si>
-  <si>
-    <t>Tax residence</t>
-  </si>
-  <si>
-    <t>DE</t>
-  </si>
-  <si>
-    <t>IE</t>
-  </si>
-  <si>
-    <t>Optimises office rent</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Optimises business travel / other expenses</t>
-  </si>
-  <si>
-    <t>Car depreciation support</t>
-  </si>
-  <si>
-    <t>Investment planning support</t>
-  </si>
-  <si>
-    <t>Pension reserve included</t>
-  </si>
-  <si>
-    <t>Director fee required</t>
-  </si>
-  <si>
-    <t>Previous accounting fee</t>
-  </si>
-  <si>
-    <t>RB Accounting, Legal, Structuring</t>
-  </si>
-  <si>
-    <t>Employee surcharge</t>
-  </si>
-  <si>
-    <t>Pension surcharge</t>
-  </si>
-  <si>
-    <t>Dual tax jurisdiction surcharge</t>
-  </si>
-  <si>
-    <t>Director surcharge (discounted)</t>
-  </si>
-  <si>
-    <t>Total RB fee</t>
-  </si>
-  <si>
-    <t>Company model</t>
-  </si>
-  <si>
-    <t>Estimated status quo profit</t>
-  </si>
-  <si>
-    <t>Office rent deductible</t>
-  </si>
-  <si>
-    <t>Business travel / other deductible</t>
-  </si>
-  <si>
-    <t>Other investment planning benefit</t>
-  </si>
-  <si>
-    <t>Annual car depreciation deductible</t>
-  </si>
-  <si>
-    <t>Pension reserve contribution</t>
-  </si>
-  <si>
-    <t>IE director fee deductible</t>
-  </si>
-  <si>
-    <t>RB fee deductible</t>
-  </si>
-  <si>
-    <t>Total additional deductions</t>
-  </si>
-  <si>
-    <t>Estimated taxable profit after scenario</t>
-  </si>
-  <si>
-    <t>Corporation tax rate</t>
-  </si>
-  <si>
-    <t>Corporation tax payable</t>
-  </si>
-  <si>
-    <t>Corporation tax saved vs before</t>
-  </si>
-  <si>
-    <t>Personal / owner value</t>
-  </si>
-  <si>
-    <t>Office rent net owner benefit</t>
-  </si>
-  <si>
-    <t>Travel / other costs shifted from personal</t>
-  </si>
-  <si>
-    <t>Investment planning benefit</t>
-  </si>
-  <si>
-    <t>Pension reserve value</t>
-  </si>
-  <si>
-    <t>Director fee net owner benefit</t>
-  </si>
-  <si>
-    <t>Outcome</t>
-  </si>
-  <si>
-    <t>Incremental value before RB fee</t>
-  </si>
-  <si>
-    <t>Avoided previous accounting fee</t>
-  </si>
-  <si>
-    <t>Net savings after RB fee</t>
-  </si>
-  <si>
-    <t>Net savings multiple of fee</t>
-  </si>
-  <si>
-    <t>Review note</t>
-  </si>
-  <si>
-    <t>Baseline only</t>
-  </si>
-  <si>
-    <t>Basic operating entity only</t>
-  </si>
-  <si>
-    <t>Full optimisation, pension reserve excluded</t>
-  </si>
-  <si>
-    <t>Pension surcharge shown separately</t>
-  </si>
-  <si>
-    <t>IE tax residence, dual jurisdiction and director split</t>
-  </si>
-  <si>
-    <t>Model checks</t>
-  </si>
-  <si>
-    <t>Taxable profit not negative?</t>
-  </si>
-  <si>
-    <t>Net savings positive?</t>
-  </si>
-  <si>
-    <t>Baseline</t>
-  </si>
-  <si>
-    <t>Fee rule status</t>
-  </si>
-  <si>
-    <t>Basic operating entity fee fixed at 500</t>
-  </si>
-  <si>
-    <t>Base plus employee surcharge if over threshold</t>
-  </si>
-  <si>
-    <t>Base plus pension surcharge and employee surcharge if over threshold</t>
-  </si>
-  <si>
-    <t>Base plus dual tax jurisdiction and discounted director surcharge</t>
-  </si>
-  <si>
-    <t>Assumptions</t>
-  </si>
-  <si>
-    <t>Status: provisional. Source: user instruction, RB internal service lists, and public DE pricing references imported 2026-06-12. Review before client reliance.</t>
-  </si>
-  <si>
-    <t>Input</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Client / company name</t>
-  </si>
-  <si>
-    <t>text</t>
-  </si>
-  <si>
-    <t>Client-facing display name</t>
-  </si>
-  <si>
-    <t>Prepared for</t>
-  </si>
-  <si>
-    <t>Contact or stakeholder</t>
-  </si>
-  <si>
-    <t>Selected scenario</t>
-  </si>
-  <si>
-    <t>Client choice pending</t>
-  </si>
-  <si>
-    <t>choice</t>
-  </si>
-  <si>
-    <t>P&amp;L add-on stays pending until a client choice is made</t>
-  </si>
-  <si>
-    <t>Total employees</t>
-  </si>
-  <si>
-    <t>count</t>
-  </si>
-  <si>
-    <t>Employee surcharge applies above the threshold below</t>
-  </si>
-  <si>
-    <t>Employee notes</t>
-  </si>
-  <si>
-    <t>Use for part-time or payroll complexity notes</t>
-  </si>
-  <si>
-    <t>Current tax residence</t>
-  </si>
-  <si>
-    <t>Option 4 models IE tax residence</t>
-  </si>
-  <si>
-    <t>Tax rates</t>
-  </si>
-  <si>
-    <t>Tax rate note</t>
-  </si>
-  <si>
-    <t>Replace rates with client-specific values</t>
-  </si>
-  <si>
-    <t>Planning rates only</t>
-  </si>
-  <si>
-    <t>DE corporation tax rate</t>
-  </si>
-  <si>
-    <t>% incl. trade tax</t>
-  </si>
-  <si>
-    <t>Planning assumption; replace with client-specific rate</t>
-  </si>
-  <si>
-    <t>IE corporation tax rate</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>Trading-rate planning assumption; confirm applicability</t>
-  </si>
-  <si>
-    <t>Owner marginal personal tax rate</t>
-  </si>
-  <si>
-    <t>Review-only rate used for net owner benefit estimates; not a client data input</t>
-  </si>
-  <si>
-    <t>Operating model</t>
-  </si>
-  <si>
-    <t>Operating model note</t>
-  </si>
-  <si>
-    <t>Status quo estimated from earnings and spend</t>
-  </si>
-  <si>
-    <t>Future gross-net calculator workflow can use https://www.brutto-netto-rechner.info/gehalt/gehaltsrechner-arbeitgeber.php</t>
-  </si>
-  <si>
-    <t>Annual revenue</t>
-  </si>
-  <si>
-    <t>EUR</t>
-  </si>
-  <si>
-    <t>Before optimisation</t>
-  </si>
-  <si>
-    <t>Current operating costs before owner planning</t>
-  </si>
-  <si>
-    <t>Exclude RB fee and optimisation items below</t>
-  </si>
-  <si>
-    <t>Baseline profit already includes current accounting fee?</t>
-  </si>
-  <si>
-    <t>Set previous accounting fee below to 0 if already embedded and not replaced</t>
-  </si>
-  <si>
-    <t>Estimated status quo profit (calculated)</t>
-  </si>
-  <si>
-    <t>Calculated from annual revenue minus current operating costs; not a client input</t>
-  </si>
-  <si>
-    <t>Office rent and expense optimisation</t>
-  </si>
-  <si>
-    <t>Office rent note</t>
-  </si>
-  <si>
-    <t>Use conservative eligible amounts</t>
-  </si>
-  <si>
-    <t>Company-paid office rent or home-office arrangement</t>
-  </si>
-  <si>
-    <t>Annual office rent company can rent to owner</t>
-  </si>
-  <si>
-    <t>Eligible office rent deductible</t>
-  </si>
-  <si>
-    <t>Used in comparison tab</t>
-  </si>
-  <si>
-    <t>Taxable share of company-paid office rent</t>
-  </si>
-  <si>
-    <t>Use 0 if tax-free and 1 if fully taxable to the owner; review case by case</t>
-  </si>
-  <si>
-    <t>Business travel deductible</t>
-  </si>
-  <si>
-    <t>Business travel moved into company</t>
-  </si>
-  <si>
-    <t>Other eligible business expenses deductible</t>
-  </si>
-  <si>
-    <t>Software, training, conferences, equipment, etc.</t>
-  </si>
-  <si>
-    <t>Car purchase / depreciation</t>
-  </si>
-  <si>
-    <t>Car purchase price</t>
-  </si>
-  <si>
-    <t>Gross planning amount</t>
-  </si>
-  <si>
-    <t>Useful life years</t>
-  </si>
-  <si>
-    <t>years</t>
-  </si>
-  <si>
-    <t>Replace with client-specific depreciation method</t>
-  </si>
-  <si>
-    <t>Business-use share</t>
-  </si>
-  <si>
-    <t>Planning share</t>
-  </si>
-  <si>
-    <t>Annual depreciation before business-use share</t>
-  </si>
-  <si>
-    <t>Straight-line placeholder</t>
-  </si>
-  <si>
-    <t>Eligible annual car depreciation</t>
-  </si>
-  <si>
-    <t>Investment and pension reserve</t>
-  </si>
-  <si>
-    <t>Retained-profit or investment planning value</t>
-  </si>
-  <si>
-    <t>Only included in Option 3</t>
-  </si>
-  <si>
-    <t>IE tax residence / director</t>
-  </si>
-  <si>
-    <t>Annual director fee deductible</t>
-  </si>
-  <si>
-    <t>Only included in Option 4</t>
-  </si>
-  <si>
-    <t>Estimated tax on director fee</t>
-  </si>
-  <si>
-    <t>Applied to director fee only to estimate after-tax owner benefit; review case by case</t>
-  </si>
-  <si>
-    <t>Current annual accounting, legal, or advisory fee that RB replaces</t>
-  </si>
-  <si>
-    <t>Option 1 Basic operating entity fee</t>
-  </si>
-  <si>
-    <t>No office rent, travel, investment, car, or pension optimisation</t>
-  </si>
-  <si>
-    <t>RB Accounting, Legal, Structuring base fee</t>
-  </si>
-  <si>
-    <t>Base fee for Options 2-4 before surcharges</t>
-  </si>
-  <si>
-    <t>Employee surcharge threshold</t>
-  </si>
-  <si>
-    <t>employees</t>
-  </si>
-  <si>
-    <t>Total employees above this threshold trigger surcharge</t>
-  </si>
-  <si>
-    <t>Employee surcharge if over threshold</t>
-  </si>
-  <si>
-    <t>Applies to optimisation options when employee count exceeds threshold</t>
-  </si>
-  <si>
-    <t>Annual surcharge shown as separate line in Option 3 for pension reserve planning plus recurring reserve accounting/year-end support</t>
-  </si>
-  <si>
-    <t>Shown as separate line in Option 4</t>
-  </si>
-  <si>
-    <t>Director surcharge discounted</t>
-  </si>
-  <si>
-    <t>Discounted director support surcharge in Option 4</t>
-  </si>
-  <si>
-    <t>Fee definitions</t>
-  </si>
-  <si>
-    <t>Current position before RB analysis</t>
-  </si>
-  <si>
-    <t>Basic operating entity, no optimisation and no investments/car depreciation support</t>
+    <t>Basic operating entity review only; excludes software/calendar setup, payroll, registrations, tax payment/correspondence/fine resolution, RBO, and investment/car/pension optimisation</t>
   </si>
   <si>
     <t>1000 plus employee surcharge</t>
   </si>
   <si>
-    <t>Office rent, business travel, eligible expenses, car depreciation, and investment/startup shareholding planning, including recurring accounting uplift where those structures are used; pension reserve excluded</t>
+    <t>Office rent, business travel, eligible expenses, car depreciation, investment/startup shareholding planning and execution where selected, and recurring accounting uplift; pension reserve excluded</t>
   </si>
   <si>
     <t>1000 plus pension surcharge plus employee surcharge if applicable</t>
@@ -537,7 +540,7 @@
     <t>1000 plus dual tax jurisdiction and discounted director surcharge plus employee surcharge if applicable</t>
   </si>
   <si>
-    <t>Option 2 scope for an IE tax resident company; director fee required</t>
+    <t>Option 2 scope for an IE tax resident company, including RBO/VIF where applicable; director fee required</t>
   </si>
   <si>
     <t>P&amp;L - add-on</t>
@@ -657,7 +660,7 @@
     <t>Standalone DE market value checked - mid</t>
   </si>
   <si>
-    <t>Status: provisional. Source: RB service-list work, user corrections, ELSTER official filing-form list, and public pricing/statutory references checked 2026-06-15. Low/mid estimates include advisory support plus third-party software, filing, payment administration and recurring accounting uplift where relevant; review before client reliance.</t>
+    <t>Status: provisional. Source: RB service-list work, user corrections, ELSTER official filing-form list, CRO/RBO filing guidance, and public pricing/statutory references checked 2026-06-15. Low/mid estimates include advisory support plus third-party software, filing, payment administration, execution support and recurring accounting uplift where relevant; review before client reliance.</t>
   </si>
   <si>
     <t>Service</t>
@@ -855,10 +858,13 @@
     <t>Investment / retained-profit and startup shareholding planning</t>
   </si>
   <si>
-    <t>Retained-profit investment planning, startup shareholding transfer planning, accounting/tax treatment review and annual investment/valuation/accounting support; investment-management fees excluded</t>
-  </si>
-  <si>
-    <t>For startup investments, include the annual accounting/tax uplift after the structure is set up</t>
+    <t>Planning + annual accounting</t>
+  </si>
+  <si>
+    <t>Planning and annual investment/accounting support only; execution of startup shareholding transfers is costed separately in the startup transfer execution row; investment-management fees excluded</t>
+  </si>
+  <si>
+    <t>Do not treat this as execution; use the separate startup shareholding transfer execution row for agreements, filings, VIF/RBO and notary coordination</t>
   </si>
   <si>
     <t>Investment account setup</t>
@@ -951,55 +957,58 @@
     <t>Change employment or director contracts and align payroll/accounting treatment</t>
   </si>
   <si>
-    <t>Share subscription / personal shareholding transfer agreements and filings</t>
-  </si>
-  <si>
-    <t>One-off + filings</t>
-  </si>
-  <si>
-    <t>Agreement drafting/review plus shareholder/company approvals, share-capital/cap-table updates, corporate-register filings and notary coordination where required; external notary/statutory fees may be extra</t>
-  </si>
-  <si>
-    <t>For moving a personal startup shareholding into a company, check filings, notary route, share-capital changes and external fees</t>
-  </si>
-  <si>
-    <t>RBO / beneficial-owner filing where applicable</t>
+    <t>Startup shareholding transfer execution, filings and notary coordination</t>
+  </si>
+  <si>
+    <t>One-off execution + filings</t>
+  </si>
+  <si>
+    <t>Execution after planning: transfer/subscription agreements, valuation/evidence pack, shareholder/company approvals, cap-table/share-capital updates, CRO/Companies Register or equivalent filings, Revenue share-transfer/stamp-duty process, RBO/VIF updates and notary coordination where required; external notary/statutory fees excluded unless paid through RB</t>
+  </si>
+  <si>
+    <t>This is the execution cost missing from the planning row; use after the client chooses the investment/startup shareholding route</t>
+  </si>
+  <si>
+    <t>RBO / beneficial-owner filing plus VIF/IPN where applicable</t>
+  </si>
+  <si>
+    <t>Event-based + annual monitoring</t>
+  </si>
+  <si>
+    <t>RBO filing after VIF/IPN where a beneficial owner has no Irish PPSN; includes VIF pack, notary/witness coordination, RBO filing, annual/trigger-event monitoring and evidence capture; external notary/statutory fees excluded unless paid through RB</t>
+  </si>
+  <si>
+    <t>Include from option 2 onwards only; for foreign individuals, plan the VIF/IPN and notary/witness step before the RBO filing</t>
+  </si>
+  <si>
+    <t>Personal tax bookkeeping and filing add-on</t>
+  </si>
+  <si>
+    <t>Optional annual</t>
+  </si>
+  <si>
+    <t>Optional annual personal tax bookkeeping and filing estimate; separate from company operating entity services</t>
+  </si>
+  <si>
+    <t>Optional personal tax support outside the core company option fee</t>
+  </si>
+  <si>
+    <t>Parental leave planning</t>
+  </si>
+  <si>
+    <t>Optional planning</t>
+  </si>
+  <si>
+    <t>Optional planning estimate for parental leave, owner salary timing, payroll impact and benefit timing</t>
+  </si>
+  <si>
+    <t>Optional planning for parental leave and owner salary timing</t>
+  </si>
+  <si>
+    <t>Client forecast and life-change planning</t>
   </si>
   <si>
     <t>Annual / event-based</t>
-  </si>
-  <si>
-    <t>Beneficial-owner filing and annual/trigger-event monitoring support; checked in all options for IE company structures</t>
-  </si>
-  <si>
-    <t>All IE company structures need beneficial-owner filing work, so this is included across plans</t>
-  </si>
-  <si>
-    <t>Personal tax bookkeeping and filing add-on</t>
-  </si>
-  <si>
-    <t>Optional annual</t>
-  </si>
-  <si>
-    <t>Optional annual personal tax bookkeeping and filing estimate; separate from company operating entity services</t>
-  </si>
-  <si>
-    <t>Optional personal tax support outside the core company option fee</t>
-  </si>
-  <si>
-    <t>Parental leave planning</t>
-  </si>
-  <si>
-    <t>Optional planning</t>
-  </si>
-  <si>
-    <t>Optional planning estimate for parental leave, owner salary timing, payroll impact and benefit timing</t>
-  </si>
-  <si>
-    <t>Optional planning for parental leave and owner salary timing</t>
-  </si>
-  <si>
-    <t>Client forecast and life-change planning</t>
   </si>
   <si>
     <t>Recurring annual or event-driven forecast updates after life/business changes; support estimate based on tax/accounting advisory time</t>
@@ -4815,7 +4824,7 @@
     </row>
     <row r="61" ht="43.5" customHeight="1">
       <c r="A61" s="52" t="s">
-        <v>4</v>
+        <v>167</v>
       </c>
       <c r="B61" s="52">
         <v>500.0</v>
@@ -4824,7 +4833,7 @@
         <v>111</v>
       </c>
       <c r="D61" s="52" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="62" ht="43.5" customHeight="1">
@@ -4832,13 +4841,13 @@
         <v>5</v>
       </c>
       <c r="B62" s="52" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C62" s="52" t="s">
         <v>111</v>
       </c>
       <c r="D62" s="52" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="63" ht="43.5" customHeight="1">
@@ -4846,13 +4855,13 @@
         <v>6</v>
       </c>
       <c r="B63" s="52" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C63" s="52" t="s">
         <v>111</v>
       </c>
       <c r="D63" s="52" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="64" ht="16.5" customHeight="1">
@@ -4860,13 +4869,13 @@
         <v>7</v>
       </c>
       <c r="B64" s="55" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C64" s="54" t="s">
         <v>111</v>
       </c>
       <c r="D64" s="54" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="65" ht="16.5" customHeight="1">
@@ -5880,17 +5889,17 @@
   <sheetData>
     <row r="1" ht="16.5" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" ht="31.5" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
       <c r="A3" s="96" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B3" s="97" t="str">
         <f>Assumptions!$B$8</f>
@@ -5899,7 +5908,7 @@
     </row>
     <row r="4" ht="16.5" customHeight="1">
       <c r="A4" s="96" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B4" s="22" t="str">
         <f t="array" ref="B4">IFERROR(INDEX('Savings comparison'!$C$46:$F$46,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0)),"")</f>
@@ -5909,54 +5918,54 @@
     <row r="5" ht="16.5" customHeight="1"/>
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
       <c r="A7" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C7" s="13">
         <f t="array" ref="C7:N7">Assumptions!$B$21/12+COLUMN(C6:N6)*0</f>
@@ -5998,10 +6007,10 @@
     </row>
     <row r="8" ht="16.5" customHeight="1">
       <c r="A8" s="98" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B8" s="99" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C8" s="100">
         <f t="array" ref="C8:N8">Assumptions!$B$22/12+COLUMN(C6:N6)*0</f>
@@ -6043,10 +6052,10 @@
     </row>
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B9" s="101" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C9" s="13">
         <f t="array" ref="C9:N9">Assumptions!$B$49/12+COLUMN(C6:N6)*0</f>
@@ -6088,10 +6097,10 @@
     </row>
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" s="98" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B10" s="99" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C10" s="100" t="str">
         <f t="array" ref="C10:N10">IFERROR(INDEX('Savings comparison'!$C$23:$F$23,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -6111,10 +6120,10 @@
     </row>
     <row r="11" ht="16.5" customHeight="1">
       <c r="A11" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B11" s="101" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C11" s="13" t="str">
         <f t="array" ref="C11:N11">IFERROR(INDEX('Savings comparison'!$C$24:$F$24,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -6134,10 +6143,10 @@
     </row>
     <row r="12" ht="16.5" customHeight="1">
       <c r="A12" s="11" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B12" s="101" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C12" s="13" t="str">
         <f t="array" ref="C12:N12">IFERROR(INDEX('Savings comparison'!$C$26:$F$26,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -6160,7 +6169,7 @@
         <v>38</v>
       </c>
       <c r="B13" s="101" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C13" s="13" t="str">
         <f t="array" ref="C13:N13">IFERROR(INDEX('Savings comparison'!$C$27:$F$27,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -6180,10 +6189,10 @@
     </row>
     <row r="14" ht="16.5" customHeight="1">
       <c r="A14" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B14" s="101" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C14" s="13" t="str">
         <f t="array" ref="C14:N14">IFERROR(INDEX('Savings comparison'!$C$28:$F$28,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -6203,10 +6212,10 @@
     </row>
     <row r="15" ht="16.5" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B15" s="101" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C15" s="13" t="str">
         <f t="array" ref="C15:N15">IFERROR(INDEX('Savings comparison'!$C$19:$F$19,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0))/12+COLUMN(C6:N6)*0,"")</f>
@@ -6242,10 +6251,10 @@
     </row>
     <row r="17" ht="16.5" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B17" s="101" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C17" s="13">
         <f t="array" ref="C17">IF(COUNTIF('Savings comparison'!$C$4:$F$4,$B$3)=0,0,C8:N8-C9:N9-C11:N11-C12:N12-C13:N13-C14:N14-C15:N15-C16:N16+C10:N10)</f>
@@ -6265,10 +6274,10 @@
     </row>
     <row r="18" ht="16.5" customHeight="1">
       <c r="A18" s="96" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B18" s="103" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C18" s="22">
         <f t="array" ref="C18">IF(COUNTIF('Savings comparison'!$C$4:$F$4,$B$3)=0,0,IF(C17:N17&gt;0,C17:N17*INDEX('Savings comparison'!$C$32:$F$32,1,MATCH($B$3,'Savings comparison'!$C$4:$F$4,0)),0))</f>
@@ -6288,10 +6297,10 @@
     </row>
     <row r="19" ht="16.5" customHeight="1">
       <c r="A19" s="96" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B19" s="103" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C19" s="22">
         <f t="array" ref="C19">IF(COUNTIF('Savings comparison'!$C$4:$F$4,$B$3)=0,0,C17:N17-C18:N18)</f>
@@ -6330,7 +6339,7 @@
         <v>77</v>
       </c>
       <c r="B21" s="103" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C21" s="104"/>
       <c r="D21" s="104"/>
@@ -7389,12 +7398,12 @@
   <sheetData>
     <row r="1" ht="27.0" customHeight="1">
       <c r="A1" s="105" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="106" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B2" s="107">
         <f>'Savings comparison'!C19</f>
@@ -7421,23 +7430,23 @@
     </row>
     <row r="3">
       <c r="A3" s="106" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B3" s="107">
         <f t="shared" ref="B3:E3" si="1">SUMIF(B8:B39,TRUE,$F$8:$F$39)</f>
-        <v>10743</v>
+        <v>6092</v>
       </c>
       <c r="C3" s="107">
         <f t="shared" si="1"/>
-        <v>19998</v>
+        <v>21348</v>
       </c>
       <c r="D3" s="107">
         <f t="shared" si="1"/>
-        <v>20898</v>
+        <v>22248</v>
       </c>
       <c r="E3" s="107">
         <f t="shared" si="1"/>
-        <v>23998</v>
+        <v>25348</v>
       </c>
       <c r="F3" s="108"/>
       <c r="G3" s="108"/>
@@ -7448,23 +7457,23 @@
     </row>
     <row r="4">
       <c r="A4" s="106" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B4" s="109">
         <f t="shared" ref="B4:E4" si="2">SUMIF(B8:B39,TRUE,$G$8:$G$39)</f>
-        <v>19802</v>
+        <v>10531</v>
       </c>
       <c r="C4" s="109">
         <f t="shared" si="2"/>
-        <v>38265</v>
+        <v>41165</v>
       </c>
       <c r="D4" s="109">
         <f t="shared" si="2"/>
-        <v>40065</v>
+        <v>42965</v>
       </c>
       <c r="E4" s="109">
         <f t="shared" si="2"/>
-        <v>46265</v>
+        <v>49165</v>
       </c>
       <c r="F4" s="110"/>
       <c r="G4" s="110"/>
@@ -7475,7 +7484,7 @@
     </row>
     <row r="5">
       <c r="A5" s="111" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" ht="42.0" customHeight="1">
@@ -7493,10 +7502,10 @@
     </row>
     <row r="7" ht="37.5" customHeight="1">
       <c r="A7" s="115" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B7" s="116" t="s">
-        <v>4</v>
+        <v>167</v>
       </c>
       <c r="C7" s="116" t="s">
         <v>5</v>
@@ -7508,27 +7517,27 @@
         <v>7</v>
       </c>
       <c r="F7" s="117" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G7" s="116" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H7" s="116" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I7" s="116" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="J7" s="116" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K7" s="118" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
       <c r="A8" s="119" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B8" s="120" t="b">
         <v>1</v>
@@ -7549,22 +7558,22 @@
         <v>1223.0</v>
       </c>
       <c r="H8" s="123" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I8" s="124" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J8" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","firma.de tax-advice benchmark plus professional-support estimate")</f>
         <v>firma.de tax-advice benchmark plus professional-support estimate</v>
       </c>
       <c r="K8" s="126" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1">
       <c r="A9" s="119" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B9" s="120" t="b">
         <v>1</v>
@@ -7585,22 +7594,22 @@
         <v>1500.0</v>
       </c>
       <c r="H9" s="123" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I9" s="124" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J9" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/satzung/","firma.de company-document benchmark plus incorporation support estimate")</f>
         <v>firma.de company-document benchmark plus incorporation support estimate</v>
       </c>
       <c r="K9" s="126" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" ht="31.5" customHeight="1">
       <c r="A10" s="119" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B10" s="120" t="b">
         <v>1</v>
@@ -7621,22 +7630,22 @@
         <v>600.0</v>
       </c>
       <c r="H10" s="123" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I10" s="124" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J10" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for document intake and admin support")</f>
         <v>StBVV-style time-fee benchmark for document intake and admin support</v>
       </c>
       <c r="K10" s="126" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" ht="31.5" customHeight="1">
       <c r="A11" s="119" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B11" s="120" t="b">
         <v>1</v>
@@ -7657,25 +7666,25 @@
         <v>2208.0</v>
       </c>
       <c r="H11" s="123" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I11" s="124" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J11" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/buchhaltung/","firma.de bookkeeping package prices including DATEV software add-on")</f>
         <v>firma.de bookkeeping package prices including DATEV software add-on</v>
       </c>
       <c r="K11" s="126" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" ht="31.5" customHeight="1">
       <c r="A12" s="119" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B12" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12" s="120" t="b">
         <v>1</v>
@@ -7693,22 +7702,22 @@
         <v>600.0</v>
       </c>
       <c r="H12" s="123" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I12" s="124" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J12" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware Office software prices used where a tool cost is needed")</f>
         <v>Lexware Office software prices used where a tool cost is needed</v>
       </c>
       <c r="K12" s="126" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13" ht="31.5" customHeight="1">
       <c r="A13" s="119" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B13" s="120" t="b">
         <v>1</v>
@@ -7729,22 +7738,22 @@
         <v>2200.0</v>
       </c>
       <c r="H13" s="123" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="I13" s="124" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J13" s="125" t="str">
         <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Umsatzsteuer-Voranmeldung and Umsatzsteuererklärung forms")</f>
         <v>ELSTER lists Umsatzsteuer-Voranmeldung and Umsatzsteuererklärung forms</v>
       </c>
       <c r="K13" s="126" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" ht="31.5" customHeight="1">
       <c r="A14" s="119" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B14" s="120" t="b">
         <v>1</v>
@@ -7765,25 +7774,25 @@
         <v>2800.0</v>
       </c>
       <c r="H14" s="123" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I14" s="124" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J14" s="125" t="str">
         <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Körperschaftsteuererklärung and Gewerbesteuererklärung; annual accounts benchmark added separately")</f>
         <v>ELSTER lists Körperschaftsteuererklärung and Gewerbesteuererklärung; annual accounts benchmark added separately</v>
       </c>
       <c r="K14" s="126" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" ht="31.5" customHeight="1">
       <c r="A15" s="119" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B15" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="120" t="b">
         <v>1</v>
@@ -7801,25 +7810,25 @@
         <v>1440.0</v>
       </c>
       <c r="H15" s="123" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="I15" s="124" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J15" s="125" t="str">
         <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Lohnsteuer-Anmeldung; estimate includes payment-run administration")</f>
         <v>ELSTER lists Lohnsteuer-Anmeldung; estimate includes payment-run administration</v>
       </c>
       <c r="K15" s="126" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" ht="31.5" customHeight="1">
       <c r="A16" s="119" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B16" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" s="120" t="b">
         <v>1</v>
@@ -7837,22 +7846,22 @@
         <v>1000.0</v>
       </c>
       <c r="H16" s="123" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I16" s="124" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J16" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware payroll filing/tool reference plus setup-support estimate")</f>
         <v>Lexware payroll filing/tool reference plus setup-support estimate</v>
       </c>
       <c r="K16" s="126" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" ht="31.5" customHeight="1">
       <c r="A17" s="119" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B17" s="120" t="b">
         <v>0</v>
@@ -7873,22 +7882,22 @@
         <v>2400.0</v>
       </c>
       <c r="H17" s="123" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I17" s="124" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J17" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for rent analysis, contract and recurring payment work")</f>
         <v>Professional time-fee benchmark for rent analysis, contract and recurring payment work</v>
       </c>
       <c r="K17" s="126" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="18" ht="31.5" customHeight="1">
       <c r="A18" s="119" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B18" s="120" t="b">
         <v>0</v>
@@ -7909,22 +7918,22 @@
         <v>1800.0</v>
       </c>
       <c r="H18" s="123" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I18" s="124" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J18" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for recurring expense and travel-support work")</f>
         <v>Professional time-fee benchmark for recurring expense and travel-support work</v>
       </c>
       <c r="K18" s="126" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" ht="31.5" customHeight="1">
       <c r="A19" s="119" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B19" s="120" t="b">
         <v>0</v>
@@ -7945,25 +7954,25 @@
         <v>2663.0</v>
       </c>
       <c r="H19" s="123" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I19" s="124" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J19" s="125" t="str">
         <f>HYPERLINK("https://www.lexware.de/preise/","Lexware invoicing, banking, payment and bookkeeping tool-cost reference")</f>
         <v>Lexware invoicing, banking, payment and bookkeeping tool-cost reference</v>
       </c>
       <c r="K19" s="126" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="20" ht="31.5" customHeight="1">
       <c r="A20" s="119" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B20" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" s="120" t="b">
         <v>1</v>
@@ -7981,25 +7990,25 @@
         <v>1200.0</v>
       </c>
       <c r="H20" s="123" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I20" s="124" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J20" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style recurring support benchmark for tax-payment tracking")</f>
         <v>StBVV-style recurring support benchmark for tax-payment tracking</v>
       </c>
       <c r="K20" s="126" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" ht="31.5" customHeight="1">
       <c r="A21" s="119" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B21" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="120" t="b">
         <v>1</v>
@@ -8017,25 +8026,25 @@
         <v>1800.0</v>
       </c>
       <c r="H21" s="123" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I21" s="124" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="J21" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for correspondence support and authority letters")</f>
         <v>Tax-advice benchmark for correspondence support and authority letters</v>
       </c>
       <c r="K21" s="126" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" ht="31.5" customHeight="1">
       <c r="A22" s="119" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B22" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="120" t="b">
         <v>1</v>
@@ -8053,22 +8062,22 @@
         <v>1500.0</v>
       </c>
       <c r="H22" s="123" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I22" s="124" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J22" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for authority correspondence and case work")</f>
         <v>Professional time-fee benchmark for authority correspondence and case work</v>
       </c>
       <c r="K22" s="126" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" ht="31.5" customHeight="1">
       <c r="A23" s="119" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B23" s="120" t="b">
         <v>0</v>
@@ -8089,22 +8098,22 @@
         <v>1300.0</v>
       </c>
       <c r="H23" s="123" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I23" s="124" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J23" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for depreciation, recurring accounting and tax-planning support")</f>
         <v>Professional benchmark for depreciation, recurring accounting and tax-planning support</v>
       </c>
       <c r="K23" s="126" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24" ht="31.5" customHeight="1">
       <c r="A24" s="119" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B24" s="120" t="b">
         <v>0</v>
@@ -8125,22 +8134,22 @@
         <v>1800.0</v>
       </c>
       <c r="H24" s="123" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="I24" s="124" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="J24" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for retained-profit, investment and recurring accounting support")</f>
         <v>Tax-advice benchmark for retained-profit, investment and recurring accounting support</v>
       </c>
       <c r="K24" s="126" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="25" ht="31.5" customHeight="1">
       <c r="A25" s="119" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B25" s="120" t="b">
         <v>0</v>
@@ -8161,22 +8170,22 @@
         <v>600.0</v>
       </c>
       <c r="H25" s="123" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I25" s="124" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="J25" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for setup and evidence handling")</f>
         <v>Professional support benchmark for setup and evidence handling</v>
       </c>
       <c r="K25" s="126" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="26" ht="31.5" customHeight="1">
       <c r="A26" s="119" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B26" s="120" t="b">
         <v>0</v>
@@ -8197,22 +8206,22 @@
         <v>1800.0</v>
       </c>
       <c r="H26" s="123" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="I26" s="124" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="J26" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for pension reserve planning and annual accounting support")</f>
         <v>Tax-advice benchmark for pension reserve planning and annual accounting support</v>
       </c>
       <c r="K26" s="126" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="27" ht="31.5" customHeight="1">
       <c r="A27" s="119" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B27" s="120" t="b">
         <v>0</v>
@@ -8233,22 +8242,22 @@
         <v>2000.0</v>
       </c>
       <c r="H27" s="123" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="I27" s="124" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="J27" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for complex cross-border tax and accounting work")</f>
         <v>Professional benchmark for complex cross-border tax and accounting work</v>
       </c>
       <c r="K27" s="126" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28" ht="31.5" customHeight="1">
       <c r="A28" s="119" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B28" s="120" t="b">
         <v>0</v>
@@ -8269,25 +8278,25 @@
         <v>6000.0</v>
       </c>
       <c r="H28" s="123" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I28" s="124" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="J28" s="125" t="str">
         <f>HYPERLINK("https://www.irishstatutebook.ie/eli/2014/act/38/section/137/enacted/en/html","Irish Companies Act director-residence reference plus annual director-service estimate")</f>
         <v>Irish Companies Act director-residence reference plus annual director-service estimate</v>
       </c>
       <c r="K28" s="126" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="29" ht="31.5" customHeight="1">
       <c r="A29" s="119" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B29" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C29" s="120" t="b">
         <v>1</v>
@@ -8305,25 +8314,25 @@
         <v>600.0</v>
       </c>
       <c r="H29" s="123" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I29" s="124" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="J29" s="125" t="str">
         <f>HYPERLINK("https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service","Bundesagentur employer-number service plus employer registration support estimate")</f>
         <v>Bundesagentur employer-number service plus employer registration support estimate</v>
       </c>
       <c r="K29" s="126" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="30" ht="31.5" customHeight="1">
       <c r="A30" s="119" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B30" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C30" s="120" t="b">
         <v>1</v>
@@ -8341,22 +8350,22 @@
         <v>531.0</v>
       </c>
       <c r="H30" s="123" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I30" s="124" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="J30" s="125" t="str">
         <f>HYPERLINK("https://service.berlin.de/dienstleistung/121921/","Berlin Gewerbeanmeldung fee reference plus registration support estimate")</f>
         <v>Berlin Gewerbeanmeldung fee reference plus registration support estimate</v>
       </c>
       <c r="K30" s="126" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="31" ht="31.5" customHeight="1">
       <c r="A31" s="119" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B31" s="120" t="b">
         <v>0</v>
@@ -8377,22 +8386,22 @@
         <v>500.0</v>
       </c>
       <c r="H31" s="123" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I31" s="124" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="J31" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for bank-account setup and records")</f>
         <v>Professional support benchmark for bank-account setup and records</v>
       </c>
       <c r="K31" s="126" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="32" ht="31.5" customHeight="1">
       <c r="A32" s="119" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B32" s="120" t="b">
         <v>0</v>
@@ -8413,22 +8422,22 @@
         <v>1200.0</v>
       </c>
       <c r="H32" s="123" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="I32" s="124" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="J32" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for service agreement support")</f>
         <v>Legal-consultation benchmark for service agreement support</v>
       </c>
       <c r="K32" s="126" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="33" ht="31.5" customHeight="1">
       <c r="A33" s="119" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B33" s="120" t="b">
         <v>0</v>
@@ -8449,22 +8458,22 @@
         <v>1000.0</v>
       </c>
       <c r="H33" s="123" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="I33" s="124" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="J33" s="125" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for employment contract change support")</f>
         <v>Legal-consultation benchmark for employment contract change support</v>
       </c>
       <c r="K33" s="126" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="34" ht="31.5" customHeight="1">
       <c r="A34" s="119" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B34" s="120" t="b">
         <v>0</v>
@@ -8479,31 +8488,31 @@
         <v>1</v>
       </c>
       <c r="F34" s="121">
-        <v>1500.0</v>
+        <v>2500.0</v>
       </c>
       <c r="G34" s="122">
-        <v>3000.0</v>
+        <v>5000.0</v>
       </c>
       <c r="H34" s="123" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="I34" s="124" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="J34" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/satzung/","Company-document benchmark plus filing and notary-coordination estimate")</f>
-        <v>Company-document benchmark plus filing and notary-coordination estimate</v>
+        <f>HYPERLINK("https://cro.ie/post-registration/company-post/share-transfer/","CRO share-transfer, stamp-duty and annual-return filing reference")</f>
+        <v>CRO share-transfer, stamp-duty and annual-return filing reference</v>
       </c>
       <c r="K34" s="126" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="35" ht="31.5" customHeight="1">
       <c r="A35" s="119" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B35" s="120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C35" s="120" t="b">
         <v>1</v>
@@ -8515,28 +8524,28 @@
         <v>1</v>
       </c>
       <c r="F35" s="121">
-        <v>300.0</v>
+        <v>650.0</v>
       </c>
       <c r="G35" s="122">
-        <v>600.0</v>
+        <v>1500.0</v>
       </c>
       <c r="H35" s="123" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="I35" s="124" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="J35" s="125" t="str">
-        <f>HYPERLINK("https://rbo.gov.ie/","RBO Ireland official filing route for relevant Irish incorporated entities")</f>
-        <v>RBO Ireland official filing route for relevant Irish incorporated entities</v>
+        <f>HYPERLINK("https://rbo.gov.ie/faqs/ppsn-why-its-required-and-what-to-do-if-you-dont-have-one/","RBO explains VIF/IPN where a beneficial owner has no Irish PPSN")</f>
+        <v>RBO explains VIF/IPN where a beneficial owner has no Irish PPSN</v>
       </c>
       <c r="K35" s="126" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="36" ht="31.5" customHeight="1">
       <c r="A36" s="119" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B36" s="120" t="b">
         <v>0</v>
@@ -8557,22 +8566,22 @@
         <v>1500.0</v>
       </c>
       <c r="H36" s="123" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="I36" s="124" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J36" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV personal tax filing and income-calculation benchmark")</f>
         <v>StBVV personal tax filing and income-calculation benchmark</v>
       </c>
       <c r="K36" s="126" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="37" ht="31.5" customHeight="1">
       <c r="A37" s="119" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B37" s="120" t="b">
         <v>0</v>
@@ -8593,22 +8602,22 @@
         <v>900.0</v>
       </c>
       <c r="H37" s="123" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="I37" s="124" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J37" s="125" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for parental leave and salary-timing planning")</f>
         <v>Professional support benchmark for parental leave and salary-timing planning</v>
       </c>
       <c r="K37" s="126" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="38" ht="31.5" customHeight="1">
       <c r="A38" s="127" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B38" s="128" t="b">
         <v>0</v>
@@ -8629,22 +8638,22 @@
         <v>1000.0</v>
       </c>
       <c r="H38" s="131" t="s">
-        <v>316</v>
+        <v>330</v>
       </c>
       <c r="I38" s="132" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="J38" s="133" t="str">
         <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for forecast and life-change planning support")</f>
         <v>Tax-advice benchmark for forecast and life-change planning support</v>
       </c>
       <c r="K38" s="134" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="39" ht="31.5" customHeight="1">
       <c r="A39" s="135" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B39" s="110" t="b">
         <v>0</v>
@@ -8665,17 +8674,17 @@
         <v>1200.0</v>
       </c>
       <c r="H39" s="137" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I39" s="110" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="J39" s="138" t="str">
         <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for recurring client support")</f>
         <v>StBVV-style time-fee benchmark for recurring client support</v>
       </c>
       <c r="K39" s="110" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add proof labels for mid estimates
</commit_message>
<xml_diff>
--- a/clients/Companies/_template/savings-calculation-template.xlsx
+++ b/clients/Companies/_template/savings-calculation-template.xlsx
@@ -654,13 +654,13 @@
     <t>RB option fee</t>
   </si>
   <si>
-    <t>Standalone DE market value checked - low</t>
-  </si>
-  <si>
-    <t>Standalone DE market value checked - mid</t>
-  </si>
-  <si>
-    <t>Status: provisional. Source: RB service-list work, user corrections, ELSTER official filing-form list, CRO/RBO filing guidance, and public pricing/statutory references checked 2026-06-15. Low/mid estimates include advisory support plus third-party software, filing, payment administration, execution support and recurring accounting uplift where relevant; review before client reliance.</t>
+    <t>Standalone DE estimate - low</t>
+  </si>
+  <si>
+    <t>Standalone DE estimate - mid / proofed</t>
+  </si>
+  <si>
+    <t>Status: provisional. Source: RB service-list work, user corrections, public pricing/statutory references checked 2026-06-15. Mid estimates now distinguish quoted package arithmetic from professional-time estimates; where no public fixed package was found, the proof cell says so. Review: final pricing should be quoted before client reliance.</t>
   </si>
   <si>
     <t>Service</t>
@@ -669,7 +669,7 @@
     <t>Low-end DE estimate</t>
   </si>
   <si>
-    <t>Mid-end DE estimate</t>
+    <t>Mid DE estimate (proofed)</t>
   </si>
   <si>
     <t>Timing</t>
@@ -678,7 +678,7 @@
     <t>Basis / cost components</t>
   </si>
   <si>
-    <t>Linked explanation</t>
+    <t>Mid estimate proof / linked source</t>
   </si>
   <si>
     <t>RB / client discussion point</t>
@@ -753,7 +753,7 @@
     <t>Annual accounts, e-Bilanz and corporate/trade tax filings</t>
   </si>
   <si>
-    <t>Annual accounts, disclosure/filing, e-Bilanz transmission, corporate tax return and trade tax return; VAT filings are costed in the VAT row</t>
+    <t>Annual accounts, disclosure/filing, e-Bilanz transmission, corporate tax return and trade tax return; mid uses public package arithmetic (2499 + 99 disclosure + 139 setup); VAT filings are costed in the VAT row</t>
   </si>
   <si>
     <t>Annual filing scope should cover accounts, e-Bilanz, corporation tax and trade tax; VAT is shown separately</t>
@@ -7461,19 +7461,19 @@
       </c>
       <c r="B4" s="109">
         <f t="shared" ref="B4:E4" si="2">SUMIF(B8:B39,TRUE,$G$8:$G$39)</f>
-        <v>10531</v>
+        <v>10468</v>
       </c>
       <c r="C4" s="109">
         <f t="shared" si="2"/>
-        <v>41165</v>
+        <v>41102</v>
       </c>
       <c r="D4" s="109">
         <f t="shared" si="2"/>
-        <v>42965</v>
+        <v>42902</v>
       </c>
       <c r="E4" s="109">
         <f t="shared" si="2"/>
-        <v>49165</v>
+        <v>49102</v>
       </c>
       <c r="F4" s="110"/>
       <c r="G4" s="110"/>
@@ -7564,8 +7564,8 @@
         <v>224</v>
       </c>
       <c r="J8" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","firma.de tax-advice benchmark plus professional-support estimate")</f>
-        <v>firma.de tax-advice benchmark plus professional-support estimate</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min tax advice; mid assumes ~7h review/scoping, not a fixed package quote")</f>
+        <v>Proof: €89/30-min tax advice; mid assumes ~7h review/scoping, not a fixed package quote</v>
       </c>
       <c r="K8" s="126" t="s">
         <v>225</v>
@@ -7600,8 +7600,8 @@
         <v>227</v>
       </c>
       <c r="J9" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/satzung/","firma.de company-document benchmark plus incorporation support estimate")</f>
-        <v>firma.de company-document benchmark plus incorporation support estimate</v>
+        <f>HYPERLINK("https://www.firma.de/satzung/","Proof: Satzung Pro €999 + €99/h extra legal time; mid adds setup/compliance support")</f>
+        <v>Proof: Satzung Pro €999 + €99/h extra legal time; mid adds setup/compliance support</v>
       </c>
       <c r="K9" s="126" t="s">
         <v>228</v>
@@ -7636,8 +7636,8 @@
         <v>230</v>
       </c>
       <c r="J10" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for document intake and admin support")</f>
-        <v>StBVV-style time-fee benchmark for document intake and admin support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min tax-advice benchmark; mid assumes ~3-4h intake, not a package quote")</f>
+        <v>Proof: €89/30-min tax-advice benchmark; mid assumes ~3-4h intake, not a package quote</v>
       </c>
       <c r="K10" s="126" t="s">
         <v>231</v>
@@ -7672,8 +7672,8 @@
         <v>234</v>
       </c>
       <c r="J11" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/buchhaltung/","firma.de bookkeeping package prices including DATEV software add-on")</f>
-        <v>firma.de bookkeeping package prices including DATEV software add-on</v>
+        <f>HYPERLINK("https://www.firma.de/buchhaltung/","Proof: quoted Basis €169/month + DATEV €15/month = €2,208/year")</f>
+        <v>Proof: quoted Basis €169/month + DATEV €15/month = €2,208/year</v>
       </c>
       <c r="K11" s="126" t="s">
         <v>235</v>
@@ -7708,8 +7708,8 @@
         <v>238</v>
       </c>
       <c r="J12" s="125" t="str">
-        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware Office software prices used where a tool cost is needed")</f>
-        <v>Lexware Office software prices used where a tool cost is needed</v>
+        <f>HYPERLINK("https://www.lexware.de/preise/","Proof: Lexware tool floor €7.90-€32.90/month; mid assumes setup/configuration time")</f>
+        <v>Proof: Lexware tool floor €7.90-€32.90/month; mid assumes setup/configuration time</v>
       </c>
       <c r="K12" s="126" t="s">
         <v>239</v>
@@ -7744,8 +7744,8 @@
         <v>242</v>
       </c>
       <c r="J13" s="125" t="str">
-        <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Umsatzsteuer-Voranmeldung and Umsatzsteuererklärung forms")</f>
-        <v>ELSTER lists Umsatzsteuer-Voranmeldung and Umsatzsteuererklärung forms</v>
+        <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","Proof: ELSTER VAT forms + €89/30-min benchmark; mid assumes recurring filing/payment work")</f>
+        <v>Proof: ELSTER VAT forms + €89/30-min benchmark; mid assumes recurring filing/payment work</v>
       </c>
       <c r="K13" s="126" t="s">
         <v>243</v>
@@ -7771,7 +7771,7 @@
         <v>1700.0</v>
       </c>
       <c r="G14" s="122">
-        <v>2800.0</v>
+        <v>2737.0</v>
       </c>
       <c r="H14" s="123" t="s">
         <v>233</v>
@@ -7780,8 +7780,8 @@
         <v>245</v>
       </c>
       <c r="J14" s="125" t="str">
-        <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Körperschaftsteuererklärung and Gewerbesteuererklärung; annual accounts benchmark added separately")</f>
-        <v>ELSTER lists Körperschaftsteuererklärung and Gewerbesteuererklärung; annual accounts benchmark added separately</v>
+        <f>HYPERLINK("https://www.firma.de/jahresabschluss-kapitalgesellschaft/","Proof: Premium €2,499 + €99 disclosure + €139 setup = €2,737; source includes tax/e-Bilanz scope")</f>
+        <v>Proof: Premium €2,499 + €99 disclosure + €139 setup = €2,737; source includes tax/e-Bilanz scope</v>
       </c>
       <c r="K14" s="126" t="s">
         <v>246</v>
@@ -7816,8 +7816,8 @@
         <v>249</v>
       </c>
       <c r="J15" s="125" t="str">
-        <f>HYPERLINK("https://www.elster.de/eportal/formulare-leistungen/alleformulare","ELSTER lists Lohnsteuer-Anmeldung; estimate includes payment-run administration")</f>
-        <v>ELSTER lists Lohnsteuer-Anmeldung; estimate includes payment-run administration</v>
+        <f>HYPERLINK("https://www.lexware.de/preise/","Proof: payroll tool €12.90/month + integrated payments; mid adds ~6h/year admin/payment time")</f>
+        <v>Proof: payroll tool €12.90/month + integrated payments; mid adds ~6h/year admin/payment time</v>
       </c>
       <c r="K15" s="126" t="s">
         <v>250</v>
@@ -7852,8 +7852,8 @@
         <v>253</v>
       </c>
       <c r="J16" s="125" t="str">
-        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware payroll filing/tool reference plus setup-support estimate")</f>
-        <v>Lexware payroll filing/tool reference plus setup-support estimate</v>
+        <f>HYPERLINK("https://www.firma.de/lohnabrechnung/","Proof: public payroll package proves filing scope; mid assumes ~5-6h catch-up/setup time")</f>
+        <v>Proof: public payroll package proves filing scope; mid assumes ~5-6h catch-up/setup time</v>
       </c>
       <c r="K16" s="126" t="s">
         <v>254</v>
@@ -7888,8 +7888,8 @@
         <v>257</v>
       </c>
       <c r="J17" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for rent analysis, contract and recurring payment work")</f>
-        <v>Professional time-fee benchmark for rent analysis, contract and recurring payment work</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~13h/year rent benchmarking/contract/payment admin")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~13h/year rent benchmarking/contract/payment admin</v>
       </c>
       <c r="K17" s="126" t="s">
         <v>258</v>
@@ -7924,8 +7924,8 @@
         <v>260</v>
       </c>
       <c r="J18" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for recurring expense and travel-support work")</f>
-        <v>Professional time-fee benchmark for recurring expense and travel-support work</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~10h/year travel/per-diem/reimbursement admin")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~10h/year travel/per-diem/reimbursement admin</v>
       </c>
       <c r="K18" s="126" t="s">
         <v>261</v>
@@ -7960,8 +7960,8 @@
         <v>263</v>
       </c>
       <c r="J19" s="125" t="str">
-        <f>HYPERLINK("https://www.lexware.de/preise/","Lexware invoicing, banking, payment and bookkeeping tool-cost reference")</f>
-        <v>Lexware invoicing, banking, payment and bookkeeping tool-cost reference</v>
+        <f>HYPERLINK("https://www.lexware.de/preise/","Proof: Lexware XL €32.90/month tool floor; mid adds recurring AP/AR labour time")</f>
+        <v>Proof: Lexware XL €32.90/month tool floor; mid adds recurring AP/AR labour time</v>
       </c>
       <c r="K19" s="126" t="s">
         <v>264</v>
@@ -7996,8 +7996,8 @@
         <v>266</v>
       </c>
       <c r="J20" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style recurring support benchmark for tax-payment tracking")</f>
-        <v>StBVV-style recurring support benchmark for tax-payment tracking</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~7h/year tracking and payments")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~7h/year tracking and payments</v>
       </c>
       <c r="K20" s="126" t="s">
         <v>267</v>
@@ -8032,8 +8032,8 @@
         <v>269</v>
       </c>
       <c r="J21" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for correspondence support and authority letters")</f>
-        <v>Tax-advice benchmark for correspondence support and authority letters</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~10h/year recurring tax letters/correspondence")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~10h/year recurring tax letters/correspondence</v>
       </c>
       <c r="K21" s="126" t="s">
         <v>270</v>
@@ -8068,8 +8068,8 @@
         <v>273</v>
       </c>
       <c r="J22" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional time-fee benchmark for authority correspondence and case work")</f>
-        <v>Professional time-fee benchmark for authority correspondence and case work</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~8-9h case work; fines/penalties excluded")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~8-9h case work; fines/penalties excluded</v>
       </c>
       <c r="K22" s="126" t="s">
         <v>274</v>
@@ -8104,8 +8104,8 @@
         <v>277</v>
       </c>
       <c r="J23" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for depreciation, recurring accounting and tax-planning support")</f>
-        <v>Professional benchmark for depreciation, recurring accounting and tax-planning support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~7h/year car depreciation/private-use accounting")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~7h/year car depreciation/private-use accounting</v>
       </c>
       <c r="K23" s="126" t="s">
         <v>278</v>
@@ -8140,8 +8140,8 @@
         <v>281</v>
       </c>
       <c r="J24" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for retained-profit, investment and recurring accounting support")</f>
-        <v>Tax-advice benchmark for retained-profit, investment and recurring accounting support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~10h/year retained-profit/investment accounting support")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~10h/year retained-profit/investment accounting support</v>
       </c>
       <c r="K24" s="126" t="s">
         <v>282</v>
@@ -8176,8 +8176,8 @@
         <v>284</v>
       </c>
       <c r="J25" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for setup and evidence handling")</f>
-        <v>Professional support benchmark for setup and evidence handling</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~3-4h setup/evidence workflow, not investment management")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~3-4h setup/evidence workflow, not investment management</v>
       </c>
       <c r="K25" s="126" t="s">
         <v>285</v>
@@ -8212,8 +8212,8 @@
         <v>287</v>
       </c>
       <c r="J26" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for pension reserve planning and annual accounting support")</f>
-        <v>Tax-advice benchmark for pension reserve planning and annual accounting support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~10h/year pension-reserve planning/accounting uplift")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~10h/year pension-reserve planning/accounting uplift</v>
       </c>
       <c r="K26" s="126" t="s">
         <v>288</v>
@@ -8248,8 +8248,8 @@
         <v>291</v>
       </c>
       <c r="J27" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional benchmark for complex cross-border tax and accounting work")</f>
-        <v>Professional benchmark for complex cross-border tax and accounting work</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~11h cross-border review/coordination; final quote needed")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~11h cross-border review/coordination; final quote needed</v>
       </c>
       <c r="K27" s="126" t="s">
         <v>292</v>
@@ -8284,8 +8284,8 @@
         <v>294</v>
       </c>
       <c r="J28" s="125" t="str">
-        <f>HYPERLINK("https://www.irishstatutebook.ie/eli/2014/act/38/section/137/enacted/en/html","Irish Companies Act director-residence reference plus annual director-service estimate")</f>
-        <v>Irish Companies Act director-residence reference plus annual director-service estimate</v>
+        <f>HYPERLINK("https://www.irishstatutebook.ie/eli/2014/act/38/section/137/enacted/en/html","Proof: statutory director-residence trigger; €6,000 is quote-required annual director-service placeholder")</f>
+        <v>Proof: statutory director-residence trigger; €6,000 is quote-required annual director-service placeholder</v>
       </c>
       <c r="K28" s="126" t="s">
         <v>295</v>
@@ -8320,8 +8320,8 @@
         <v>297</v>
       </c>
       <c r="J29" s="125" t="str">
-        <f>HYPERLINK("https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service","Bundesagentur employer-number service plus employer registration support estimate")</f>
-        <v>Bundesagentur employer-number service plus employer registration support estimate</v>
+        <f>HYPERLINK("https://www.arbeitsagentur.de/unternehmen/betriebsnummern-service","Proof: official employer-number process + ~3-4h registration support estimate")</f>
+        <v>Proof: official employer-number process + ~3-4h registration support estimate</v>
       </c>
       <c r="K29" s="126" t="s">
         <v>298</v>
@@ -8356,8 +8356,8 @@
         <v>300</v>
       </c>
       <c r="J30" s="125" t="str">
-        <f>HYPERLINK("https://service.berlin.de/dienstleistung/121921/","Berlin Gewerbeanmeldung fee reference plus registration support estimate")</f>
-        <v>Berlin Gewerbeanmeldung fee reference plus registration support estimate</v>
+        <f>HYPERLINK("https://service.berlin.de/dienstleistung/121921/","Proof: Berlin fee €31 + support time; mid estimate includes registration handling")</f>
+        <v>Proof: Berlin fee €31 + support time; mid estimate includes registration handling</v>
       </c>
       <c r="K30" s="126" t="s">
         <v>301</v>
@@ -8392,8 +8392,8 @@
         <v>303</v>
       </c>
       <c r="J31" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for bank-account setup and records")</f>
-        <v>Professional support benchmark for bank-account setup and records</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~3h bank/access/accounting setup")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~3h bank/access/accounting setup</v>
       </c>
       <c r="K31" s="126" t="s">
         <v>304</v>
@@ -8428,8 +8428,8 @@
         <v>307</v>
       </c>
       <c r="J32" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for service agreement support")</f>
-        <v>Legal-consultation benchmark for service agreement support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Proof: €135/45-min legal advice; mid assumes ~6-7h contract/accounting alignment")</f>
+        <v>Proof: €135/45-min legal advice; mid assumes ~6-7h contract/accounting alignment</v>
       </c>
       <c r="K32" s="126" t="s">
         <v>308</v>
@@ -8464,8 +8464,8 @@
         <v>311</v>
       </c>
       <c r="J33" s="125" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Legal-consultation benchmark for employment contract change support")</f>
-        <v>Legal-consultation benchmark for employment contract change support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-anwalt/","Proof: €135/45-min legal advice; mid assumes ~5-6h employment/director-contract change support")</f>
+        <v>Proof: €135/45-min legal advice; mid assumes ~5-6h employment/director-contract change support</v>
       </c>
       <c r="K33" s="126" t="s">
         <v>312</v>
@@ -8500,8 +8500,8 @@
         <v>315</v>
       </c>
       <c r="J34" s="125" t="str">
-        <f>HYPERLINK("https://cro.ie/post-registration/company-post/share-transfer/","CRO share-transfer, stamp-duty and annual-return filing reference")</f>
-        <v>CRO share-transfer, stamp-duty and annual-return filing reference</v>
+        <f>HYPERLINK("https://www.firma.de/satzung/","Proof: Satzung Pro €999 + €99/h extra legal time; startup transfer execution remains quote-sensitive")</f>
+        <v>Proof: Satzung Pro €999 + €99/h extra legal time; startup transfer execution remains quote-sensitive</v>
       </c>
       <c r="K34" s="126" t="s">
         <v>316</v>
@@ -8536,8 +8536,8 @@
         <v>319</v>
       </c>
       <c r="J35" s="125" t="str">
-        <f>HYPERLINK("https://rbo.gov.ie/faqs/ppsn-why-its-required-and-what-to-do-if-you-dont-have-one/","RBO explains VIF/IPN where a beneficial owner has no Irish PPSN")</f>
-        <v>RBO explains VIF/IPN where a beneficial owner has no Irish PPSN</v>
+        <f>HYPERLINK("https://rbo.gov.ie/faqs/ppsn-why-its-required-and-what-to-do-if-you-dont-have-one/","Proof: RBO VIF/IPN requirement; €1,500 is coordination/notary-time estimate, not an official filing fee")</f>
+        <v>Proof: RBO VIF/IPN requirement; €1,500 is coordination/notary-time estimate, not an official filing fee</v>
       </c>
       <c r="K35" s="126" t="s">
         <v>320</v>
@@ -8572,8 +8572,8 @@
         <v>323</v>
       </c>
       <c r="J36" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV personal tax filing and income-calculation benchmark")</f>
-        <v>StBVV personal tax filing and income-calculation benchmark</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min tax advice; mid assumes ~8h annual personal tax bookkeeping/filing support")</f>
+        <v>Proof: €89/30-min tax advice; mid assumes ~8h annual personal tax bookkeeping/filing support</v>
       </c>
       <c r="K36" s="126" t="s">
         <v>324</v>
@@ -8608,8 +8608,8 @@
         <v>327</v>
       </c>
       <c r="J37" s="125" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","Professional support benchmark for parental leave and salary-timing planning")</f>
-        <v>Professional support benchmark for parental leave and salary-timing planning</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min tax advice; mid assumes ~5h planning support, not benefit entitlement advice")</f>
+        <v>Proof: €89/30-min tax advice; mid assumes ~5h planning support, not benefit entitlement advice</v>
       </c>
       <c r="K37" s="126" t="s">
         <v>328</v>
@@ -8644,8 +8644,8 @@
         <v>331</v>
       </c>
       <c r="J38" s="133" t="str">
-        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Tax-advice benchmark for forecast and life-change planning support")</f>
-        <v>Tax-advice benchmark for forecast and life-change planning support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~5-6h annual/event forecast updates")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~5-6h annual/event forecast updates</v>
       </c>
       <c r="K38" s="134" t="s">
         <v>332</v>
@@ -8680,8 +8680,8 @@
         <v>334</v>
       </c>
       <c r="J39" s="138" t="str">
-        <f>HYPERLINK("https://www.gesetze-im-internet.de/stbgebv/BJNR014420981.html","StBVV-style time-fee benchmark for recurring client support")</f>
-        <v>StBVV-style time-fee benchmark for recurring client support</v>
+        <f>HYPERLINK("https://www.firma.de/beratung-steuerberater/","Proof: €89/30-min benchmark; mid assumes ~6-7h annual client support")</f>
+        <v>Proof: €89/30-min benchmark; mid assumes ~6-7h annual client support</v>
       </c>
       <c r="K39" s="110" t="s">
         <v>335</v>

</xml_diff>